<commit_message>
Add IROS 2026 participants
</commit_message>
<xml_diff>
--- a/Registration.xlsx
+++ b/Registration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tsamak\Workspace\AutoDRIVE-RoboRacer-Sim-Racing-Participation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73570B97-F6C7-4C45-A5A5-2AE7C9B4C0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3627A9-44AA-461C-A9B6-212EB97ECB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="4" xr2:uid="{5D9342A3-8B90-4963-824C-8C358DE1DB7F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="5" xr2:uid="{5D9342A3-8B90-4963-824C-8C358DE1DB7F}"/>
   </bookViews>
   <sheets>
     <sheet name="IROS 2024" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="ICRA 2025" sheetId="4" r:id="rId3"/>
     <sheet name="CDC-TF 2025" sheetId="5" r:id="rId4"/>
     <sheet name="ICRA 2026" sheetId="6" r:id="rId5"/>
+    <sheet name="IROS 2026" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1687" uniqueCount="1125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1987" uniqueCount="1259">
   <si>
     <t>SAGOL</t>
   </si>
@@ -3415,6 +3416,408 @@
   </si>
   <si>
     <t>Assiut Core</t>
+  </si>
+  <si>
+    <t>GhostLine Racing</t>
+  </si>
+  <si>
+    <t>Shreyash Kinhikar</t>
+  </si>
+  <si>
+    <t>VectorDrive</t>
+  </si>
+  <si>
+    <t>Abdulrahman Saadeldin</t>
+  </si>
+  <si>
+    <t>Rohit Balaji N</t>
+  </si>
+  <si>
+    <t>Siga Siga Racing Team</t>
+  </si>
+  <si>
+    <t>Nikita Fokin</t>
+  </si>
+  <si>
+    <t>Nikolay Mikolaychuk</t>
+  </si>
+  <si>
+    <t>K. Smirnov Robotics LTD</t>
+  </si>
+  <si>
+    <t>Lunia</t>
+  </si>
+  <si>
+    <t>Zehao Wang</t>
+  </si>
+  <si>
+    <t>KU Leuven</t>
+  </si>
+  <si>
+    <t>Belgium</t>
+  </si>
+  <si>
+    <t>Cedric Hollande</t>
+  </si>
+  <si>
+    <t>xLAB, University of Pennsylvania</t>
+  </si>
+  <si>
+    <t>Traxon Racing</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>Ram Charan Akula</t>
+  </si>
+  <si>
+    <t>F1A</t>
+  </si>
+  <si>
+    <t>Shadow Ri</t>
+  </si>
+  <si>
+    <t>Sonic Ri</t>
+  </si>
+  <si>
+    <t>XOYO</t>
+  </si>
+  <si>
+    <t>Shashank</t>
+  </si>
+  <si>
+    <t>Chaarvi</t>
+  </si>
+  <si>
+    <t>Santhosh</t>
+  </si>
+  <si>
+    <t>Dhanalaxmi</t>
+  </si>
+  <si>
+    <t>M. S. Ramaiah University of Applied Sciences</t>
+  </si>
+  <si>
+    <t>Huginn &amp; Muninn</t>
+  </si>
+  <si>
+    <t>Aditya Choudhary</t>
+  </si>
+  <si>
+    <t>Ahmed El Ashiry</t>
+  </si>
+  <si>
+    <t>Hakuna_Matata</t>
+  </si>
+  <si>
+    <t>Shalem Bakth Singh Badampudi</t>
+  </si>
+  <si>
+    <t>Venkata Manvitha Tatikonda</t>
+  </si>
+  <si>
+    <t>Anudeep Dondapati</t>
+  </si>
+  <si>
+    <t>Venkata Karthik Thallam</t>
+  </si>
+  <si>
+    <t>armoured_alpha</t>
+  </si>
+  <si>
+    <t>nxtwave</t>
+  </si>
+  <si>
+    <t>Barq Racing</t>
+  </si>
+  <si>
+    <t>Abdullah Naeem</t>
+  </si>
+  <si>
+    <t>Muhammad Usman</t>
+  </si>
+  <si>
+    <t>Adil Mubashir Chaudhry</t>
+  </si>
+  <si>
+    <t>Sree Aslesh Penisetty</t>
+  </si>
+  <si>
+    <t>Team Abhiyaan</t>
+  </si>
+  <si>
+    <t>Alan Royce Gabriel Samuel</t>
+  </si>
+  <si>
+    <t>Ashwaat Tarun Thirukumarsubbiah Shriraam</t>
+  </si>
+  <si>
+    <t>Madhav Pradeep</t>
+  </si>
+  <si>
+    <t>Yash Purswani</t>
+  </si>
+  <si>
+    <t>singleroom</t>
+  </si>
+  <si>
+    <t>Manish Rasamalla</t>
+  </si>
+  <si>
+    <t>CEM Navigators</t>
+  </si>
+  <si>
+    <t>Shyam Rithin Suresh Kumar</t>
+  </si>
+  <si>
+    <t>Chitra Kaverappa</t>
+  </si>
+  <si>
+    <t>Manikandan Ganesan</t>
+  </si>
+  <si>
+    <t>Torque Dirty To Me</t>
+  </si>
+  <si>
+    <t>Krishna Chochipatla</t>
+  </si>
+  <si>
+    <t>Phantom Arrow</t>
+  </si>
+  <si>
+    <t>APEX</t>
+  </si>
+  <si>
+    <t>Dongbeen Jeon</t>
+  </si>
+  <si>
+    <t>Youngrok Kim</t>
+  </si>
+  <si>
+    <t>Joonhyung Im</t>
+  </si>
+  <si>
+    <t>Minji Jung</t>
+  </si>
+  <si>
+    <t>Jaehyung Choi</t>
+  </si>
+  <si>
+    <t>Inje University</t>
+  </si>
+  <si>
+    <t>Solo Dev</t>
+  </si>
+  <si>
+    <t>Yiu Wa Hung</t>
+  </si>
+  <si>
+    <t>Rodrigo Alcobero</t>
+  </si>
+  <si>
+    <t>Ignacio Bugueno</t>
+  </si>
+  <si>
+    <t>Argentina, Chile, Ecuador</t>
+  </si>
+  <si>
+    <t>Tk</t>
+  </si>
+  <si>
+    <t>Fangfei Fan</t>
+  </si>
+  <si>
+    <t>The University of New South Wales</t>
+  </si>
+  <si>
+    <t>YallaAE</t>
+  </si>
+  <si>
+    <t>MBZUAI</t>
+  </si>
+  <si>
+    <t>Botzilla</t>
+  </si>
+  <si>
+    <t>Nilum Mudaliarachchi</t>
+  </si>
+  <si>
+    <t>Tharusha Udana</t>
+  </si>
+  <si>
+    <t>University of Moratuwa</t>
+  </si>
+  <si>
+    <t>DaVinci</t>
+  </si>
+  <si>
+    <t>Ishan Bala</t>
+  </si>
+  <si>
+    <t>SpaceRacer</t>
+  </si>
+  <si>
+    <t>Junseo Jang</t>
+  </si>
+  <si>
+    <t>Jong-ah Ha</t>
+  </si>
+  <si>
+    <t>Jaehyeong Kim</t>
+  </si>
+  <si>
+    <t>Go-Go-Taro</t>
+  </si>
+  <si>
+    <t>Team Proboticists</t>
+  </si>
+  <si>
+    <t>Ankit Meda</t>
+  </si>
+  <si>
+    <t>Deepak G</t>
+  </si>
+  <si>
+    <t>Vidit Gupta</t>
+  </si>
+  <si>
+    <t>Priyanshu Bansal</t>
+  </si>
+  <si>
+    <t>Vansh Lohia</t>
+  </si>
+  <si>
+    <t>FirstName LastName</t>
+  </si>
+  <si>
+    <t>Penguin</t>
+  </si>
+  <si>
+    <t>Private</t>
+  </si>
+  <si>
+    <t>Madagascar</t>
+  </si>
+  <si>
+    <t>rulim</t>
+  </si>
+  <si>
+    <t>Mikhail Shulga</t>
+  </si>
+  <si>
+    <t>MIPT</t>
+  </si>
+  <si>
+    <t>Steven Joseph Ibrahim</t>
+  </si>
+  <si>
+    <t>Mohammed Yasser Mohammed</t>
+  </si>
+  <si>
+    <t>Sajda Mohammed Shaker</t>
+  </si>
+  <si>
+    <t>Jana Mahmoud Fahmy</t>
+  </si>
+  <si>
+    <t>Mohamed Fouad Elgohary</t>
+  </si>
+  <si>
+    <t>ASUF1Tenth</t>
+  </si>
+  <si>
+    <t>Mohamed Hany</t>
+  </si>
+  <si>
+    <t>Moaz Ahmed</t>
+  </si>
+  <si>
+    <t>Mohamed Mahmoud</t>
+  </si>
+  <si>
+    <t>Belal Anas</t>
+  </si>
+  <si>
+    <t>Faculty of Engineering, Ain Shams University</t>
+  </si>
+  <si>
+    <t>Light Year</t>
+  </si>
+  <si>
+    <t>Aahan Kumbham</t>
+  </si>
+  <si>
+    <t>Panther Creek High School</t>
+  </si>
+  <si>
+    <t>UNISAFE</t>
+  </si>
+  <si>
+    <t>Jaechan Shin</t>
+  </si>
+  <si>
+    <t>Sunhwi Kim</t>
+  </si>
+  <si>
+    <t>Ulsan National Institute of Science and Technology (UNIST)</t>
+  </si>
+  <si>
+    <t>*whoosh*</t>
+  </si>
+  <si>
+    <t>Abhishek Lakote</t>
+  </si>
+  <si>
+    <t>Aryan Pokhriyal</t>
+  </si>
+  <si>
+    <t>Mahin Sankleja</t>
+  </si>
+  <si>
+    <t>Oishi Nandi</t>
+  </si>
+  <si>
+    <t>Ratharv Rathore</t>
+  </si>
+  <si>
+    <t>Siddharth Sreejith</t>
+  </si>
+  <si>
+    <t>Uday Kalyan S</t>
+  </si>
+  <si>
+    <t>Uddipto Mandal</t>
+  </si>
+  <si>
+    <t>Yash Shah</t>
+  </si>
+  <si>
+    <t>Rostamza_JKU_ITS</t>
+  </si>
+  <si>
+    <t>Johannes Kepler University Linz</t>
+  </si>
+  <si>
+    <t>Alvin Cheriyan</t>
+  </si>
+  <si>
+    <t>Vishal Senthilkumar</t>
+  </si>
+  <si>
+    <t>Nikhilram</t>
+  </si>
+  <si>
+    <t>Siddharth R</t>
+  </si>
+  <si>
+    <t>Deva Kaushik</t>
+  </si>
+  <si>
+    <t>Δ 2RQ</t>
+  </si>
+  <si>
+    <t>Krishn Singh</t>
   </si>
 </sst>
 </file>
@@ -5794,85 +6197,37 @@
     </row>
   </sheetData>
   <mergeCells count="124">
-    <mergeCell ref="E159:E161"/>
-    <mergeCell ref="E135:E137"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="E142:E148"/>
-    <mergeCell ref="E149:E152"/>
-    <mergeCell ref="E154:E158"/>
-    <mergeCell ref="E111:E116"/>
-    <mergeCell ref="E117:E118"/>
-    <mergeCell ref="E122:E123"/>
-    <mergeCell ref="E124:E131"/>
-    <mergeCell ref="E132:E134"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="E99:E102"/>
-    <mergeCell ref="E103:E105"/>
-    <mergeCell ref="E106:E107"/>
-    <mergeCell ref="E108:E110"/>
-    <mergeCell ref="E71:E76"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="E84:E89"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="E35:E46"/>
-    <mergeCell ref="E50:E54"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E59:E65"/>
-    <mergeCell ref="E67:E70"/>
-    <mergeCell ref="E6:E14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E21:E24"/>
-    <mergeCell ref="E27:E31"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="A27:A31"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A35:A46"/>
-    <mergeCell ref="B35:B46"/>
-    <mergeCell ref="A6:A14"/>
-    <mergeCell ref="B6:B14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="B21:B24"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A71:A76"/>
-    <mergeCell ref="B71:B76"/>
-    <mergeCell ref="A77:A78"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="A50:A54"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="A59:A65"/>
-    <mergeCell ref="B59:B65"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="A99:A102"/>
-    <mergeCell ref="B99:B102"/>
-    <mergeCell ref="A103:A105"/>
-    <mergeCell ref="B103:B105"/>
-    <mergeCell ref="A81:A82"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="A84:A89"/>
-    <mergeCell ref="B84:B89"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="A117:A118"/>
-    <mergeCell ref="B117:B118"/>
-    <mergeCell ref="A122:A123"/>
-    <mergeCell ref="B122:B123"/>
-    <mergeCell ref="A124:A131"/>
-    <mergeCell ref="B124:B131"/>
-    <mergeCell ref="A106:A107"/>
-    <mergeCell ref="B106:B107"/>
-    <mergeCell ref="A108:A110"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="A111:A116"/>
-    <mergeCell ref="B111:B116"/>
+    <mergeCell ref="D27:D31"/>
+    <mergeCell ref="D21:D24"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="D6:D14"/>
+    <mergeCell ref="D81:D82"/>
+    <mergeCell ref="D77:D78"/>
+    <mergeCell ref="D71:D76"/>
+    <mergeCell ref="D67:D70"/>
+    <mergeCell ref="D59:D65"/>
+    <mergeCell ref="D55:D56"/>
+    <mergeCell ref="D50:D54"/>
+    <mergeCell ref="D35:D46"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="D103:D105"/>
+    <mergeCell ref="D99:D102"/>
+    <mergeCell ref="D111:D116"/>
+    <mergeCell ref="D108:D110"/>
+    <mergeCell ref="D106:D107"/>
+    <mergeCell ref="D117:D118"/>
+    <mergeCell ref="D95:D97"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="D84:D89"/>
+    <mergeCell ref="D154:D158"/>
+    <mergeCell ref="D159:D161"/>
+    <mergeCell ref="D124:D131"/>
+    <mergeCell ref="D122:D123"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="D135:D137"/>
+    <mergeCell ref="D132:D134"/>
+    <mergeCell ref="D149:D152"/>
+    <mergeCell ref="D142:D148"/>
     <mergeCell ref="A142:A148"/>
     <mergeCell ref="B142:B148"/>
     <mergeCell ref="A159:A161"/>
@@ -5887,37 +6242,85 @@
     <mergeCell ref="B135:B137"/>
     <mergeCell ref="A138:A141"/>
     <mergeCell ref="B138:B141"/>
-    <mergeCell ref="D154:D158"/>
-    <mergeCell ref="D159:D161"/>
-    <mergeCell ref="D124:D131"/>
-    <mergeCell ref="D122:D123"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="D135:D137"/>
-    <mergeCell ref="D132:D134"/>
-    <mergeCell ref="D149:D152"/>
-    <mergeCell ref="D142:D148"/>
-    <mergeCell ref="D103:D105"/>
-    <mergeCell ref="D99:D102"/>
-    <mergeCell ref="D111:D116"/>
-    <mergeCell ref="D108:D110"/>
-    <mergeCell ref="D106:D107"/>
-    <mergeCell ref="D117:D118"/>
-    <mergeCell ref="D95:D97"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="D84:D89"/>
-    <mergeCell ref="D27:D31"/>
-    <mergeCell ref="D21:D24"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="D6:D14"/>
-    <mergeCell ref="D81:D82"/>
-    <mergeCell ref="D77:D78"/>
-    <mergeCell ref="D71:D76"/>
-    <mergeCell ref="D67:D70"/>
-    <mergeCell ref="D59:D65"/>
-    <mergeCell ref="D55:D56"/>
-    <mergeCell ref="D50:D54"/>
-    <mergeCell ref="D35:D46"/>
-    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="A117:A118"/>
+    <mergeCell ref="B117:B118"/>
+    <mergeCell ref="A122:A123"/>
+    <mergeCell ref="B122:B123"/>
+    <mergeCell ref="A124:A131"/>
+    <mergeCell ref="B124:B131"/>
+    <mergeCell ref="A106:A107"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="A108:A110"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="A111:A116"/>
+    <mergeCell ref="B111:B116"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="A99:A102"/>
+    <mergeCell ref="B99:B102"/>
+    <mergeCell ref="A103:A105"/>
+    <mergeCell ref="B103:B105"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="A84:A89"/>
+    <mergeCell ref="B84:B89"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A71:A76"/>
+    <mergeCell ref="B71:B76"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="A50:A54"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="A59:A65"/>
+    <mergeCell ref="B59:B65"/>
+    <mergeCell ref="A27:A31"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A35:A46"/>
+    <mergeCell ref="B35:B46"/>
+    <mergeCell ref="A6:A14"/>
+    <mergeCell ref="B6:B14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="E35:E46"/>
+    <mergeCell ref="E50:E54"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E59:E65"/>
+    <mergeCell ref="E67:E70"/>
+    <mergeCell ref="E6:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E21:E24"/>
+    <mergeCell ref="E27:E31"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="E99:E102"/>
+    <mergeCell ref="E103:E105"/>
+    <mergeCell ref="E106:E107"/>
+    <mergeCell ref="E108:E110"/>
+    <mergeCell ref="E71:E76"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="E84:E89"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="E159:E161"/>
+    <mergeCell ref="E135:E137"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="E142:E148"/>
+    <mergeCell ref="E149:E152"/>
+    <mergeCell ref="E154:E158"/>
+    <mergeCell ref="E111:E116"/>
+    <mergeCell ref="E117:E118"/>
+    <mergeCell ref="E122:E123"/>
+    <mergeCell ref="E124:E131"/>
+    <mergeCell ref="E132:E134"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -7889,47 +8292,85 @@
     </row>
   </sheetData>
   <mergeCells count="144">
-    <mergeCell ref="E157:E159"/>
-    <mergeCell ref="E160:E164"/>
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="E170:E171"/>
-    <mergeCell ref="E102:E111"/>
-    <mergeCell ref="E112:E116"/>
-    <mergeCell ref="E117:E122"/>
-    <mergeCell ref="E123:E129"/>
-    <mergeCell ref="E130:E141"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="E150:E151"/>
-    <mergeCell ref="E152:E156"/>
-    <mergeCell ref="E68:E69"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="E75:E78"/>
-    <mergeCell ref="E80:E82"/>
-    <mergeCell ref="E84:E85"/>
-    <mergeCell ref="E86:E91"/>
-    <mergeCell ref="E92:E94"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="D62:D64"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E4:E7"/>
-    <mergeCell ref="E8:E15"/>
-    <mergeCell ref="E16:E19"/>
-    <mergeCell ref="E21:E23"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="E26:E30"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="E33:E37"/>
-    <mergeCell ref="E38:E45"/>
-    <mergeCell ref="E46:E51"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="E62:E64"/>
-    <mergeCell ref="E66:E67"/>
-    <mergeCell ref="B8:B15"/>
-    <mergeCell ref="D8:D15"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="D76:D78"/>
+    <mergeCell ref="D71:D73"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="D92:D94"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="A46:A51"/>
+    <mergeCell ref="B46:B51"/>
+    <mergeCell ref="D46:D51"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="B62:B64"/>
+    <mergeCell ref="A152:A156"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="A150:A151"/>
+    <mergeCell ref="A123:A129"/>
+    <mergeCell ref="A130:A141"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="A75:A78"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="A170:A171"/>
+    <mergeCell ref="B170:B171"/>
+    <mergeCell ref="D170:D171"/>
+    <mergeCell ref="A160:A164"/>
+    <mergeCell ref="B160:B164"/>
+    <mergeCell ref="D160:D164"/>
+    <mergeCell ref="A157:A159"/>
+    <mergeCell ref="B157:B159"/>
+    <mergeCell ref="D157:D159"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="B75:B78"/>
+    <mergeCell ref="B80:B82"/>
+    <mergeCell ref="D80:D82"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="D84:D85"/>
+    <mergeCell ref="B112:B116"/>
+    <mergeCell ref="D112:D116"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="D95:D97"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B86:B91"/>
+    <mergeCell ref="D86:D91"/>
+    <mergeCell ref="A112:A116"/>
+    <mergeCell ref="A86:A91"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="A102:A111"/>
+    <mergeCell ref="A117:A122"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="D150:D151"/>
+    <mergeCell ref="B152:B156"/>
+    <mergeCell ref="D152:D156"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="B117:B122"/>
+    <mergeCell ref="D117:D122"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="B102:B111"/>
+    <mergeCell ref="D102:D111"/>
+    <mergeCell ref="B123:B129"/>
+    <mergeCell ref="D123:D129"/>
+    <mergeCell ref="B130:B141"/>
+    <mergeCell ref="D130:D141"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="D2:D3"/>
@@ -7954,85 +8395,47 @@
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="D16:D19"/>
     <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="D150:D151"/>
-    <mergeCell ref="B152:B156"/>
-    <mergeCell ref="D152:D156"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="B117:B122"/>
-    <mergeCell ref="D117:D122"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="B102:B111"/>
-    <mergeCell ref="D102:D111"/>
-    <mergeCell ref="B123:B129"/>
-    <mergeCell ref="D123:D129"/>
-    <mergeCell ref="B130:B141"/>
-    <mergeCell ref="D130:D141"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="B75:B78"/>
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="D80:D82"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="D84:D85"/>
-    <mergeCell ref="B112:B116"/>
-    <mergeCell ref="D112:D116"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="D95:D97"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B86:B91"/>
-    <mergeCell ref="D86:D91"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="A170:A171"/>
-    <mergeCell ref="B170:B171"/>
-    <mergeCell ref="D170:D171"/>
-    <mergeCell ref="A160:A164"/>
-    <mergeCell ref="B160:B164"/>
-    <mergeCell ref="D160:D164"/>
-    <mergeCell ref="A157:A159"/>
-    <mergeCell ref="B157:B159"/>
-    <mergeCell ref="D157:D159"/>
-    <mergeCell ref="A112:A116"/>
-    <mergeCell ref="A86:A91"/>
-    <mergeCell ref="A84:A85"/>
-    <mergeCell ref="A102:A111"/>
-    <mergeCell ref="A117:A122"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="A152:A156"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="A150:A151"/>
-    <mergeCell ref="A123:A129"/>
-    <mergeCell ref="A130:A141"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A75:A78"/>
-    <mergeCell ref="A66:A67"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="D76:D78"/>
-    <mergeCell ref="D71:D73"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="D92:D94"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="A46:A51"/>
-    <mergeCell ref="B46:B51"/>
-    <mergeCell ref="D46:D51"/>
-    <mergeCell ref="A52:A53"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="B62:B64"/>
+    <mergeCell ref="D62:D64"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="E8:E15"/>
+    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="E26:E30"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="E33:E37"/>
+    <mergeCell ref="E38:E45"/>
+    <mergeCell ref="E46:E51"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="E62:E64"/>
+    <mergeCell ref="E66:E67"/>
+    <mergeCell ref="B8:B15"/>
+    <mergeCell ref="D8:D15"/>
+    <mergeCell ref="E68:E69"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="E75:E78"/>
+    <mergeCell ref="E80:E82"/>
+    <mergeCell ref="E84:E85"/>
+    <mergeCell ref="E86:E91"/>
+    <mergeCell ref="E92:E94"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="E157:E159"/>
+    <mergeCell ref="E160:E164"/>
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="E170:E171"/>
+    <mergeCell ref="E102:E111"/>
+    <mergeCell ref="E112:E116"/>
+    <mergeCell ref="E117:E122"/>
+    <mergeCell ref="E123:E129"/>
+    <mergeCell ref="E130:E141"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="E150:E151"/>
+    <mergeCell ref="E152:E156"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -9867,90 +10270,29 @@
     </row>
   </sheetData>
   <mergeCells count="132">
-    <mergeCell ref="A145:A147"/>
-    <mergeCell ref="B145:B147"/>
-    <mergeCell ref="D145:D147"/>
-    <mergeCell ref="E145:E147"/>
-    <mergeCell ref="A149:A150"/>
-    <mergeCell ref="B149:B150"/>
-    <mergeCell ref="D149:D150"/>
-    <mergeCell ref="E149:E150"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="D131:D133"/>
-    <mergeCell ref="E131:E133"/>
-    <mergeCell ref="A135:A138"/>
-    <mergeCell ref="B135:B138"/>
-    <mergeCell ref="D135:D138"/>
-    <mergeCell ref="E135:E138"/>
-    <mergeCell ref="A139:A141"/>
-    <mergeCell ref="B139:B141"/>
-    <mergeCell ref="D139:D141"/>
-    <mergeCell ref="E139:E141"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="D114:D117"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="A118:A127"/>
-    <mergeCell ref="B118:B127"/>
-    <mergeCell ref="D118:D127"/>
-    <mergeCell ref="E118:E127"/>
-    <mergeCell ref="A81:A85"/>
-    <mergeCell ref="B81:B85"/>
-    <mergeCell ref="D81:D85"/>
-    <mergeCell ref="E81:E85"/>
-    <mergeCell ref="E87:E89"/>
-    <mergeCell ref="A90:A91"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="D90:D91"/>
-    <mergeCell ref="E90:E91"/>
-    <mergeCell ref="D1:D4"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E1:E4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="B65:B71"/>
-    <mergeCell ref="D65:D71"/>
-    <mergeCell ref="D73:D75"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="E57:E59"/>
-    <mergeCell ref="A60:A64"/>
-    <mergeCell ref="B60:B64"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="B51:B53"/>
-    <mergeCell ref="D51:D53"/>
-    <mergeCell ref="E51:E53"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="E42:E46"/>
-    <mergeCell ref="E73:E75"/>
-    <mergeCell ref="A73:A75"/>
-    <mergeCell ref="B73:B75"/>
-    <mergeCell ref="E65:E71"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="D48:D50"/>
+    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="A129:A130"/>
+    <mergeCell ref="B129:B130"/>
+    <mergeCell ref="D129:D130"/>
+    <mergeCell ref="E129:E130"/>
+    <mergeCell ref="A87:A89"/>
+    <mergeCell ref="B87:B89"/>
+    <mergeCell ref="D87:D89"/>
+    <mergeCell ref="A92:A97"/>
+    <mergeCell ref="B92:B97"/>
+    <mergeCell ref="D92:D97"/>
+    <mergeCell ref="E92:E97"/>
+    <mergeCell ref="A99:A109"/>
+    <mergeCell ref="B99:B109"/>
+    <mergeCell ref="D99:D109"/>
+    <mergeCell ref="E99:E109"/>
+    <mergeCell ref="A76:A80"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="D76:D80"/>
+    <mergeCell ref="E76:E80"/>
+    <mergeCell ref="A65:A71"/>
     <mergeCell ref="D29:D31"/>
     <mergeCell ref="E29:E31"/>
     <mergeCell ref="A20:A22"/>
@@ -9975,30 +10317,91 @@
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="B29:B31"/>
     <mergeCell ref="B1:B4"/>
+    <mergeCell ref="B65:B71"/>
+    <mergeCell ref="D65:D71"/>
+    <mergeCell ref="D73:D75"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="E57:E59"/>
+    <mergeCell ref="A60:A64"/>
+    <mergeCell ref="B60:B64"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="D51:D53"/>
+    <mergeCell ref="E51:E53"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="E42:E46"/>
+    <mergeCell ref="E73:E75"/>
+    <mergeCell ref="A73:A75"/>
+    <mergeCell ref="B73:B75"/>
+    <mergeCell ref="E65:E71"/>
     <mergeCell ref="A48:A50"/>
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="D48:D50"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="A129:A130"/>
-    <mergeCell ref="B129:B130"/>
-    <mergeCell ref="D129:D130"/>
-    <mergeCell ref="E129:E130"/>
-    <mergeCell ref="A87:A89"/>
-    <mergeCell ref="B87:B89"/>
-    <mergeCell ref="D87:D89"/>
-    <mergeCell ref="A92:A97"/>
-    <mergeCell ref="B92:B97"/>
-    <mergeCell ref="D92:D97"/>
-    <mergeCell ref="E92:E97"/>
-    <mergeCell ref="A99:A109"/>
-    <mergeCell ref="B99:B109"/>
-    <mergeCell ref="D99:D109"/>
-    <mergeCell ref="E99:E109"/>
-    <mergeCell ref="A76:A80"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="D76:D80"/>
-    <mergeCell ref="E76:E80"/>
-    <mergeCell ref="A65:A71"/>
+    <mergeCell ref="D1:D4"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E1:E4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="A81:A85"/>
+    <mergeCell ref="B81:B85"/>
+    <mergeCell ref="D81:D85"/>
+    <mergeCell ref="E81:E85"/>
+    <mergeCell ref="E87:E89"/>
+    <mergeCell ref="A90:A91"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="D90:D91"/>
+    <mergeCell ref="E90:E91"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="D114:D117"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="A118:A127"/>
+    <mergeCell ref="B118:B127"/>
+    <mergeCell ref="D118:D127"/>
+    <mergeCell ref="E118:E127"/>
+    <mergeCell ref="A145:A147"/>
+    <mergeCell ref="B145:B147"/>
+    <mergeCell ref="D145:D147"/>
+    <mergeCell ref="E145:E147"/>
+    <mergeCell ref="A149:A150"/>
+    <mergeCell ref="B149:B150"/>
+    <mergeCell ref="D149:D150"/>
+    <mergeCell ref="E149:E150"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="D131:D133"/>
+    <mergeCell ref="E131:E133"/>
+    <mergeCell ref="A135:A138"/>
+    <mergeCell ref="B135:B138"/>
+    <mergeCell ref="D135:D138"/>
+    <mergeCell ref="E135:E138"/>
+    <mergeCell ref="A139:A141"/>
+    <mergeCell ref="B139:B141"/>
+    <mergeCell ref="D139:D141"/>
+    <mergeCell ref="E139:E141"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -11797,31 +12200,57 @@
     </row>
   </sheetData>
   <mergeCells count="92">
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="D36:D38"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="B28:B31"/>
-    <mergeCell ref="A32:A35"/>
-    <mergeCell ref="B32:B35"/>
-    <mergeCell ref="D32:D35"/>
-    <mergeCell ref="E32:E35"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D83:D89"/>
-    <mergeCell ref="E83:E89"/>
-    <mergeCell ref="A62:A67"/>
-    <mergeCell ref="B62:B67"/>
-    <mergeCell ref="D62:D67"/>
-    <mergeCell ref="E62:E67"/>
-    <mergeCell ref="A69:A72"/>
-    <mergeCell ref="B69:B72"/>
-    <mergeCell ref="D69:D72"/>
-    <mergeCell ref="E69:E72"/>
-    <mergeCell ref="A73:A82"/>
-    <mergeCell ref="B73:B82"/>
-    <mergeCell ref="D73:D82"/>
-    <mergeCell ref="E73:E82"/>
+    <mergeCell ref="A90:A95"/>
+    <mergeCell ref="A96:A100"/>
+    <mergeCell ref="A57:A61"/>
+    <mergeCell ref="A49:A54"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="A42:A47"/>
+    <mergeCell ref="A83:A89"/>
+    <mergeCell ref="A154:A156"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="D154:D156"/>
+    <mergeCell ref="E154:E156"/>
+    <mergeCell ref="A157:A158"/>
+    <mergeCell ref="B157:B158"/>
+    <mergeCell ref="D157:D158"/>
+    <mergeCell ref="E157:E158"/>
+    <mergeCell ref="D90:D95"/>
+    <mergeCell ref="E90:E95"/>
+    <mergeCell ref="B96:B100"/>
+    <mergeCell ref="D96:D100"/>
+    <mergeCell ref="E96:E100"/>
+    <mergeCell ref="B90:B95"/>
+    <mergeCell ref="D49:D54"/>
+    <mergeCell ref="E49:E54"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="D57:D61"/>
+    <mergeCell ref="E57:E61"/>
+    <mergeCell ref="B49:B54"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="B42:B47"/>
+    <mergeCell ref="D42:D47"/>
+    <mergeCell ref="E42:E47"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="A15:A24"/>
+    <mergeCell ref="B15:B24"/>
+    <mergeCell ref="D15:D24"/>
+    <mergeCell ref="E15:E24"/>
+    <mergeCell ref="D28:D31"/>
+    <mergeCell ref="E28:E31"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="E5:E8"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="B9:B13"/>
+    <mergeCell ref="D9:D13"/>
+    <mergeCell ref="E9:E13"/>
     <mergeCell ref="A129:A151"/>
     <mergeCell ref="B129:B151"/>
     <mergeCell ref="D129:D151"/>
@@ -11838,57 +12267,31 @@
     <mergeCell ref="B126:B128"/>
     <mergeCell ref="D126:D128"/>
     <mergeCell ref="E126:E128"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="D5:D8"/>
-    <mergeCell ref="E5:E8"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="B9:B13"/>
-    <mergeCell ref="D9:D13"/>
-    <mergeCell ref="E9:E13"/>
-    <mergeCell ref="A15:A24"/>
-    <mergeCell ref="B15:B24"/>
-    <mergeCell ref="D15:D24"/>
-    <mergeCell ref="E15:E24"/>
-    <mergeCell ref="D28:D31"/>
-    <mergeCell ref="E28:E31"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="D39:D41"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="B42:B47"/>
-    <mergeCell ref="D42:D47"/>
-    <mergeCell ref="E42:E47"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="D49:D54"/>
-    <mergeCell ref="E49:E54"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="D57:D61"/>
-    <mergeCell ref="E57:E61"/>
-    <mergeCell ref="B49:B54"/>
-    <mergeCell ref="D90:D95"/>
-    <mergeCell ref="E90:E95"/>
-    <mergeCell ref="B96:B100"/>
-    <mergeCell ref="D96:D100"/>
-    <mergeCell ref="E96:E100"/>
-    <mergeCell ref="B90:B95"/>
-    <mergeCell ref="A154:A156"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="D154:D156"/>
-    <mergeCell ref="E154:E156"/>
-    <mergeCell ref="A157:A158"/>
-    <mergeCell ref="B157:B158"/>
-    <mergeCell ref="D157:D158"/>
-    <mergeCell ref="E157:E158"/>
-    <mergeCell ref="A90:A95"/>
-    <mergeCell ref="A96:A100"/>
-    <mergeCell ref="A57:A61"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A42:A47"/>
-    <mergeCell ref="A83:A89"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D83:D89"/>
+    <mergeCell ref="E83:E89"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="B62:B67"/>
+    <mergeCell ref="D62:D67"/>
+    <mergeCell ref="E62:E67"/>
+    <mergeCell ref="A69:A72"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="D69:D72"/>
+    <mergeCell ref="E69:E72"/>
+    <mergeCell ref="A73:A82"/>
+    <mergeCell ref="B73:B82"/>
+    <mergeCell ref="D73:D82"/>
+    <mergeCell ref="E73:E82"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="D36:D38"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="B32:B35"/>
+    <mergeCell ref="D32:D35"/>
+    <mergeCell ref="E32:E35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14301,102 +14704,30 @@
     </row>
   </sheetData>
   <mergeCells count="144">
-    <mergeCell ref="A182:A183"/>
-    <mergeCell ref="B182:B183"/>
-    <mergeCell ref="D182:D183"/>
-    <mergeCell ref="E182:E183"/>
-    <mergeCell ref="A185:A191"/>
-    <mergeCell ref="B185:B191"/>
-    <mergeCell ref="D185:D191"/>
-    <mergeCell ref="E185:E191"/>
-    <mergeCell ref="A176:A177"/>
-    <mergeCell ref="B176:B177"/>
-    <mergeCell ref="D176:D177"/>
-    <mergeCell ref="E176:E177"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="A168:A170"/>
-    <mergeCell ref="B168:B170"/>
-    <mergeCell ref="D168:D170"/>
-    <mergeCell ref="E168:E170"/>
-    <mergeCell ref="A171:A175"/>
-    <mergeCell ref="B171:B175"/>
-    <mergeCell ref="D171:D175"/>
-    <mergeCell ref="E171:E175"/>
-    <mergeCell ref="A154:A161"/>
-    <mergeCell ref="B154:B161"/>
-    <mergeCell ref="D154:D161"/>
-    <mergeCell ref="E154:E161"/>
-    <mergeCell ref="A163:A165"/>
-    <mergeCell ref="B163:B165"/>
-    <mergeCell ref="D163:D165"/>
-    <mergeCell ref="E163:E165"/>
-    <mergeCell ref="A145:A149"/>
-    <mergeCell ref="B145:B149"/>
-    <mergeCell ref="D145:D149"/>
-    <mergeCell ref="E145:E149"/>
-    <mergeCell ref="A151:A153"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="D151:D153"/>
-    <mergeCell ref="E151:E153"/>
-    <mergeCell ref="D139:D141"/>
-    <mergeCell ref="E139:E141"/>
-    <mergeCell ref="A142:A143"/>
-    <mergeCell ref="B142:B143"/>
-    <mergeCell ref="D142:D143"/>
-    <mergeCell ref="E142:E143"/>
-    <mergeCell ref="D125:D127"/>
-    <mergeCell ref="E125:E127"/>
-    <mergeCell ref="A132:A133"/>
-    <mergeCell ref="B132:B133"/>
-    <mergeCell ref="D132:D133"/>
-    <mergeCell ref="E132:E133"/>
-    <mergeCell ref="A111:A112"/>
-    <mergeCell ref="B111:B112"/>
-    <mergeCell ref="D111:D112"/>
-    <mergeCell ref="E111:E112"/>
-    <mergeCell ref="A115:A123"/>
-    <mergeCell ref="B115:B123"/>
-    <mergeCell ref="D115:D123"/>
-    <mergeCell ref="E115:E123"/>
-    <mergeCell ref="A103:A106"/>
-    <mergeCell ref="B103:B106"/>
-    <mergeCell ref="D103:D106"/>
-    <mergeCell ref="E103:E106"/>
-    <mergeCell ref="A107:A110"/>
-    <mergeCell ref="B107:B110"/>
-    <mergeCell ref="D107:D110"/>
-    <mergeCell ref="E107:E110"/>
-    <mergeCell ref="D97:D99"/>
-    <mergeCell ref="E97:E99"/>
-    <mergeCell ref="A101:A102"/>
-    <mergeCell ref="B101:B102"/>
-    <mergeCell ref="D101:D102"/>
-    <mergeCell ref="E101:E102"/>
-    <mergeCell ref="D81:D87"/>
-    <mergeCell ref="E81:E87"/>
-    <mergeCell ref="A90:A96"/>
-    <mergeCell ref="B90:B96"/>
-    <mergeCell ref="D90:D96"/>
-    <mergeCell ref="E90:E96"/>
-    <mergeCell ref="D68:D77"/>
-    <mergeCell ref="E68:E77"/>
-    <mergeCell ref="A78:A79"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="D78:D79"/>
-    <mergeCell ref="E78:E79"/>
-    <mergeCell ref="A59:A67"/>
-    <mergeCell ref="B59:B67"/>
-    <mergeCell ref="D59:D67"/>
-    <mergeCell ref="E59:E67"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="D10:D14"/>
+    <mergeCell ref="E10:E14"/>
+    <mergeCell ref="A195:A198"/>
+    <mergeCell ref="B195:B198"/>
+    <mergeCell ref="D195:D198"/>
+    <mergeCell ref="E195:E198"/>
+    <mergeCell ref="A199:A201"/>
+    <mergeCell ref="B199:B201"/>
+    <mergeCell ref="D199:D201"/>
+    <mergeCell ref="E199:E201"/>
+    <mergeCell ref="D29:D35"/>
+    <mergeCell ref="E29:E35"/>
+    <mergeCell ref="A38:A42"/>
+    <mergeCell ref="B38:B42"/>
+    <mergeCell ref="D38:D42"/>
+    <mergeCell ref="E38:E42"/>
+    <mergeCell ref="D16:D25"/>
+    <mergeCell ref="E16:E25"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="D26:D28"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="D53:D58"/>
+    <mergeCell ref="E53:E58"/>
     <mergeCell ref="A4:A8"/>
     <mergeCell ref="B4:B8"/>
     <mergeCell ref="D4:D8"/>
@@ -14421,30 +14752,1865 @@
     <mergeCell ref="B29:B35"/>
     <mergeCell ref="A16:A25"/>
     <mergeCell ref="B16:B25"/>
-    <mergeCell ref="D10:D14"/>
-    <mergeCell ref="E10:E14"/>
-    <mergeCell ref="A195:A198"/>
-    <mergeCell ref="B195:B198"/>
-    <mergeCell ref="D195:D198"/>
-    <mergeCell ref="E195:E198"/>
-    <mergeCell ref="A199:A201"/>
-    <mergeCell ref="B199:B201"/>
-    <mergeCell ref="D199:D201"/>
-    <mergeCell ref="E199:E201"/>
-    <mergeCell ref="D29:D35"/>
-    <mergeCell ref="E29:E35"/>
-    <mergeCell ref="A38:A42"/>
-    <mergeCell ref="B38:B42"/>
-    <mergeCell ref="D38:D42"/>
-    <mergeCell ref="E38:E42"/>
-    <mergeCell ref="D16:D25"/>
-    <mergeCell ref="E16:E25"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="D26:D28"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="D53:D58"/>
-    <mergeCell ref="E53:E58"/>
+    <mergeCell ref="A59:A67"/>
+    <mergeCell ref="B59:B67"/>
+    <mergeCell ref="D59:D67"/>
+    <mergeCell ref="E59:E67"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="D81:D87"/>
+    <mergeCell ref="E81:E87"/>
+    <mergeCell ref="A90:A96"/>
+    <mergeCell ref="B90:B96"/>
+    <mergeCell ref="D90:D96"/>
+    <mergeCell ref="E90:E96"/>
+    <mergeCell ref="D68:D77"/>
+    <mergeCell ref="E68:E77"/>
+    <mergeCell ref="A78:A79"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="D78:D79"/>
+    <mergeCell ref="E78:E79"/>
+    <mergeCell ref="A103:A106"/>
+    <mergeCell ref="B103:B106"/>
+    <mergeCell ref="D103:D106"/>
+    <mergeCell ref="E103:E106"/>
+    <mergeCell ref="A107:A110"/>
+    <mergeCell ref="B107:B110"/>
+    <mergeCell ref="D107:D110"/>
+    <mergeCell ref="E107:E110"/>
+    <mergeCell ref="D97:D99"/>
+    <mergeCell ref="E97:E99"/>
+    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="B101:B102"/>
+    <mergeCell ref="D101:D102"/>
+    <mergeCell ref="E101:E102"/>
+    <mergeCell ref="D125:D127"/>
+    <mergeCell ref="E125:E127"/>
+    <mergeCell ref="A132:A133"/>
+    <mergeCell ref="B132:B133"/>
+    <mergeCell ref="D132:D133"/>
+    <mergeCell ref="E132:E133"/>
+    <mergeCell ref="A111:A112"/>
+    <mergeCell ref="B111:B112"/>
+    <mergeCell ref="D111:D112"/>
+    <mergeCell ref="E111:E112"/>
+    <mergeCell ref="A115:A123"/>
+    <mergeCell ref="B115:B123"/>
+    <mergeCell ref="D115:D123"/>
+    <mergeCell ref="E115:E123"/>
+    <mergeCell ref="A145:A149"/>
+    <mergeCell ref="B145:B149"/>
+    <mergeCell ref="D145:D149"/>
+    <mergeCell ref="E145:E149"/>
+    <mergeCell ref="A151:A153"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="D151:D153"/>
+    <mergeCell ref="E151:E153"/>
+    <mergeCell ref="D139:D141"/>
+    <mergeCell ref="E139:E141"/>
+    <mergeCell ref="A142:A143"/>
+    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="D142:D143"/>
+    <mergeCell ref="E142:E143"/>
+    <mergeCell ref="A168:A170"/>
+    <mergeCell ref="B168:B170"/>
+    <mergeCell ref="D168:D170"/>
+    <mergeCell ref="E168:E170"/>
+    <mergeCell ref="A171:A175"/>
+    <mergeCell ref="B171:B175"/>
+    <mergeCell ref="D171:D175"/>
+    <mergeCell ref="E171:E175"/>
+    <mergeCell ref="A154:A161"/>
+    <mergeCell ref="B154:B161"/>
+    <mergeCell ref="D154:D161"/>
+    <mergeCell ref="E154:E161"/>
+    <mergeCell ref="A163:A165"/>
+    <mergeCell ref="B163:B165"/>
+    <mergeCell ref="D163:D165"/>
+    <mergeCell ref="E163:E165"/>
+    <mergeCell ref="A182:A183"/>
+    <mergeCell ref="B182:B183"/>
+    <mergeCell ref="D182:D183"/>
+    <mergeCell ref="E182:E183"/>
+    <mergeCell ref="A185:A191"/>
+    <mergeCell ref="B185:B191"/>
+    <mergeCell ref="D185:D191"/>
+    <mergeCell ref="E185:E191"/>
+    <mergeCell ref="A176:A177"/>
+    <mergeCell ref="B176:B177"/>
+    <mergeCell ref="D176:D177"/>
+    <mergeCell ref="E176:E177"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="E178:E181"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC4CFA97-D216-4292-8965-1641300B15B3}">
+  <dimension ref="A1:E135"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="4.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.36328125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="39.1796875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="29.90625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.7265625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="2">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1126</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>1128</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>965</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1129</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>5</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="2" t="s">
+        <v>1132</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>1135</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>1136</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>1087</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>1138</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>1139</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>1017</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>1026</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="2" t="s">
+        <v>1018</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="2" t="s">
+        <v>1019</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="2" t="s">
+        <v>1020</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="2" t="s">
+        <v>1021</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="2" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="2" t="s">
+        <v>1023</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="2" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="2" t="s">
+        <v>1025</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
+        <v>10</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
+        <v>11</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>1142</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
+        <v>12</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>970</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>971</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>978</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>13</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>1144</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>1143</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="2" t="s">
+        <v>1145</v>
+      </c>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>14</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>1147</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>1151</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="2" t="s">
+        <v>1148</v>
+      </c>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="2" t="s">
+        <v>1149</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="2" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" s="2">
+        <v>15</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>1153</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" s="4">
+        <v>16</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>688</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>693</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="2" t="s">
+        <v>1154</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" s="4">
+        <v>17</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>1156</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="2" t="s">
+        <v>1158</v>
+      </c>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="2" t="s">
+        <v>1159</v>
+      </c>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="2">
+        <v>18</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38" s="2">
+        <v>19</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>1049</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" s="4">
+        <v>20</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="2" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="2" t="s">
+        <v>1165</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" s="2">
+        <v>21</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>1028</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" s="2">
+        <v>22</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>1166</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44" s="4">
+        <v>23</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>1168</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="2" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" s="4"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="2" t="s">
+        <v>1170</v>
+      </c>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" s="4"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48" s="2">
+        <v>24</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" s="2">
+        <v>25</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>1173</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" s="4">
+        <v>26</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>1174</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" s="4"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="2" t="s">
+        <v>1176</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" s="4"/>
+      <c r="B52" s="4"/>
+      <c r="C52" s="2" t="s">
+        <v>1177</v>
+      </c>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" s="2">
+        <v>27</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>1178</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>1179</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54" s="2">
+        <v>28</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>889</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" s="4">
+        <v>29</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>1181</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>1182</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>1187</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" s="4"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="2" t="s">
+        <v>1183</v>
+      </c>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A57" s="4"/>
+      <c r="B57" s="4"/>
+      <c r="C57" s="2" t="s">
+        <v>1184</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="2" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" s="2">
+        <v>30</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>1188</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" s="4">
+        <v>31</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>680</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>1192</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" s="4"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="2" t="s">
+        <v>1190</v>
+      </c>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65" s="4"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="2" t="s">
+        <v>1191</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66" s="2">
+        <v>32</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>1194</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67" s="2">
+        <v>33</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>1196</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>1197</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A68" s="4">
+        <v>34</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>1198</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>1199</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>1201</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69" s="4"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="2" t="s">
+        <v>1200</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70" s="2">
+        <v>35</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A71" s="2">
+        <v>36</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>860</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A72" s="4">
+        <v>37</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>1204</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>927</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" s="4"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="2" t="s">
+        <v>928</v>
+      </c>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74" s="4">
+        <v>38</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A75" s="4"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="2" t="s">
+        <v>1206</v>
+      </c>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A76" s="4"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="2" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D76" s="4"/>
+      <c r="E76" s="4"/>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A77" s="2">
+        <v>39</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>1208</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A78" s="4">
+        <v>40</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>1209</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A79" s="4"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="2" t="s">
+        <v>1210</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4"/>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A80" s="4"/>
+      <c r="B80" s="4"/>
+      <c r="C80" s="2" t="s">
+        <v>1211</v>
+      </c>
+      <c r="D80" s="4"/>
+      <c r="E80" s="4"/>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A81" s="4"/>
+      <c r="B81" s="4"/>
+      <c r="C81" s="2" t="s">
+        <v>1212</v>
+      </c>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4"/>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A82" s="4"/>
+      <c r="B82" s="4"/>
+      <c r="C82" s="2" t="s">
+        <v>1213</v>
+      </c>
+      <c r="D82" s="4"/>
+      <c r="E82" s="4"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A83" s="4"/>
+      <c r="B83" s="4"/>
+      <c r="C83" s="2" t="s">
+        <v>1214</v>
+      </c>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A84" s="2">
+        <v>41</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>1215</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A85" s="2">
+        <v>42</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>1216</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>1217</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A86" s="2">
+        <v>43</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A87" s="2">
+        <v>44</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>1220</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>1221</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A88" s="4">
+        <v>45</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>964</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E88" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A89" s="4"/>
+      <c r="B89" s="4"/>
+      <c r="C89" s="2" t="s">
+        <v>1222</v>
+      </c>
+      <c r="D89" s="4"/>
+      <c r="E89" s="4"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A90" s="4"/>
+      <c r="B90" s="4"/>
+      <c r="C90" s="2" t="s">
+        <v>823</v>
+      </c>
+      <c r="D90" s="4"/>
+      <c r="E90" s="4"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A91" s="4"/>
+      <c r="B91" s="4"/>
+      <c r="C91" s="2" t="s">
+        <v>1223</v>
+      </c>
+      <c r="D91" s="4"/>
+      <c r="E91" s="4"/>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A92" s="4"/>
+      <c r="B92" s="4"/>
+      <c r="C92" s="2" t="s">
+        <v>1224</v>
+      </c>
+      <c r="D92" s="4"/>
+      <c r="E92" s="4"/>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A93" s="4"/>
+      <c r="B93" s="4"/>
+      <c r="C93" s="2" t="s">
+        <v>960</v>
+      </c>
+      <c r="D93" s="4"/>
+      <c r="E93" s="4"/>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A94" s="4"/>
+      <c r="B94" s="4"/>
+      <c r="C94" s="2" t="s">
+        <v>959</v>
+      </c>
+      <c r="D94" s="4"/>
+      <c r="E94" s="4"/>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A95" s="4"/>
+      <c r="B95" s="4"/>
+      <c r="C95" s="2" t="s">
+        <v>1225</v>
+      </c>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A96" s="4"/>
+      <c r="B96" s="4"/>
+      <c r="C96" s="2" t="s">
+        <v>1226</v>
+      </c>
+      <c r="D96" s="4"/>
+      <c r="E96" s="4"/>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A97" s="4"/>
+      <c r="B97" s="4"/>
+      <c r="C97" s="2" t="s">
+        <v>743</v>
+      </c>
+      <c r="D97" s="4"/>
+      <c r="E97" s="4"/>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A98" s="4"/>
+      <c r="B98" s="4"/>
+      <c r="C98" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="D98" s="4"/>
+      <c r="E98" s="4"/>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A99" s="4">
+        <v>46</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>1228</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>1232</v>
+      </c>
+      <c r="E99" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A100" s="4"/>
+      <c r="B100" s="4"/>
+      <c r="C100" s="2" t="s">
+        <v>1229</v>
+      </c>
+      <c r="D100" s="4"/>
+      <c r="E100" s="4"/>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A101" s="4"/>
+      <c r="B101" s="4"/>
+      <c r="C101" s="2" t="s">
+        <v>1230</v>
+      </c>
+      <c r="D101" s="4"/>
+      <c r="E101" s="4"/>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A102" s="4"/>
+      <c r="B102" s="4"/>
+      <c r="C102" s="2" t="s">
+        <v>1231</v>
+      </c>
+      <c r="D102" s="4"/>
+      <c r="E102" s="4"/>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A103" s="2">
+        <v>47</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>1233</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>1234</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>1235</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A104" s="4">
+        <v>48</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E104" s="4" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A105" s="4"/>
+      <c r="B105" s="4"/>
+      <c r="C105" s="2" t="s">
+        <v>1096</v>
+      </c>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4"/>
+    </row>
+    <row r="106" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A106" s="4">
+        <v>49</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>1236</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>1239</v>
+      </c>
+      <c r="E106" s="4" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A107" s="4"/>
+      <c r="B107" s="4"/>
+      <c r="C107" s="2" t="s">
+        <v>1238</v>
+      </c>
+      <c r="D107" s="4"/>
+      <c r="E107" s="4"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A108" s="2">
+        <v>50</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>1240</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A109" s="4">
+        <v>51</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>777</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A110" s="4"/>
+      <c r="B110" s="4"/>
+      <c r="C110" s="2" t="s">
+        <v>1241</v>
+      </c>
+      <c r="D110" s="4"/>
+      <c r="E110" s="4"/>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A111" s="4"/>
+      <c r="B111" s="4"/>
+      <c r="C111" s="2" t="s">
+        <v>1242</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A112" s="4"/>
+      <c r="B112" s="4"/>
+      <c r="C112" s="2" t="s">
+        <v>1243</v>
+      </c>
+      <c r="D112" s="4"/>
+      <c r="E112" s="4"/>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A113" s="4"/>
+      <c r="B113" s="4"/>
+      <c r="C113" s="2" t="s">
+        <v>786</v>
+      </c>
+      <c r="D113" s="4"/>
+      <c r="E113" s="4"/>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A114" s="4"/>
+      <c r="B114" s="4"/>
+      <c r="C114" s="2" t="s">
+        <v>1244</v>
+      </c>
+      <c r="D114" s="4"/>
+      <c r="E114" s="4"/>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A115" s="4"/>
+      <c r="B115" s="4"/>
+      <c r="C115" s="2" t="s">
+        <v>1245</v>
+      </c>
+      <c r="D115" s="4"/>
+      <c r="E115" s="4"/>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A116" s="4"/>
+      <c r="B116" s="4"/>
+      <c r="C116" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="D116" s="4"/>
+      <c r="E116" s="4"/>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A117" s="4"/>
+      <c r="B117" s="4"/>
+      <c r="C117" s="2" t="s">
+        <v>781</v>
+      </c>
+      <c r="D117" s="4"/>
+      <c r="E117" s="4"/>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A118" s="4"/>
+      <c r="B118" s="4"/>
+      <c r="C118" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="D118" s="4"/>
+      <c r="E118" s="4"/>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A119" s="4"/>
+      <c r="B119" s="4"/>
+      <c r="C119" s="2" t="s">
+        <v>778</v>
+      </c>
+      <c r="D119" s="4"/>
+      <c r="E119" s="4"/>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A120" s="4"/>
+      <c r="B120" s="4"/>
+      <c r="C120" s="2" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D120" s="4"/>
+      <c r="E120" s="4"/>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A121" s="4"/>
+      <c r="B121" s="4"/>
+      <c r="C121" s="2" t="s">
+        <v>1248</v>
+      </c>
+      <c r="D121" s="4"/>
+      <c r="E121" s="4"/>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A122" s="4"/>
+      <c r="B122" s="4"/>
+      <c r="C122" s="2" t="s">
+        <v>1249</v>
+      </c>
+      <c r="D122" s="4"/>
+      <c r="E122" s="4"/>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A123" s="4"/>
+      <c r="B123" s="4"/>
+      <c r="C123" s="2" t="s">
+        <v>779</v>
+      </c>
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A124" s="2">
+        <v>52</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>1250</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>1005</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A125" s="4">
+        <v>53</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>1103</v>
+      </c>
+      <c r="D125" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E125" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A126" s="4"/>
+      <c r="B126" s="4"/>
+      <c r="C126" s="2" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D126" s="4"/>
+      <c r="E126" s="4"/>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A127" s="4">
+        <v>54</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>1168</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E127" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A128" s="4"/>
+      <c r="B128" s="4"/>
+      <c r="C128" s="2" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D128" s="4"/>
+      <c r="E128" s="4"/>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A129" s="4"/>
+      <c r="B129" s="4"/>
+      <c r="C129" s="2" t="s">
+        <v>1170</v>
+      </c>
+      <c r="D129" s="4"/>
+      <c r="E129" s="4"/>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A130" s="4"/>
+      <c r="B130" s="4"/>
+      <c r="C130" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="D130" s="4"/>
+      <c r="E130" s="4"/>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A131" s="4"/>
+      <c r="B131" s="4"/>
+      <c r="C131" s="2" t="s">
+        <v>1253</v>
+      </c>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A132" s="4"/>
+      <c r="B132" s="4"/>
+      <c r="C132" s="2" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D132" s="4"/>
+      <c r="E132" s="4"/>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A133" s="4"/>
+      <c r="B133" s="4"/>
+      <c r="C133" s="2" t="s">
+        <v>1255</v>
+      </c>
+      <c r="D133" s="4"/>
+      <c r="E133" s="4"/>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A134" s="4"/>
+      <c r="B134" s="4"/>
+      <c r="C134" s="2" t="s">
+        <v>1256</v>
+      </c>
+      <c r="D134" s="4"/>
+      <c r="E134" s="4"/>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A135" s="2">
+        <v>55</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>1257</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>1258</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="88">
+    <mergeCell ref="D125:D126"/>
+    <mergeCell ref="E125:E126"/>
+    <mergeCell ref="A127:A134"/>
+    <mergeCell ref="B127:B134"/>
+    <mergeCell ref="D127:D134"/>
+    <mergeCell ref="E127:E134"/>
+    <mergeCell ref="D106:D107"/>
+    <mergeCell ref="E106:E107"/>
+    <mergeCell ref="A109:A123"/>
+    <mergeCell ref="B109:B123"/>
+    <mergeCell ref="D109:D123"/>
+    <mergeCell ref="E109:E123"/>
+    <mergeCell ref="D99:D102"/>
+    <mergeCell ref="E99:E102"/>
+    <mergeCell ref="A104:A105"/>
+    <mergeCell ref="B104:B105"/>
+    <mergeCell ref="D104:D105"/>
+    <mergeCell ref="E104:E105"/>
+    <mergeCell ref="D78:D83"/>
+    <mergeCell ref="E78:E83"/>
+    <mergeCell ref="A88:A98"/>
+    <mergeCell ref="B88:B98"/>
+    <mergeCell ref="D88:D98"/>
+    <mergeCell ref="E88:E98"/>
+    <mergeCell ref="D72:D73"/>
+    <mergeCell ref="E72:E73"/>
+    <mergeCell ref="A74:A76"/>
+    <mergeCell ref="B74:B76"/>
+    <mergeCell ref="D74:D76"/>
+    <mergeCell ref="E74:E76"/>
+    <mergeCell ref="D61:D65"/>
+    <mergeCell ref="E61:E65"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="E68:E69"/>
+    <mergeCell ref="D50:D52"/>
+    <mergeCell ref="E50:E52"/>
+    <mergeCell ref="A55:A59"/>
+    <mergeCell ref="B55:B59"/>
+    <mergeCell ref="D55:D59"/>
+    <mergeCell ref="E55:E59"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="A44:A47"/>
+    <mergeCell ref="B44:B47"/>
+    <mergeCell ref="D44:D47"/>
+    <mergeCell ref="E44:E47"/>
+    <mergeCell ref="D30:D32"/>
+    <mergeCell ref="E30:E32"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="D33:D36"/>
+    <mergeCell ref="E33:E36"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="A25:A28"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="D25:D28"/>
+    <mergeCell ref="E25:E28"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="A11:A19"/>
+    <mergeCell ref="B11:B19"/>
+    <mergeCell ref="D11:D19"/>
+    <mergeCell ref="E11:E19"/>
+    <mergeCell ref="A125:A126"/>
+    <mergeCell ref="B125:B126"/>
+    <mergeCell ref="A106:A107"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="A99:A102"/>
+    <mergeCell ref="B99:B102"/>
+    <mergeCell ref="A78:A83"/>
+    <mergeCell ref="B78:B83"/>
+    <mergeCell ref="A72:A73"/>
+    <mergeCell ref="B72:B73"/>
+    <mergeCell ref="A61:A65"/>
+    <mergeCell ref="B61:B65"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="B50:B52"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add participant analysis for IROS 2024
</commit_message>
<xml_diff>
--- a/Registration.xlsx
+++ b/Registration.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tsamak\Workspace\AutoDRIVE-RoboRacer-Sim-Racing-Participation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3627A9-44AA-461C-A9B6-212EB97ECB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D7CB4F3-39F3-4BD5-B7A2-AD8952BF4608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="5" xr2:uid="{5D9342A3-8B90-4963-824C-8C358DE1DB7F}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1987" uniqueCount="1259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1980" uniqueCount="1259">
   <si>
     <t>SAGOL</t>
   </si>
@@ -6197,37 +6197,85 @@
     </row>
   </sheetData>
   <mergeCells count="124">
-    <mergeCell ref="D27:D31"/>
-    <mergeCell ref="D21:D24"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="D6:D14"/>
-    <mergeCell ref="D81:D82"/>
-    <mergeCell ref="D77:D78"/>
-    <mergeCell ref="D71:D76"/>
-    <mergeCell ref="D67:D70"/>
-    <mergeCell ref="D59:D65"/>
-    <mergeCell ref="D55:D56"/>
-    <mergeCell ref="D50:D54"/>
-    <mergeCell ref="D35:D46"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="D103:D105"/>
-    <mergeCell ref="D99:D102"/>
-    <mergeCell ref="D111:D116"/>
-    <mergeCell ref="D108:D110"/>
-    <mergeCell ref="D106:D107"/>
-    <mergeCell ref="D117:D118"/>
-    <mergeCell ref="D95:D97"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="D84:D89"/>
-    <mergeCell ref="D154:D158"/>
-    <mergeCell ref="D159:D161"/>
-    <mergeCell ref="D124:D131"/>
-    <mergeCell ref="D122:D123"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="D135:D137"/>
-    <mergeCell ref="D132:D134"/>
-    <mergeCell ref="D149:D152"/>
-    <mergeCell ref="D142:D148"/>
+    <mergeCell ref="E159:E161"/>
+    <mergeCell ref="E135:E137"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="E142:E148"/>
+    <mergeCell ref="E149:E152"/>
+    <mergeCell ref="E154:E158"/>
+    <mergeCell ref="E111:E116"/>
+    <mergeCell ref="E117:E118"/>
+    <mergeCell ref="E122:E123"/>
+    <mergeCell ref="E124:E131"/>
+    <mergeCell ref="E132:E134"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="E99:E102"/>
+    <mergeCell ref="E103:E105"/>
+    <mergeCell ref="E106:E107"/>
+    <mergeCell ref="E108:E110"/>
+    <mergeCell ref="E71:E76"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="E84:E89"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="E35:E46"/>
+    <mergeCell ref="E50:E54"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E59:E65"/>
+    <mergeCell ref="E67:E70"/>
+    <mergeCell ref="E6:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E21:E24"/>
+    <mergeCell ref="E27:E31"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="A27:A31"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A35:A46"/>
+    <mergeCell ref="B35:B46"/>
+    <mergeCell ref="A6:A14"/>
+    <mergeCell ref="B6:B14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A71:A76"/>
+    <mergeCell ref="B71:B76"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="A50:A54"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="A59:A65"/>
+    <mergeCell ref="B59:B65"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="A99:A102"/>
+    <mergeCell ref="B99:B102"/>
+    <mergeCell ref="A103:A105"/>
+    <mergeCell ref="B103:B105"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="A84:A89"/>
+    <mergeCell ref="B84:B89"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A117:A118"/>
+    <mergeCell ref="B117:B118"/>
+    <mergeCell ref="A122:A123"/>
+    <mergeCell ref="B122:B123"/>
+    <mergeCell ref="A124:A131"/>
+    <mergeCell ref="B124:B131"/>
+    <mergeCell ref="A106:A107"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="A108:A110"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="A111:A116"/>
+    <mergeCell ref="B111:B116"/>
     <mergeCell ref="A142:A148"/>
     <mergeCell ref="B142:B148"/>
     <mergeCell ref="A159:A161"/>
@@ -6242,85 +6290,37 @@
     <mergeCell ref="B135:B137"/>
     <mergeCell ref="A138:A141"/>
     <mergeCell ref="B138:B141"/>
-    <mergeCell ref="A117:A118"/>
-    <mergeCell ref="B117:B118"/>
-    <mergeCell ref="A122:A123"/>
-    <mergeCell ref="B122:B123"/>
-    <mergeCell ref="A124:A131"/>
-    <mergeCell ref="B124:B131"/>
-    <mergeCell ref="A106:A107"/>
-    <mergeCell ref="B106:B107"/>
-    <mergeCell ref="A108:A110"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="A111:A116"/>
-    <mergeCell ref="B111:B116"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="A99:A102"/>
-    <mergeCell ref="B99:B102"/>
-    <mergeCell ref="A103:A105"/>
-    <mergeCell ref="B103:B105"/>
-    <mergeCell ref="A81:A82"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="A84:A89"/>
-    <mergeCell ref="B84:B89"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A71:A76"/>
-    <mergeCell ref="B71:B76"/>
-    <mergeCell ref="A77:A78"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="A50:A54"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="A59:A65"/>
-    <mergeCell ref="B59:B65"/>
-    <mergeCell ref="A27:A31"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A35:A46"/>
-    <mergeCell ref="B35:B46"/>
-    <mergeCell ref="A6:A14"/>
-    <mergeCell ref="B6:B14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="B21:B24"/>
-    <mergeCell ref="E35:E46"/>
-    <mergeCell ref="E50:E54"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E59:E65"/>
-    <mergeCell ref="E67:E70"/>
-    <mergeCell ref="E6:E14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E21:E24"/>
-    <mergeCell ref="E27:E31"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="E99:E102"/>
-    <mergeCell ref="E103:E105"/>
-    <mergeCell ref="E106:E107"/>
-    <mergeCell ref="E108:E110"/>
-    <mergeCell ref="E71:E76"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="E84:E89"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="E159:E161"/>
-    <mergeCell ref="E135:E137"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="E142:E148"/>
-    <mergeCell ref="E149:E152"/>
-    <mergeCell ref="E154:E158"/>
-    <mergeCell ref="E111:E116"/>
-    <mergeCell ref="E117:E118"/>
-    <mergeCell ref="E122:E123"/>
-    <mergeCell ref="E124:E131"/>
-    <mergeCell ref="E132:E134"/>
+    <mergeCell ref="D154:D158"/>
+    <mergeCell ref="D159:D161"/>
+    <mergeCell ref="D124:D131"/>
+    <mergeCell ref="D122:D123"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="D135:D137"/>
+    <mergeCell ref="D132:D134"/>
+    <mergeCell ref="D149:D152"/>
+    <mergeCell ref="D142:D148"/>
+    <mergeCell ref="D103:D105"/>
+    <mergeCell ref="D99:D102"/>
+    <mergeCell ref="D111:D116"/>
+    <mergeCell ref="D108:D110"/>
+    <mergeCell ref="D106:D107"/>
+    <mergeCell ref="D117:D118"/>
+    <mergeCell ref="D95:D97"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="D84:D89"/>
+    <mergeCell ref="D27:D31"/>
+    <mergeCell ref="D21:D24"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="D6:D14"/>
+    <mergeCell ref="D81:D82"/>
+    <mergeCell ref="D77:D78"/>
+    <mergeCell ref="D71:D76"/>
+    <mergeCell ref="D67:D70"/>
+    <mergeCell ref="D59:D65"/>
+    <mergeCell ref="D55:D56"/>
+    <mergeCell ref="D50:D54"/>
+    <mergeCell ref="D35:D46"/>
+    <mergeCell ref="D33:D34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -8292,85 +8292,44 @@
     </row>
   </sheetData>
   <mergeCells count="144">
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="D76:D78"/>
-    <mergeCell ref="D71:D73"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="D92:D94"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="A46:A51"/>
-    <mergeCell ref="B46:B51"/>
-    <mergeCell ref="D46:D51"/>
-    <mergeCell ref="A52:A53"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="B62:B64"/>
-    <mergeCell ref="A152:A156"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="A150:A151"/>
-    <mergeCell ref="A123:A129"/>
-    <mergeCell ref="A130:A141"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A75:A78"/>
-    <mergeCell ref="A66:A67"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="A170:A171"/>
-    <mergeCell ref="B170:B171"/>
-    <mergeCell ref="D170:D171"/>
-    <mergeCell ref="A160:A164"/>
-    <mergeCell ref="B160:B164"/>
-    <mergeCell ref="D160:D164"/>
-    <mergeCell ref="A157:A159"/>
-    <mergeCell ref="B157:B159"/>
-    <mergeCell ref="D157:D159"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="B75:B78"/>
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="D80:D82"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="D84:D85"/>
-    <mergeCell ref="B112:B116"/>
-    <mergeCell ref="D112:D116"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="D95:D97"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B86:B91"/>
-    <mergeCell ref="D86:D91"/>
-    <mergeCell ref="A112:A116"/>
-    <mergeCell ref="A86:A91"/>
-    <mergeCell ref="A84:A85"/>
-    <mergeCell ref="A102:A111"/>
-    <mergeCell ref="A117:A122"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="D150:D151"/>
-    <mergeCell ref="B152:B156"/>
-    <mergeCell ref="D152:D156"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="B117:B122"/>
-    <mergeCell ref="D117:D122"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="B102:B111"/>
-    <mergeCell ref="D102:D111"/>
-    <mergeCell ref="B123:B129"/>
-    <mergeCell ref="D123:D129"/>
-    <mergeCell ref="B130:B141"/>
-    <mergeCell ref="D130:D141"/>
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="E170:E171"/>
+    <mergeCell ref="E102:E111"/>
+    <mergeCell ref="E112:E116"/>
+    <mergeCell ref="E117:E122"/>
+    <mergeCell ref="E123:E129"/>
+    <mergeCell ref="E130:E141"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="E150:E151"/>
+    <mergeCell ref="E152:E156"/>
+    <mergeCell ref="E75:E78"/>
+    <mergeCell ref="E80:E82"/>
+    <mergeCell ref="E84:E85"/>
+    <mergeCell ref="E86:E91"/>
+    <mergeCell ref="E92:E94"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="E157:E159"/>
+    <mergeCell ref="E160:E164"/>
+    <mergeCell ref="E38:E45"/>
+    <mergeCell ref="E46:E51"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="E62:E64"/>
+    <mergeCell ref="E66:E67"/>
+    <mergeCell ref="B8:B15"/>
+    <mergeCell ref="D8:D15"/>
+    <mergeCell ref="E68:E69"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="E8:E15"/>
+    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="E26:E30"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="E33:E37"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="D2:D3"/>
@@ -8395,47 +8354,88 @@
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="D16:D19"/>
     <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="D150:D151"/>
+    <mergeCell ref="B152:B156"/>
+    <mergeCell ref="D152:D156"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="B117:B122"/>
+    <mergeCell ref="D117:D122"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="B102:B111"/>
+    <mergeCell ref="D102:D111"/>
+    <mergeCell ref="B123:B129"/>
+    <mergeCell ref="D123:D129"/>
+    <mergeCell ref="B130:B141"/>
+    <mergeCell ref="D130:D141"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="B75:B78"/>
+    <mergeCell ref="B80:B82"/>
+    <mergeCell ref="D80:D82"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="D84:D85"/>
+    <mergeCell ref="B112:B116"/>
+    <mergeCell ref="D112:D116"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="D95:D97"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B86:B91"/>
+    <mergeCell ref="D86:D91"/>
+    <mergeCell ref="A112:A116"/>
+    <mergeCell ref="A86:A91"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="A102:A111"/>
+    <mergeCell ref="A117:A122"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="A170:A171"/>
+    <mergeCell ref="B170:B171"/>
+    <mergeCell ref="D170:D171"/>
+    <mergeCell ref="A160:A164"/>
+    <mergeCell ref="B160:B164"/>
+    <mergeCell ref="D160:D164"/>
+    <mergeCell ref="A157:A159"/>
+    <mergeCell ref="B157:B159"/>
+    <mergeCell ref="D157:D159"/>
+    <mergeCell ref="A152:A156"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="A150:A151"/>
+    <mergeCell ref="A123:A129"/>
+    <mergeCell ref="A130:A141"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="A75:A78"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="D76:D78"/>
+    <mergeCell ref="D71:D73"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="D92:D94"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="A46:A51"/>
+    <mergeCell ref="B46:B51"/>
+    <mergeCell ref="D46:D51"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="B62:B64"/>
     <mergeCell ref="D62:D64"/>
     <mergeCell ref="B66:B67"/>
     <mergeCell ref="D66:D67"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E4:E7"/>
-    <mergeCell ref="E8:E15"/>
-    <mergeCell ref="E16:E19"/>
-    <mergeCell ref="E21:E23"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="E26:E30"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="E33:E37"/>
-    <mergeCell ref="E38:E45"/>
-    <mergeCell ref="E46:E51"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="E62:E64"/>
-    <mergeCell ref="E66:E67"/>
-    <mergeCell ref="B8:B15"/>
-    <mergeCell ref="D8:D15"/>
-    <mergeCell ref="E68:E69"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="E75:E78"/>
-    <mergeCell ref="E80:E82"/>
-    <mergeCell ref="E84:E85"/>
-    <mergeCell ref="E86:E91"/>
-    <mergeCell ref="E92:E94"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="E157:E159"/>
-    <mergeCell ref="E160:E164"/>
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="E170:E171"/>
-    <mergeCell ref="E102:E111"/>
-    <mergeCell ref="E112:E116"/>
-    <mergeCell ref="E117:E122"/>
-    <mergeCell ref="E123:E129"/>
-    <mergeCell ref="E130:E141"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="E150:E151"/>
-    <mergeCell ref="E152:E156"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10270,29 +10270,90 @@
     </row>
   </sheetData>
   <mergeCells count="132">
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="D48:D50"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="A129:A130"/>
-    <mergeCell ref="B129:B130"/>
-    <mergeCell ref="D129:D130"/>
-    <mergeCell ref="E129:E130"/>
-    <mergeCell ref="A87:A89"/>
-    <mergeCell ref="B87:B89"/>
-    <mergeCell ref="D87:D89"/>
-    <mergeCell ref="A92:A97"/>
-    <mergeCell ref="B92:B97"/>
-    <mergeCell ref="D92:D97"/>
-    <mergeCell ref="E92:E97"/>
-    <mergeCell ref="A99:A109"/>
-    <mergeCell ref="B99:B109"/>
-    <mergeCell ref="D99:D109"/>
-    <mergeCell ref="E99:E109"/>
-    <mergeCell ref="A76:A80"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="D76:D80"/>
-    <mergeCell ref="E76:E80"/>
-    <mergeCell ref="A65:A71"/>
+    <mergeCell ref="A145:A147"/>
+    <mergeCell ref="B145:B147"/>
+    <mergeCell ref="D145:D147"/>
+    <mergeCell ref="E145:E147"/>
+    <mergeCell ref="A149:A150"/>
+    <mergeCell ref="B149:B150"/>
+    <mergeCell ref="D149:D150"/>
+    <mergeCell ref="E149:E150"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="D131:D133"/>
+    <mergeCell ref="E131:E133"/>
+    <mergeCell ref="A135:A138"/>
+    <mergeCell ref="B135:B138"/>
+    <mergeCell ref="D135:D138"/>
+    <mergeCell ref="E135:E138"/>
+    <mergeCell ref="A139:A141"/>
+    <mergeCell ref="B139:B141"/>
+    <mergeCell ref="D139:D141"/>
+    <mergeCell ref="E139:E141"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="D114:D117"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="A118:A127"/>
+    <mergeCell ref="B118:B127"/>
+    <mergeCell ref="D118:D127"/>
+    <mergeCell ref="E118:E127"/>
+    <mergeCell ref="A81:A85"/>
+    <mergeCell ref="B81:B85"/>
+    <mergeCell ref="D81:D85"/>
+    <mergeCell ref="E81:E85"/>
+    <mergeCell ref="E87:E89"/>
+    <mergeCell ref="A90:A91"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="D90:D91"/>
+    <mergeCell ref="E90:E91"/>
+    <mergeCell ref="D1:D4"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E1:E4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="D65:D71"/>
+    <mergeCell ref="D73:D75"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="E57:E59"/>
+    <mergeCell ref="A60:A64"/>
+    <mergeCell ref="B60:B64"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="D51:D53"/>
+    <mergeCell ref="E51:E53"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="E42:E46"/>
+    <mergeCell ref="E73:E75"/>
+    <mergeCell ref="A73:A75"/>
+    <mergeCell ref="B73:B75"/>
+    <mergeCell ref="E65:E71"/>
+    <mergeCell ref="A48:A50"/>
     <mergeCell ref="D29:D31"/>
     <mergeCell ref="E29:E31"/>
     <mergeCell ref="A20:A22"/>
@@ -10317,91 +10378,30 @@
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="B29:B31"/>
     <mergeCell ref="B1:B4"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="D48:D50"/>
+    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="A129:A130"/>
+    <mergeCell ref="B129:B130"/>
+    <mergeCell ref="D129:D130"/>
+    <mergeCell ref="E129:E130"/>
+    <mergeCell ref="A87:A89"/>
+    <mergeCell ref="B87:B89"/>
+    <mergeCell ref="D87:D89"/>
+    <mergeCell ref="A92:A97"/>
+    <mergeCell ref="B92:B97"/>
+    <mergeCell ref="D92:D97"/>
+    <mergeCell ref="E92:E97"/>
+    <mergeCell ref="A99:A109"/>
+    <mergeCell ref="B99:B109"/>
+    <mergeCell ref="D99:D109"/>
+    <mergeCell ref="E99:E109"/>
+    <mergeCell ref="A76:A80"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="D76:D80"/>
+    <mergeCell ref="E76:E80"/>
+    <mergeCell ref="A65:A71"/>
     <mergeCell ref="B65:B71"/>
-    <mergeCell ref="D65:D71"/>
-    <mergeCell ref="D73:D75"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="E57:E59"/>
-    <mergeCell ref="A60:A64"/>
-    <mergeCell ref="B60:B64"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="B51:B53"/>
-    <mergeCell ref="D51:D53"/>
-    <mergeCell ref="E51:E53"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="E42:E46"/>
-    <mergeCell ref="E73:E75"/>
-    <mergeCell ref="A73:A75"/>
-    <mergeCell ref="B73:B75"/>
-    <mergeCell ref="E65:E71"/>
-    <mergeCell ref="A48:A50"/>
-    <mergeCell ref="D1:D4"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E1:E4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="A81:A85"/>
-    <mergeCell ref="B81:B85"/>
-    <mergeCell ref="D81:D85"/>
-    <mergeCell ref="E81:E85"/>
-    <mergeCell ref="E87:E89"/>
-    <mergeCell ref="A90:A91"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="D90:D91"/>
-    <mergeCell ref="E90:E91"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="D114:D117"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="A118:A127"/>
-    <mergeCell ref="B118:B127"/>
-    <mergeCell ref="D118:D127"/>
-    <mergeCell ref="E118:E127"/>
-    <mergeCell ref="A145:A147"/>
-    <mergeCell ref="B145:B147"/>
-    <mergeCell ref="D145:D147"/>
-    <mergeCell ref="E145:E147"/>
-    <mergeCell ref="A149:A150"/>
-    <mergeCell ref="B149:B150"/>
-    <mergeCell ref="D149:D150"/>
-    <mergeCell ref="E149:E150"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="D131:D133"/>
-    <mergeCell ref="E131:E133"/>
-    <mergeCell ref="A135:A138"/>
-    <mergeCell ref="B135:B138"/>
-    <mergeCell ref="D135:D138"/>
-    <mergeCell ref="E135:E138"/>
-    <mergeCell ref="A139:A141"/>
-    <mergeCell ref="B139:B141"/>
-    <mergeCell ref="D139:D141"/>
-    <mergeCell ref="E139:E141"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -12200,57 +12200,31 @@
     </row>
   </sheetData>
   <mergeCells count="92">
-    <mergeCell ref="A90:A95"/>
-    <mergeCell ref="A96:A100"/>
-    <mergeCell ref="A57:A61"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A42:A47"/>
-    <mergeCell ref="A83:A89"/>
-    <mergeCell ref="A154:A156"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="D154:D156"/>
-    <mergeCell ref="E154:E156"/>
-    <mergeCell ref="A157:A158"/>
-    <mergeCell ref="B157:B158"/>
-    <mergeCell ref="D157:D158"/>
-    <mergeCell ref="E157:E158"/>
-    <mergeCell ref="D90:D95"/>
-    <mergeCell ref="E90:E95"/>
-    <mergeCell ref="B96:B100"/>
-    <mergeCell ref="D96:D100"/>
-    <mergeCell ref="E96:E100"/>
-    <mergeCell ref="B90:B95"/>
-    <mergeCell ref="D49:D54"/>
-    <mergeCell ref="E49:E54"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="D57:D61"/>
-    <mergeCell ref="E57:E61"/>
-    <mergeCell ref="B49:B54"/>
-    <mergeCell ref="D39:D41"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="B42:B47"/>
-    <mergeCell ref="D42:D47"/>
-    <mergeCell ref="E42:E47"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="A15:A24"/>
-    <mergeCell ref="B15:B24"/>
-    <mergeCell ref="D15:D24"/>
-    <mergeCell ref="E15:E24"/>
-    <mergeCell ref="D28:D31"/>
-    <mergeCell ref="E28:E31"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="D5:D8"/>
-    <mergeCell ref="E5:E8"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="B9:B13"/>
-    <mergeCell ref="D9:D13"/>
-    <mergeCell ref="E9:E13"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="D36:D38"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="B32:B35"/>
+    <mergeCell ref="D32:D35"/>
+    <mergeCell ref="E32:E35"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D83:D89"/>
+    <mergeCell ref="E83:E89"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="B62:B67"/>
+    <mergeCell ref="D62:D67"/>
+    <mergeCell ref="E62:E67"/>
+    <mergeCell ref="A69:A72"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="D69:D72"/>
+    <mergeCell ref="E69:E72"/>
+    <mergeCell ref="A73:A82"/>
+    <mergeCell ref="B73:B82"/>
+    <mergeCell ref="D73:D82"/>
+    <mergeCell ref="E73:E82"/>
     <mergeCell ref="A129:A151"/>
     <mergeCell ref="B129:B151"/>
     <mergeCell ref="D129:D151"/>
@@ -12267,31 +12241,57 @@
     <mergeCell ref="B126:B128"/>
     <mergeCell ref="D126:D128"/>
     <mergeCell ref="E126:E128"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D83:D89"/>
-    <mergeCell ref="E83:E89"/>
-    <mergeCell ref="A62:A67"/>
-    <mergeCell ref="B62:B67"/>
-    <mergeCell ref="D62:D67"/>
-    <mergeCell ref="E62:E67"/>
-    <mergeCell ref="A69:A72"/>
-    <mergeCell ref="B69:B72"/>
-    <mergeCell ref="D69:D72"/>
-    <mergeCell ref="E69:E72"/>
-    <mergeCell ref="A73:A82"/>
-    <mergeCell ref="B73:B82"/>
-    <mergeCell ref="D73:D82"/>
-    <mergeCell ref="E73:E82"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="D36:D38"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="B28:B31"/>
-    <mergeCell ref="A32:A35"/>
-    <mergeCell ref="B32:B35"/>
-    <mergeCell ref="D32:D35"/>
-    <mergeCell ref="E32:E35"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="E5:E8"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="B9:B13"/>
+    <mergeCell ref="D9:D13"/>
+    <mergeCell ref="E9:E13"/>
+    <mergeCell ref="A15:A24"/>
+    <mergeCell ref="B15:B24"/>
+    <mergeCell ref="D15:D24"/>
+    <mergeCell ref="E15:E24"/>
+    <mergeCell ref="D28:D31"/>
+    <mergeCell ref="E28:E31"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="B42:B47"/>
+    <mergeCell ref="D42:D47"/>
+    <mergeCell ref="E42:E47"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="D49:D54"/>
+    <mergeCell ref="E49:E54"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="D57:D61"/>
+    <mergeCell ref="E57:E61"/>
+    <mergeCell ref="B49:B54"/>
+    <mergeCell ref="D90:D95"/>
+    <mergeCell ref="E90:E95"/>
+    <mergeCell ref="B96:B100"/>
+    <mergeCell ref="D96:D100"/>
+    <mergeCell ref="E96:E100"/>
+    <mergeCell ref="B90:B95"/>
+    <mergeCell ref="A154:A156"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="D154:D156"/>
+    <mergeCell ref="E154:E156"/>
+    <mergeCell ref="A157:A158"/>
+    <mergeCell ref="B157:B158"/>
+    <mergeCell ref="D157:D158"/>
+    <mergeCell ref="E157:E158"/>
+    <mergeCell ref="A90:A95"/>
+    <mergeCell ref="A96:A100"/>
+    <mergeCell ref="A57:A61"/>
+    <mergeCell ref="A49:A54"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="A42:A47"/>
+    <mergeCell ref="A83:A89"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14704,6 +14704,126 @@
     </row>
   </sheetData>
   <mergeCells count="144">
+    <mergeCell ref="A182:A183"/>
+    <mergeCell ref="B182:B183"/>
+    <mergeCell ref="D182:D183"/>
+    <mergeCell ref="E182:E183"/>
+    <mergeCell ref="A185:A191"/>
+    <mergeCell ref="B185:B191"/>
+    <mergeCell ref="D185:D191"/>
+    <mergeCell ref="E185:E191"/>
+    <mergeCell ref="A176:A177"/>
+    <mergeCell ref="B176:B177"/>
+    <mergeCell ref="D176:D177"/>
+    <mergeCell ref="E176:E177"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="A168:A170"/>
+    <mergeCell ref="B168:B170"/>
+    <mergeCell ref="D168:D170"/>
+    <mergeCell ref="E168:E170"/>
+    <mergeCell ref="A171:A175"/>
+    <mergeCell ref="B171:B175"/>
+    <mergeCell ref="D171:D175"/>
+    <mergeCell ref="E171:E175"/>
+    <mergeCell ref="A154:A161"/>
+    <mergeCell ref="B154:B161"/>
+    <mergeCell ref="D154:D161"/>
+    <mergeCell ref="E154:E161"/>
+    <mergeCell ref="A163:A165"/>
+    <mergeCell ref="B163:B165"/>
+    <mergeCell ref="D163:D165"/>
+    <mergeCell ref="E163:E165"/>
+    <mergeCell ref="A145:A149"/>
+    <mergeCell ref="B145:B149"/>
+    <mergeCell ref="D145:D149"/>
+    <mergeCell ref="E145:E149"/>
+    <mergeCell ref="A151:A153"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="D151:D153"/>
+    <mergeCell ref="E151:E153"/>
+    <mergeCell ref="D139:D141"/>
+    <mergeCell ref="E139:E141"/>
+    <mergeCell ref="A142:A143"/>
+    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="D142:D143"/>
+    <mergeCell ref="E142:E143"/>
+    <mergeCell ref="D125:D127"/>
+    <mergeCell ref="E125:E127"/>
+    <mergeCell ref="A132:A133"/>
+    <mergeCell ref="B132:B133"/>
+    <mergeCell ref="D132:D133"/>
+    <mergeCell ref="E132:E133"/>
+    <mergeCell ref="A111:A112"/>
+    <mergeCell ref="B111:B112"/>
+    <mergeCell ref="D111:D112"/>
+    <mergeCell ref="E111:E112"/>
+    <mergeCell ref="A115:A123"/>
+    <mergeCell ref="B115:B123"/>
+    <mergeCell ref="D115:D123"/>
+    <mergeCell ref="E115:E123"/>
+    <mergeCell ref="A103:A106"/>
+    <mergeCell ref="B103:B106"/>
+    <mergeCell ref="D103:D106"/>
+    <mergeCell ref="E103:E106"/>
+    <mergeCell ref="A107:A110"/>
+    <mergeCell ref="B107:B110"/>
+    <mergeCell ref="D107:D110"/>
+    <mergeCell ref="E107:E110"/>
+    <mergeCell ref="D97:D99"/>
+    <mergeCell ref="E97:E99"/>
+    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="B101:B102"/>
+    <mergeCell ref="D101:D102"/>
+    <mergeCell ref="E101:E102"/>
+    <mergeCell ref="D81:D87"/>
+    <mergeCell ref="E81:E87"/>
+    <mergeCell ref="A90:A96"/>
+    <mergeCell ref="B90:B96"/>
+    <mergeCell ref="D90:D96"/>
+    <mergeCell ref="E90:E96"/>
+    <mergeCell ref="D68:D77"/>
+    <mergeCell ref="E68:E77"/>
+    <mergeCell ref="A78:A79"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="D78:D79"/>
+    <mergeCell ref="E78:E79"/>
+    <mergeCell ref="A59:A67"/>
+    <mergeCell ref="B59:B67"/>
+    <mergeCell ref="D59:D67"/>
+    <mergeCell ref="E59:E67"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="D4:D8"/>
+    <mergeCell ref="E4:E8"/>
+    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="A139:A141"/>
+    <mergeCell ref="B139:B141"/>
+    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="B125:B127"/>
+    <mergeCell ref="A97:A99"/>
+    <mergeCell ref="B97:B99"/>
+    <mergeCell ref="A81:A87"/>
+    <mergeCell ref="B81:B87"/>
+    <mergeCell ref="A68:A77"/>
+    <mergeCell ref="B68:B77"/>
+    <mergeCell ref="A53:A58"/>
+    <mergeCell ref="B53:B58"/>
+    <mergeCell ref="A46:A48"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="A29:A35"/>
+    <mergeCell ref="B29:B35"/>
+    <mergeCell ref="A16:A25"/>
+    <mergeCell ref="B16:B25"/>
     <mergeCell ref="D10:D14"/>
     <mergeCell ref="E10:E14"/>
     <mergeCell ref="A195:A198"/>
@@ -14728,126 +14848,6 @@
     <mergeCell ref="E26:E28"/>
     <mergeCell ref="D53:D58"/>
     <mergeCell ref="E53:E58"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="B4:B8"/>
-    <mergeCell ref="D4:D8"/>
-    <mergeCell ref="E4:E8"/>
-    <mergeCell ref="A10:A14"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="A139:A141"/>
-    <mergeCell ref="B139:B141"/>
-    <mergeCell ref="A125:A127"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="A97:A99"/>
-    <mergeCell ref="B97:B99"/>
-    <mergeCell ref="A81:A87"/>
-    <mergeCell ref="B81:B87"/>
-    <mergeCell ref="A68:A77"/>
-    <mergeCell ref="B68:B77"/>
-    <mergeCell ref="A53:A58"/>
-    <mergeCell ref="B53:B58"/>
-    <mergeCell ref="A46:A48"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="A29:A35"/>
-    <mergeCell ref="B29:B35"/>
-    <mergeCell ref="A16:A25"/>
-    <mergeCell ref="B16:B25"/>
-    <mergeCell ref="A59:A67"/>
-    <mergeCell ref="B59:B67"/>
-    <mergeCell ref="D59:D67"/>
-    <mergeCell ref="E59:E67"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="D81:D87"/>
-    <mergeCell ref="E81:E87"/>
-    <mergeCell ref="A90:A96"/>
-    <mergeCell ref="B90:B96"/>
-    <mergeCell ref="D90:D96"/>
-    <mergeCell ref="E90:E96"/>
-    <mergeCell ref="D68:D77"/>
-    <mergeCell ref="E68:E77"/>
-    <mergeCell ref="A78:A79"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="D78:D79"/>
-    <mergeCell ref="E78:E79"/>
-    <mergeCell ref="A103:A106"/>
-    <mergeCell ref="B103:B106"/>
-    <mergeCell ref="D103:D106"/>
-    <mergeCell ref="E103:E106"/>
-    <mergeCell ref="A107:A110"/>
-    <mergeCell ref="B107:B110"/>
-    <mergeCell ref="D107:D110"/>
-    <mergeCell ref="E107:E110"/>
-    <mergeCell ref="D97:D99"/>
-    <mergeCell ref="E97:E99"/>
-    <mergeCell ref="A101:A102"/>
-    <mergeCell ref="B101:B102"/>
-    <mergeCell ref="D101:D102"/>
-    <mergeCell ref="E101:E102"/>
-    <mergeCell ref="D125:D127"/>
-    <mergeCell ref="E125:E127"/>
-    <mergeCell ref="A132:A133"/>
-    <mergeCell ref="B132:B133"/>
-    <mergeCell ref="D132:D133"/>
-    <mergeCell ref="E132:E133"/>
-    <mergeCell ref="A111:A112"/>
-    <mergeCell ref="B111:B112"/>
-    <mergeCell ref="D111:D112"/>
-    <mergeCell ref="E111:E112"/>
-    <mergeCell ref="A115:A123"/>
-    <mergeCell ref="B115:B123"/>
-    <mergeCell ref="D115:D123"/>
-    <mergeCell ref="E115:E123"/>
-    <mergeCell ref="A145:A149"/>
-    <mergeCell ref="B145:B149"/>
-    <mergeCell ref="D145:D149"/>
-    <mergeCell ref="E145:E149"/>
-    <mergeCell ref="A151:A153"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="D151:D153"/>
-    <mergeCell ref="E151:E153"/>
-    <mergeCell ref="D139:D141"/>
-    <mergeCell ref="E139:E141"/>
-    <mergeCell ref="A142:A143"/>
-    <mergeCell ref="B142:B143"/>
-    <mergeCell ref="D142:D143"/>
-    <mergeCell ref="E142:E143"/>
-    <mergeCell ref="A168:A170"/>
-    <mergeCell ref="B168:B170"/>
-    <mergeCell ref="D168:D170"/>
-    <mergeCell ref="E168:E170"/>
-    <mergeCell ref="A171:A175"/>
-    <mergeCell ref="B171:B175"/>
-    <mergeCell ref="D171:D175"/>
-    <mergeCell ref="E171:E175"/>
-    <mergeCell ref="A154:A161"/>
-    <mergeCell ref="B154:B161"/>
-    <mergeCell ref="D154:D161"/>
-    <mergeCell ref="E154:E161"/>
-    <mergeCell ref="A163:A165"/>
-    <mergeCell ref="B163:B165"/>
-    <mergeCell ref="D163:D165"/>
-    <mergeCell ref="E163:E165"/>
-    <mergeCell ref="A182:A183"/>
-    <mergeCell ref="B182:B183"/>
-    <mergeCell ref="D182:D183"/>
-    <mergeCell ref="E182:E183"/>
-    <mergeCell ref="A185:A191"/>
-    <mergeCell ref="B185:B191"/>
-    <mergeCell ref="D185:D191"/>
-    <mergeCell ref="E185:E191"/>
-    <mergeCell ref="A176:A177"/>
-    <mergeCell ref="B176:B177"/>
-    <mergeCell ref="D176:D177"/>
-    <mergeCell ref="E176:E177"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="E178:E181"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14855,7 +14855,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC4CFA97-D216-4292-8965-1641300B15B3}">
-  <dimension ref="A1:E135"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.08984375" style="3" bestFit="1" customWidth="1"/>
@@ -15430,75 +15430,83 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" s="4">
+      <c r="A44" s="2">
         <v>23</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>1167</v>
+      <c r="B44" s="2" t="s">
+        <v>1035</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>1168</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="E44" s="4" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" s="2">
+        <v>24</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>1173</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="2" t="s">
-        <v>1169</v>
-      </c>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-    </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" s="4"/>
-      <c r="B46" s="4"/>
+      <c r="A46" s="4">
+        <v>25</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>1174</v>
+      </c>
       <c r="C46" s="2" t="s">
-        <v>1170</v>
-      </c>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+        <v>1175</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="4"/>
       <c r="B47" s="4"/>
       <c r="C47" s="2" t="s">
-        <v>1171</v>
+        <v>1176</v>
       </c>
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="2">
-        <v>24</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>1035</v>
-      </c>
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
       <c r="C48" s="2" t="s">
-        <v>1036</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>851</v>
-      </c>
+        <v>1177</v>
+      </c>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>1172</v>
+        <v>1178</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>1173</v>
+        <v>1179</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>248</v>
@@ -15508,114 +15516,114 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="4">
-        <v>26</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>1174</v>
+      <c r="A50" s="2">
+        <v>27</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>1180</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1175</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>468</v>
+        <v>889</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>616</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="4"/>
-      <c r="B51" s="4"/>
+      <c r="A51" s="4">
+        <v>28</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>1181</v>
+      </c>
       <c r="C51" s="2" t="s">
-        <v>1176</v>
-      </c>
-      <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
+        <v>1182</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>1187</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>531</v>
+      </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="4"/>
       <c r="B52" s="4"/>
       <c r="C52" s="2" t="s">
-        <v>1177</v>
+        <v>1183</v>
       </c>
       <c r="D52" s="4"/>
       <c r="E52" s="4"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" s="2">
-        <v>27</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>1178</v>
-      </c>
+      <c r="A53" s="4"/>
+      <c r="B53" s="4"/>
       <c r="C53" s="2" t="s">
-        <v>1179</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>468</v>
-      </c>
+        <v>1184</v>
+      </c>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" s="2">
-        <v>28</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>1180</v>
-      </c>
+      <c r="A54" s="4"/>
+      <c r="B54" s="4"/>
       <c r="C54" s="2" t="s">
-        <v>889</v>
-      </c>
-      <c r="D54" s="2" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" s="4"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" s="2">
+        <v>29</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>1188</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E54" s="2" t="s">
+      <c r="E56" s="2" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A55" s="4">
-        <v>29</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>1181</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>1182</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>1187</v>
-      </c>
-      <c r="E55" s="4" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A56" s="4"/>
-      <c r="B56" s="4"/>
-      <c r="C56" s="2" t="s">
-        <v>1183</v>
-      </c>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
-    </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A57" s="4"/>
-      <c r="B57" s="4"/>
+      <c r="A57" s="4">
+        <v>30</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>669</v>
+      </c>
       <c r="C57" s="2" t="s">
-        <v>1184</v>
-      </c>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
+        <v>673</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>680</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>1192</v>
+      </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="4"/>
       <c r="B58" s="4"/>
       <c r="C58" s="2" t="s">
-        <v>1185</v>
+        <v>678</v>
       </c>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -15624,223 +15632,223 @@
       <c r="A59" s="4"/>
       <c r="B59" s="4"/>
       <c r="C59" s="2" t="s">
-        <v>1186</v>
+        <v>670</v>
       </c>
       <c r="D59" s="4"/>
       <c r="E59" s="4"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A60" s="2">
-        <v>30</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>1188</v>
-      </c>
+      <c r="A60" s="4"/>
+      <c r="B60" s="4"/>
       <c r="C60" s="2" t="s">
-        <v>1189</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>616</v>
-      </c>
+        <v>1190</v>
+      </c>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A61" s="4">
+      <c r="A61" s="4"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="2" t="s">
+        <v>1191</v>
+      </c>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" s="2">
         <v>31</v>
       </c>
-      <c r="B61" s="4" t="s">
-        <v>669</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>673</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>680</v>
-      </c>
-      <c r="E61" s="4" t="s">
-        <v>1192</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A62" s="4"/>
-      <c r="B62" s="4"/>
+      <c r="B62" s="2" t="s">
+        <v>1193</v>
+      </c>
       <c r="C62" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
+        <v>1194</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>854</v>
+      </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A63" s="4"/>
-      <c r="B63" s="4"/>
+      <c r="A63" s="2">
+        <v>32</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>1196</v>
+      </c>
       <c r="C63" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
+        <v>476</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>1197</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>477</v>
+      </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A64" s="4"/>
-      <c r="B64" s="4"/>
+      <c r="A64" s="4">
+        <v>33</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>1198</v>
+      </c>
       <c r="C64" s="2" t="s">
-        <v>1190</v>
-      </c>
-      <c r="D64" s="4"/>
-      <c r="E64" s="4"/>
+        <v>1199</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>1201</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="4"/>
       <c r="B65" s="4"/>
       <c r="C65" s="2" t="s">
-        <v>1191</v>
+        <v>1200</v>
       </c>
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>1193</v>
+        <v>1202</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>1194</v>
+        <v>1203</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>1195</v>
+        <v>2</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>854</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>1196</v>
+        <v>1011</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>476</v>
+        <v>381</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>1197</v>
+        <v>860</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>477</v>
+        <v>513</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="4">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>1198</v>
+        <v>1204</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>1199</v>
+        <v>927</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>1201</v>
+        <v>929</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>541</v>
+        <v>652</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="4"/>
       <c r="B69" s="4"/>
       <c r="C69" s="2" t="s">
-        <v>1200</v>
+        <v>928</v>
       </c>
       <c r="D69" s="4"/>
       <c r="E69" s="4"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A70" s="2">
-        <v>35</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>1202</v>
+      <c r="A70" s="4">
+        <v>37</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>177</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>1203</v>
-      </c>
-      <c r="D70" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71" s="4"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="2" t="s">
+        <v>1206</v>
+      </c>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A72" s="4"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="2" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" s="2">
+        <v>38</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>1208</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E70" s="2" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A71" s="2">
-        <v>36</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>1011</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>860</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A72" s="4">
-        <v>37</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>1204</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>927</v>
-      </c>
-      <c r="D72" s="4" t="s">
-        <v>929</v>
-      </c>
-      <c r="E72" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A73" s="4"/>
-      <c r="B73" s="4"/>
-      <c r="C73" s="2" t="s">
-        <v>928</v>
-      </c>
-      <c r="D73" s="4"/>
-      <c r="E73" s="4"/>
+      <c r="E73" s="2" t="s">
+        <v>559</v>
+      </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="4">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>177</v>
+        <v>1209</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>1205</v>
+        <v>509</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>184</v>
+        <v>248</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>531</v>
+        <v>468</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="4"/>
       <c r="B75" s="4"/>
       <c r="C75" s="2" t="s">
-        <v>1206</v>
+        <v>1210</v>
       </c>
       <c r="D75" s="4"/>
       <c r="E75" s="4"/>
@@ -15849,180 +15857,164 @@
       <c r="A76" s="4"/>
       <c r="B76" s="4"/>
       <c r="C76" s="2" t="s">
-        <v>1207</v>
+        <v>1211</v>
       </c>
       <c r="D76" s="4"/>
       <c r="E76" s="4"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A77" s="2">
-        <v>39</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>1208</v>
-      </c>
+      <c r="A77" s="4"/>
+      <c r="B77" s="4"/>
       <c r="C77" s="2" t="s">
-        <v>634</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>559</v>
-      </c>
+        <v>1212</v>
+      </c>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A78" s="4">
-        <v>40</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>1209</v>
-      </c>
+      <c r="A78" s="4"/>
+      <c r="B78" s="4"/>
       <c r="C78" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="E78" s="4" t="s">
-        <v>468</v>
-      </c>
+        <v>1213</v>
+      </c>
+      <c r="D78" s="4"/>
+      <c r="E78" s="4"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="4"/>
       <c r="B79" s="4"/>
       <c r="C79" s="2" t="s">
-        <v>1210</v>
+        <v>1214</v>
       </c>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A80" s="4"/>
-      <c r="B80" s="4"/>
+      <c r="A80" s="2">
+        <v>40</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>1215</v>
+      </c>
       <c r="C80" s="2" t="s">
-        <v>1211</v>
-      </c>
-      <c r="D80" s="4"/>
-      <c r="E80" s="4"/>
+        <v>429</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A81" s="4"/>
-      <c r="B81" s="4"/>
+      <c r="A81" s="2">
+        <v>41</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>1216</v>
+      </c>
       <c r="C81" s="2" t="s">
-        <v>1212</v>
-      </c>
-      <c r="D81" s="4"/>
-      <c r="E81" s="4"/>
+        <v>1217</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>1218</v>
+      </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A82" s="4"/>
-      <c r="B82" s="4"/>
+      <c r="A82" s="2">
+        <v>42</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>522</v>
+      </c>
       <c r="C82" s="2" t="s">
-        <v>1213</v>
-      </c>
-      <c r="D82" s="4"/>
-      <c r="E82" s="4"/>
+        <v>91</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A83" s="4"/>
-      <c r="B83" s="4"/>
+      <c r="A83" s="2">
+        <v>43</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>1219</v>
+      </c>
       <c r="C83" s="2" t="s">
-        <v>1214</v>
-      </c>
-      <c r="D83" s="4"/>
-      <c r="E83" s="4"/>
+        <v>1220</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>1221</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>846</v>
+      </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A84" s="2">
-        <v>41</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>1215</v>
+      <c r="A84" s="4">
+        <v>44</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>384</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E84" s="2" t="s">
-        <v>468</v>
+        <v>964</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>491</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A85" s="2">
-        <v>42</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>1216</v>
-      </c>
+      <c r="A85" s="4"/>
+      <c r="B85" s="4"/>
       <c r="C85" s="2" t="s">
-        <v>1217</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E85" s="2" t="s">
-        <v>1218</v>
-      </c>
+        <v>1222</v>
+      </c>
+      <c r="D85" s="4"/>
+      <c r="E85" s="4"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A86" s="2">
-        <v>43</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>522</v>
-      </c>
+      <c r="A86" s="4"/>
+      <c r="B86" s="4"/>
       <c r="C86" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E86" s="2" t="s">
-        <v>468</v>
-      </c>
+        <v>823</v>
+      </c>
+      <c r="D86" s="4"/>
+      <c r="E86" s="4"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A87" s="2">
-        <v>44</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>1219</v>
-      </c>
+      <c r="A87" s="4"/>
+      <c r="B87" s="4"/>
       <c r="C87" s="2" t="s">
-        <v>1220</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>1221</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>846</v>
-      </c>
+        <v>1223</v>
+      </c>
+      <c r="D87" s="4"/>
+      <c r="E87" s="4"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A88" s="4">
-        <v>45</v>
-      </c>
-      <c r="B88" s="4" t="s">
-        <v>384</v>
-      </c>
+      <c r="A88" s="4"/>
+      <c r="B88" s="4"/>
       <c r="C88" s="2" t="s">
-        <v>964</v>
-      </c>
-      <c r="D88" s="4" t="s">
-        <v>395</v>
-      </c>
-      <c r="E88" s="4" t="s">
-        <v>491</v>
-      </c>
+        <v>1224</v>
+      </c>
+      <c r="D88" s="4"/>
+      <c r="E88" s="4"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="4"/>
       <c r="B89" s="4"/>
       <c r="C89" s="2" t="s">
-        <v>1222</v>
+        <v>960</v>
       </c>
       <c r="D89" s="4"/>
       <c r="E89" s="4"/>
@@ -16031,7 +16023,7 @@
       <c r="A90" s="4"/>
       <c r="B90" s="4"/>
       <c r="C90" s="2" t="s">
-        <v>823</v>
+        <v>959</v>
       </c>
       <c r="D90" s="4"/>
       <c r="E90" s="4"/>
@@ -16040,7 +16032,7 @@
       <c r="A91" s="4"/>
       <c r="B91" s="4"/>
       <c r="C91" s="2" t="s">
-        <v>1223</v>
+        <v>1225</v>
       </c>
       <c r="D91" s="4"/>
       <c r="E91" s="4"/>
@@ -16049,7 +16041,7 @@
       <c r="A92" s="4"/>
       <c r="B92" s="4"/>
       <c r="C92" s="2" t="s">
-        <v>1224</v>
+        <v>1226</v>
       </c>
       <c r="D92" s="4"/>
       <c r="E92" s="4"/>
@@ -16058,7 +16050,7 @@
       <c r="A93" s="4"/>
       <c r="B93" s="4"/>
       <c r="C93" s="2" t="s">
-        <v>960</v>
+        <v>743</v>
       </c>
       <c r="D93" s="4"/>
       <c r="E93" s="4"/>
@@ -16067,25 +16059,33 @@
       <c r="A94" s="4"/>
       <c r="B94" s="4"/>
       <c r="C94" s="2" t="s">
-        <v>959</v>
+        <v>744</v>
       </c>
       <c r="D94" s="4"/>
       <c r="E94" s="4"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A95" s="4"/>
-      <c r="B95" s="4"/>
+      <c r="A95" s="4">
+        <v>45</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>1227</v>
+      </c>
       <c r="C95" s="2" t="s">
-        <v>1225</v>
-      </c>
-      <c r="D95" s="4"/>
-      <c r="E95" s="4"/>
+        <v>1228</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>1232</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>491</v>
+      </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="4"/>
       <c r="B96" s="4"/>
       <c r="C96" s="2" t="s">
-        <v>1226</v>
+        <v>1229</v>
       </c>
       <c r="D96" s="4"/>
       <c r="E96" s="4"/>
@@ -16094,7 +16094,7 @@
       <c r="A97" s="4"/>
       <c r="B97" s="4"/>
       <c r="C97" s="2" t="s">
-        <v>743</v>
+        <v>1230</v>
       </c>
       <c r="D97" s="4"/>
       <c r="E97" s="4"/>
@@ -16103,163 +16103,155 @@
       <c r="A98" s="4"/>
       <c r="B98" s="4"/>
       <c r="C98" s="2" t="s">
-        <v>744</v>
+        <v>1231</v>
       </c>
       <c r="D98" s="4"/>
       <c r="E98" s="4"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A99" s="4">
+      <c r="A99" s="2">
         <v>46</v>
       </c>
-      <c r="B99" s="4" t="s">
-        <v>1227</v>
+      <c r="B99" s="2" t="s">
+        <v>1233</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>1228</v>
-      </c>
-      <c r="D99" s="4" t="s">
-        <v>1232</v>
-      </c>
-      <c r="E99" s="4" t="s">
-        <v>491</v>
+        <v>1234</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>1235</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>486</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A100" s="4"/>
-      <c r="B100" s="4"/>
+      <c r="A100" s="4">
+        <v>47</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>1095</v>
+      </c>
       <c r="C100" s="2" t="s">
-        <v>1229</v>
-      </c>
-      <c r="D100" s="4"/>
-      <c r="E100" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>531</v>
+      </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="4"/>
       <c r="B101" s="4"/>
       <c r="C101" s="2" t="s">
-        <v>1230</v>
+        <v>1096</v>
       </c>
       <c r="D101" s="4"/>
       <c r="E101" s="4"/>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A102" s="4"/>
-      <c r="B102" s="4"/>
+    <row r="102" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A102" s="4">
+        <v>48</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>1236</v>
+      </c>
       <c r="C102" s="2" t="s">
-        <v>1231</v>
-      </c>
-      <c r="D102" s="4"/>
-      <c r="E102" s="4"/>
+        <v>1237</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>1239</v>
+      </c>
+      <c r="E102" s="4" t="s">
+        <v>531</v>
+      </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A103" s="2">
-        <v>47</v>
-      </c>
-      <c r="B103" s="2" t="s">
-        <v>1233</v>
-      </c>
+      <c r="A103" s="4"/>
+      <c r="B103" s="4"/>
       <c r="C103" s="2" t="s">
-        <v>1234</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>1235</v>
-      </c>
-      <c r="E103" s="2" t="s">
-        <v>486</v>
-      </c>
+        <v>1238</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A104" s="4">
-        <v>48</v>
-      </c>
-      <c r="B104" s="4" t="s">
-        <v>1095</v>
+      <c r="A104" s="2">
+        <v>49</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>1240</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D104" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D104" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E104" s="4" t="s">
-        <v>531</v>
+      <c r="E104" s="2" t="s">
+        <v>491</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A105" s="4"/>
-      <c r="B105" s="4"/>
+      <c r="A105" s="4">
+        <v>50</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>420</v>
+      </c>
       <c r="C105" s="2" t="s">
-        <v>1096</v>
-      </c>
-      <c r="D105" s="4"/>
-      <c r="E105" s="4"/>
-    </row>
-    <row r="106" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A106" s="4">
-        <v>49</v>
-      </c>
-      <c r="B106" s="4" t="s">
-        <v>1236</v>
-      </c>
+        <v>777</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="E105" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A106" s="4"/>
+      <c r="B106" s="4"/>
       <c r="C106" s="2" t="s">
-        <v>1237</v>
-      </c>
-      <c r="D106" s="4" t="s">
-        <v>1239</v>
-      </c>
-      <c r="E106" s="4" t="s">
-        <v>531</v>
-      </c>
+        <v>1241</v>
+      </c>
+      <c r="D106" s="4"/>
+      <c r="E106" s="4"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="4"/>
       <c r="B107" s="4"/>
       <c r="C107" s="2" t="s">
-        <v>1238</v>
+        <v>1242</v>
       </c>
       <c r="D107" s="4"/>
       <c r="E107" s="4"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A108" s="2">
-        <v>50</v>
-      </c>
-      <c r="B108" s="2" t="s">
-        <v>1240</v>
-      </c>
+      <c r="A108" s="4"/>
+      <c r="B108" s="4"/>
       <c r="C108" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D108" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E108" s="2" t="s">
-        <v>491</v>
-      </c>
+        <v>1243</v>
+      </c>
+      <c r="D108" s="4"/>
+      <c r="E108" s="4"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A109" s="4">
-        <v>51</v>
-      </c>
-      <c r="B109" s="4" t="s">
-        <v>420</v>
-      </c>
+      <c r="A109" s="4"/>
+      <c r="B109" s="4"/>
       <c r="C109" s="2" t="s">
-        <v>777</v>
-      </c>
-      <c r="D109" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="E109" s="4" t="s">
-        <v>468</v>
-      </c>
+        <v>786</v>
+      </c>
+      <c r="D109" s="4"/>
+      <c r="E109" s="4"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="4"/>
       <c r="B110" s="4"/>
       <c r="C110" s="2" t="s">
-        <v>1241</v>
+        <v>1244</v>
       </c>
       <c r="D110" s="4"/>
       <c r="E110" s="4"/>
@@ -16268,7 +16260,7 @@
       <c r="A111" s="4"/>
       <c r="B111" s="4"/>
       <c r="C111" s="2" t="s">
-        <v>1242</v>
+        <v>1245</v>
       </c>
       <c r="D111" s="4"/>
       <c r="E111" s="4"/>
@@ -16277,7 +16269,7 @@
       <c r="A112" s="4"/>
       <c r="B112" s="4"/>
       <c r="C112" s="2" t="s">
-        <v>1243</v>
+        <v>427</v>
       </c>
       <c r="D112" s="4"/>
       <c r="E112" s="4"/>
@@ -16286,7 +16278,7 @@
       <c r="A113" s="4"/>
       <c r="B113" s="4"/>
       <c r="C113" s="2" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="D113" s="4"/>
       <c r="E113" s="4"/>
@@ -16295,7 +16287,7 @@
       <c r="A114" s="4"/>
       <c r="B114" s="4"/>
       <c r="C114" s="2" t="s">
-        <v>1244</v>
+        <v>1246</v>
       </c>
       <c r="D114" s="4"/>
       <c r="E114" s="4"/>
@@ -16304,7 +16296,7 @@
       <c r="A115" s="4"/>
       <c r="B115" s="4"/>
       <c r="C115" s="2" t="s">
-        <v>1245</v>
+        <v>778</v>
       </c>
       <c r="D115" s="4"/>
       <c r="E115" s="4"/>
@@ -16313,7 +16305,7 @@
       <c r="A116" s="4"/>
       <c r="B116" s="4"/>
       <c r="C116" s="2" t="s">
-        <v>427</v>
+        <v>1247</v>
       </c>
       <c r="D116" s="4"/>
       <c r="E116" s="4"/>
@@ -16322,7 +16314,7 @@
       <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="2" t="s">
-        <v>781</v>
+        <v>1248</v>
       </c>
       <c r="D117" s="4"/>
       <c r="E117" s="4"/>
@@ -16331,7 +16323,7 @@
       <c r="A118" s="4"/>
       <c r="B118" s="4"/>
       <c r="C118" s="2" t="s">
-        <v>1246</v>
+        <v>1249</v>
       </c>
       <c r="D118" s="4"/>
       <c r="E118" s="4"/>
@@ -16340,112 +16332,112 @@
       <c r="A119" s="4"/>
       <c r="B119" s="4"/>
       <c r="C119" s="2" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="D119" s="4"/>
       <c r="E119" s="4"/>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A120" s="4"/>
-      <c r="B120" s="4"/>
+      <c r="A120" s="2">
+        <v>51</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>1250</v>
+      </c>
       <c r="C120" s="2" t="s">
-        <v>1247</v>
-      </c>
-      <c r="D120" s="4"/>
-      <c r="E120" s="4"/>
+        <v>1005</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>1010</v>
+      </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A121" s="4"/>
-      <c r="B121" s="4"/>
+      <c r="A121" s="4">
+        <v>52</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>1102</v>
+      </c>
       <c r="C121" s="2" t="s">
-        <v>1248</v>
-      </c>
-      <c r="D121" s="4"/>
-      <c r="E121" s="4"/>
+        <v>1103</v>
+      </c>
+      <c r="D121" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E121" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="2" t="s">
-        <v>1249</v>
+        <v>1252</v>
       </c>
       <c r="D122" s="4"/>
       <c r="E122" s="4"/>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A123" s="4"/>
-      <c r="B123" s="4"/>
+      <c r="A123" s="4">
+        <v>53</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>1167</v>
+      </c>
       <c r="C123" s="2" t="s">
-        <v>779</v>
-      </c>
-      <c r="D123" s="4"/>
-      <c r="E123" s="4"/>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A124" s="2">
-        <v>52</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>1250</v>
-      </c>
+        <v>1168</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E123" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A124" s="4"/>
+      <c r="B124" s="4"/>
       <c r="C124" s="2" t="s">
-        <v>1005</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>1251</v>
-      </c>
-      <c r="E124" s="2" t="s">
-        <v>1010</v>
-      </c>
+        <v>1169</v>
+      </c>
+      <c r="D124" s="4"/>
+      <c r="E124" s="4"/>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A125" s="4">
-        <v>53</v>
-      </c>
-      <c r="B125" s="4" t="s">
-        <v>1102</v>
-      </c>
+      <c r="A125" s="4"/>
+      <c r="B125" s="4"/>
       <c r="C125" s="2" t="s">
-        <v>1103</v>
-      </c>
-      <c r="D125" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E125" s="4" t="s">
-        <v>468</v>
-      </c>
+        <v>1170</v>
+      </c>
+      <c r="D125" s="4"/>
+      <c r="E125" s="4"/>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="4"/>
       <c r="B126" s="4"/>
       <c r="C126" s="2" t="s">
-        <v>1252</v>
+        <v>1171</v>
       </c>
       <c r="D126" s="4"/>
       <c r="E126" s="4"/>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A127" s="4">
-        <v>54</v>
-      </c>
-      <c r="B127" s="4" t="s">
-        <v>1167</v>
-      </c>
+      <c r="A127" s="4"/>
+      <c r="B127" s="4"/>
       <c r="C127" s="2" t="s">
-        <v>1168</v>
-      </c>
-      <c r="D127" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="E127" s="4" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="128" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>1253</v>
+      </c>
+      <c r="D127" s="4"/>
+      <c r="E127" s="4"/>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="4"/>
       <c r="B128" s="4"/>
       <c r="C128" s="2" t="s">
-        <v>1169</v>
+        <v>1254</v>
       </c>
       <c r="D128" s="4"/>
       <c r="E128" s="4"/>
@@ -16454,7 +16446,7 @@
       <c r="A129" s="4"/>
       <c r="B129" s="4"/>
       <c r="C129" s="2" t="s">
-        <v>1170</v>
+        <v>1255</v>
       </c>
       <c r="D129" s="4"/>
       <c r="E129" s="4"/>
@@ -16463,154 +16455,114 @@
       <c r="A130" s="4"/>
       <c r="B130" s="4"/>
       <c r="C130" s="2" t="s">
-        <v>1171</v>
+        <v>1256</v>
       </c>
       <c r="D130" s="4"/>
       <c r="E130" s="4"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A131" s="4"/>
-      <c r="B131" s="4"/>
+      <c r="A131" s="2">
+        <v>54</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>1257</v>
+      </c>
       <c r="C131" s="2" t="s">
-        <v>1253</v>
-      </c>
-      <c r="D131" s="4"/>
-      <c r="E131" s="4"/>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A132" s="4"/>
-      <c r="B132" s="4"/>
-      <c r="C132" s="2" t="s">
-        <v>1254</v>
-      </c>
-      <c r="D132" s="4"/>
-      <c r="E132" s="4"/>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A133" s="4"/>
-      <c r="B133" s="4"/>
-      <c r="C133" s="2" t="s">
-        <v>1255</v>
-      </c>
-      <c r="D133" s="4"/>
-      <c r="E133" s="4"/>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A134" s="4"/>
-      <c r="B134" s="4"/>
-      <c r="C134" s="2" t="s">
-        <v>1256</v>
-      </c>
-      <c r="D134" s="4"/>
-      <c r="E134" s="4"/>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A135" s="2">
-        <v>55</v>
-      </c>
-      <c r="B135" s="2" t="s">
-        <v>1257</v>
-      </c>
-      <c r="C135" s="2" t="s">
         <v>1258</v>
       </c>
-      <c r="D135" s="2" t="s">
+      <c r="D131" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E135" s="2" t="s">
+      <c r="E131" s="2" t="s">
         <v>468</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="88">
-    <mergeCell ref="D125:D126"/>
-    <mergeCell ref="E125:E126"/>
-    <mergeCell ref="A127:A134"/>
-    <mergeCell ref="B127:B134"/>
-    <mergeCell ref="D127:D134"/>
-    <mergeCell ref="E127:E134"/>
-    <mergeCell ref="D106:D107"/>
-    <mergeCell ref="E106:E107"/>
-    <mergeCell ref="A109:A123"/>
-    <mergeCell ref="B109:B123"/>
-    <mergeCell ref="D109:D123"/>
-    <mergeCell ref="E109:E123"/>
-    <mergeCell ref="D99:D102"/>
-    <mergeCell ref="E99:E102"/>
-    <mergeCell ref="A104:A105"/>
-    <mergeCell ref="B104:B105"/>
-    <mergeCell ref="D104:D105"/>
-    <mergeCell ref="E104:E105"/>
-    <mergeCell ref="D78:D83"/>
-    <mergeCell ref="E78:E83"/>
-    <mergeCell ref="A88:A98"/>
-    <mergeCell ref="B88:B98"/>
-    <mergeCell ref="D88:D98"/>
-    <mergeCell ref="E88:E98"/>
-    <mergeCell ref="D72:D73"/>
-    <mergeCell ref="E72:E73"/>
-    <mergeCell ref="A74:A76"/>
-    <mergeCell ref="B74:B76"/>
-    <mergeCell ref="D74:D76"/>
-    <mergeCell ref="E74:E76"/>
-    <mergeCell ref="D61:D65"/>
-    <mergeCell ref="E61:E65"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="E68:E69"/>
-    <mergeCell ref="D50:D52"/>
-    <mergeCell ref="E50:E52"/>
-    <mergeCell ref="A55:A59"/>
-    <mergeCell ref="B55:B59"/>
-    <mergeCell ref="D55:D59"/>
-    <mergeCell ref="E55:E59"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="D39:D41"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="A44:A47"/>
-    <mergeCell ref="B44:B47"/>
-    <mergeCell ref="D44:D47"/>
-    <mergeCell ref="E44:E47"/>
+  <mergeCells count="84">
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="A11:A19"/>
+    <mergeCell ref="B11:B19"/>
+    <mergeCell ref="D11:D19"/>
+    <mergeCell ref="E11:E19"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="A25:A28"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="D25:D28"/>
+    <mergeCell ref="E25:E28"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
     <mergeCell ref="D30:D32"/>
     <mergeCell ref="E30:E32"/>
     <mergeCell ref="A33:A36"/>
     <mergeCell ref="B33:B36"/>
     <mergeCell ref="D33:D36"/>
     <mergeCell ref="E33:E36"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="A25:A28"/>
-    <mergeCell ref="B25:B28"/>
-    <mergeCell ref="D25:D28"/>
-    <mergeCell ref="E25:E28"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="A11:A19"/>
-    <mergeCell ref="B11:B19"/>
-    <mergeCell ref="D11:D19"/>
-    <mergeCell ref="E11:E19"/>
-    <mergeCell ref="A125:A126"/>
-    <mergeCell ref="B125:B126"/>
-    <mergeCell ref="A106:A107"/>
-    <mergeCell ref="B106:B107"/>
-    <mergeCell ref="A99:A102"/>
-    <mergeCell ref="B99:B102"/>
-    <mergeCell ref="A78:A83"/>
-    <mergeCell ref="B78:B83"/>
-    <mergeCell ref="A72:A73"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="A61:A65"/>
-    <mergeCell ref="B61:B65"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="B50:B52"/>
     <mergeCell ref="A30:A32"/>
     <mergeCell ref="B30:B32"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="A46:A48"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="A51:A55"/>
+    <mergeCell ref="B51:B55"/>
+    <mergeCell ref="D51:D55"/>
+    <mergeCell ref="E51:E55"/>
+    <mergeCell ref="A57:A61"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="D57:D61"/>
+    <mergeCell ref="E57:E61"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="E68:E69"/>
+    <mergeCell ref="A64:A65"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="A70:A72"/>
+    <mergeCell ref="B70:B72"/>
+    <mergeCell ref="D70:D72"/>
+    <mergeCell ref="E70:E72"/>
+    <mergeCell ref="A74:A79"/>
+    <mergeCell ref="B74:B79"/>
+    <mergeCell ref="D74:D79"/>
+    <mergeCell ref="E74:E79"/>
+    <mergeCell ref="A84:A94"/>
+    <mergeCell ref="B84:B94"/>
+    <mergeCell ref="D84:D94"/>
+    <mergeCell ref="E84:E94"/>
+    <mergeCell ref="A95:A98"/>
+    <mergeCell ref="B95:B98"/>
+    <mergeCell ref="D95:D98"/>
+    <mergeCell ref="E95:E98"/>
+    <mergeCell ref="A100:A101"/>
+    <mergeCell ref="B100:B101"/>
+    <mergeCell ref="D100:D101"/>
+    <mergeCell ref="E100:E101"/>
+    <mergeCell ref="A102:A103"/>
+    <mergeCell ref="B102:B103"/>
+    <mergeCell ref="D102:D103"/>
+    <mergeCell ref="E102:E103"/>
+    <mergeCell ref="A105:A119"/>
+    <mergeCell ref="B105:B119"/>
+    <mergeCell ref="D105:D119"/>
+    <mergeCell ref="E105:E119"/>
+    <mergeCell ref="A121:A122"/>
+    <mergeCell ref="B121:B122"/>
+    <mergeCell ref="D121:D122"/>
+    <mergeCell ref="E121:E122"/>
+    <mergeCell ref="A123:A130"/>
+    <mergeCell ref="B123:B130"/>
+    <mergeCell ref="D123:D130"/>
+    <mergeCell ref="E123:E130"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update participant analysis for IROS 2026
</commit_message>
<xml_diff>
--- a/Registration.xlsx
+++ b/Registration.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tsamak\Workspace\AutoDRIVE-RoboRacer-Sim-Racing-Participation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D7CB4F3-39F3-4BD5-B7A2-AD8952BF4608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF75D124-B283-410B-8FD6-F08DB19AD05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="5" xr2:uid="{5D9342A3-8B90-4963-824C-8C358DE1DB7F}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1980" uniqueCount="1259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1984" uniqueCount="1260">
   <si>
     <t>SAGOL</t>
   </si>
@@ -3818,6 +3818,9 @@
   </si>
   <si>
     <t>Krishn Singh</t>
+  </si>
+  <si>
+    <t>FEBAuto</t>
   </si>
 </sst>
 </file>
@@ -6197,85 +6200,37 @@
     </row>
   </sheetData>
   <mergeCells count="124">
-    <mergeCell ref="E159:E161"/>
-    <mergeCell ref="E135:E137"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="E142:E148"/>
-    <mergeCell ref="E149:E152"/>
-    <mergeCell ref="E154:E158"/>
-    <mergeCell ref="E111:E116"/>
-    <mergeCell ref="E117:E118"/>
-    <mergeCell ref="E122:E123"/>
-    <mergeCell ref="E124:E131"/>
-    <mergeCell ref="E132:E134"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="E99:E102"/>
-    <mergeCell ref="E103:E105"/>
-    <mergeCell ref="E106:E107"/>
-    <mergeCell ref="E108:E110"/>
-    <mergeCell ref="E71:E76"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="E84:E89"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="E35:E46"/>
-    <mergeCell ref="E50:E54"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E59:E65"/>
-    <mergeCell ref="E67:E70"/>
-    <mergeCell ref="E6:E14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E21:E24"/>
-    <mergeCell ref="E27:E31"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="A27:A31"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A35:A46"/>
-    <mergeCell ref="B35:B46"/>
-    <mergeCell ref="A6:A14"/>
-    <mergeCell ref="B6:B14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="B21:B24"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A71:A76"/>
-    <mergeCell ref="B71:B76"/>
-    <mergeCell ref="A77:A78"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="A50:A54"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="A59:A65"/>
-    <mergeCell ref="B59:B65"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="A99:A102"/>
-    <mergeCell ref="B99:B102"/>
-    <mergeCell ref="A103:A105"/>
-    <mergeCell ref="B103:B105"/>
-    <mergeCell ref="A81:A82"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="A84:A89"/>
-    <mergeCell ref="B84:B89"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="A117:A118"/>
-    <mergeCell ref="B117:B118"/>
-    <mergeCell ref="A122:A123"/>
-    <mergeCell ref="B122:B123"/>
-    <mergeCell ref="A124:A131"/>
-    <mergeCell ref="B124:B131"/>
-    <mergeCell ref="A106:A107"/>
-    <mergeCell ref="B106:B107"/>
-    <mergeCell ref="A108:A110"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="A111:A116"/>
-    <mergeCell ref="B111:B116"/>
+    <mergeCell ref="D27:D31"/>
+    <mergeCell ref="D21:D24"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="D6:D14"/>
+    <mergeCell ref="D81:D82"/>
+    <mergeCell ref="D77:D78"/>
+    <mergeCell ref="D71:D76"/>
+    <mergeCell ref="D67:D70"/>
+    <mergeCell ref="D59:D65"/>
+    <mergeCell ref="D55:D56"/>
+    <mergeCell ref="D50:D54"/>
+    <mergeCell ref="D35:D46"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="D103:D105"/>
+    <mergeCell ref="D99:D102"/>
+    <mergeCell ref="D111:D116"/>
+    <mergeCell ref="D108:D110"/>
+    <mergeCell ref="D106:D107"/>
+    <mergeCell ref="D117:D118"/>
+    <mergeCell ref="D95:D97"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="D84:D89"/>
+    <mergeCell ref="D154:D158"/>
+    <mergeCell ref="D159:D161"/>
+    <mergeCell ref="D124:D131"/>
+    <mergeCell ref="D122:D123"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="D135:D137"/>
+    <mergeCell ref="D132:D134"/>
+    <mergeCell ref="D149:D152"/>
+    <mergeCell ref="D142:D148"/>
     <mergeCell ref="A142:A148"/>
     <mergeCell ref="B142:B148"/>
     <mergeCell ref="A159:A161"/>
@@ -6290,37 +6245,85 @@
     <mergeCell ref="B135:B137"/>
     <mergeCell ref="A138:A141"/>
     <mergeCell ref="B138:B141"/>
-    <mergeCell ref="D154:D158"/>
-    <mergeCell ref="D159:D161"/>
-    <mergeCell ref="D124:D131"/>
-    <mergeCell ref="D122:D123"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="D135:D137"/>
-    <mergeCell ref="D132:D134"/>
-    <mergeCell ref="D149:D152"/>
-    <mergeCell ref="D142:D148"/>
-    <mergeCell ref="D103:D105"/>
-    <mergeCell ref="D99:D102"/>
-    <mergeCell ref="D111:D116"/>
-    <mergeCell ref="D108:D110"/>
-    <mergeCell ref="D106:D107"/>
-    <mergeCell ref="D117:D118"/>
-    <mergeCell ref="D95:D97"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="D84:D89"/>
-    <mergeCell ref="D27:D31"/>
-    <mergeCell ref="D21:D24"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="D6:D14"/>
-    <mergeCell ref="D81:D82"/>
-    <mergeCell ref="D77:D78"/>
-    <mergeCell ref="D71:D76"/>
-    <mergeCell ref="D67:D70"/>
-    <mergeCell ref="D59:D65"/>
-    <mergeCell ref="D55:D56"/>
-    <mergeCell ref="D50:D54"/>
-    <mergeCell ref="D35:D46"/>
-    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="A117:A118"/>
+    <mergeCell ref="B117:B118"/>
+    <mergeCell ref="A122:A123"/>
+    <mergeCell ref="B122:B123"/>
+    <mergeCell ref="A124:A131"/>
+    <mergeCell ref="B124:B131"/>
+    <mergeCell ref="A106:A107"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="A108:A110"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="A111:A116"/>
+    <mergeCell ref="B111:B116"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="A99:A102"/>
+    <mergeCell ref="B99:B102"/>
+    <mergeCell ref="A103:A105"/>
+    <mergeCell ref="B103:B105"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="A84:A89"/>
+    <mergeCell ref="B84:B89"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A71:A76"/>
+    <mergeCell ref="B71:B76"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="A50:A54"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="A59:A65"/>
+    <mergeCell ref="B59:B65"/>
+    <mergeCell ref="A27:A31"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A35:A46"/>
+    <mergeCell ref="B35:B46"/>
+    <mergeCell ref="A6:A14"/>
+    <mergeCell ref="B6:B14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="E35:E46"/>
+    <mergeCell ref="E50:E54"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E59:E65"/>
+    <mergeCell ref="E67:E70"/>
+    <mergeCell ref="E6:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E21:E24"/>
+    <mergeCell ref="E27:E31"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="E99:E102"/>
+    <mergeCell ref="E103:E105"/>
+    <mergeCell ref="E106:E107"/>
+    <mergeCell ref="E108:E110"/>
+    <mergeCell ref="E71:E76"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="E84:E89"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="E159:E161"/>
+    <mergeCell ref="E135:E137"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="E142:E148"/>
+    <mergeCell ref="E149:E152"/>
+    <mergeCell ref="E154:E158"/>
+    <mergeCell ref="E111:E116"/>
+    <mergeCell ref="E117:E118"/>
+    <mergeCell ref="E122:E123"/>
+    <mergeCell ref="E124:E131"/>
+    <mergeCell ref="E132:E134"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -8292,44 +8295,88 @@
     </row>
   </sheetData>
   <mergeCells count="144">
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="E170:E171"/>
-    <mergeCell ref="E102:E111"/>
-    <mergeCell ref="E112:E116"/>
-    <mergeCell ref="E117:E122"/>
-    <mergeCell ref="E123:E129"/>
-    <mergeCell ref="E130:E141"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="E150:E151"/>
-    <mergeCell ref="E152:E156"/>
-    <mergeCell ref="E75:E78"/>
-    <mergeCell ref="E80:E82"/>
-    <mergeCell ref="E84:E85"/>
-    <mergeCell ref="E86:E91"/>
-    <mergeCell ref="E92:E94"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="E157:E159"/>
-    <mergeCell ref="E160:E164"/>
-    <mergeCell ref="E38:E45"/>
-    <mergeCell ref="E46:E51"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="E62:E64"/>
-    <mergeCell ref="E66:E67"/>
-    <mergeCell ref="B8:B15"/>
-    <mergeCell ref="D8:D15"/>
-    <mergeCell ref="E68:E69"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E4:E7"/>
-    <mergeCell ref="E8:E15"/>
-    <mergeCell ref="E16:E19"/>
-    <mergeCell ref="E21:E23"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="E26:E30"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="E33:E37"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="D76:D78"/>
+    <mergeCell ref="D71:D73"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="D92:D94"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="A46:A51"/>
+    <mergeCell ref="B46:B51"/>
+    <mergeCell ref="D46:D51"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="B62:B64"/>
+    <mergeCell ref="D62:D64"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="A152:A156"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="A150:A151"/>
+    <mergeCell ref="A123:A129"/>
+    <mergeCell ref="A130:A141"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="A75:A78"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="A170:A171"/>
+    <mergeCell ref="B170:B171"/>
+    <mergeCell ref="D170:D171"/>
+    <mergeCell ref="A160:A164"/>
+    <mergeCell ref="B160:B164"/>
+    <mergeCell ref="D160:D164"/>
+    <mergeCell ref="A157:A159"/>
+    <mergeCell ref="B157:B159"/>
+    <mergeCell ref="D157:D159"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="B75:B78"/>
+    <mergeCell ref="B80:B82"/>
+    <mergeCell ref="D80:D82"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="D84:D85"/>
+    <mergeCell ref="B112:B116"/>
+    <mergeCell ref="D112:D116"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="D95:D97"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B86:B91"/>
+    <mergeCell ref="D86:D91"/>
+    <mergeCell ref="A112:A116"/>
+    <mergeCell ref="A86:A91"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="A102:A111"/>
+    <mergeCell ref="A117:A122"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="D150:D151"/>
+    <mergeCell ref="B152:B156"/>
+    <mergeCell ref="D152:D156"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="B117:B122"/>
+    <mergeCell ref="D117:D122"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="B102:B111"/>
+    <mergeCell ref="D102:D111"/>
+    <mergeCell ref="B123:B129"/>
+    <mergeCell ref="D123:D129"/>
+    <mergeCell ref="B130:B141"/>
+    <mergeCell ref="D130:D141"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="D142:D145"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="D2:D3"/>
@@ -8354,88 +8401,44 @@
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="D16:D19"/>
     <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="D150:D151"/>
-    <mergeCell ref="B152:B156"/>
-    <mergeCell ref="D152:D156"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="B117:B122"/>
-    <mergeCell ref="D117:D122"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="B102:B111"/>
-    <mergeCell ref="D102:D111"/>
-    <mergeCell ref="B123:B129"/>
-    <mergeCell ref="D123:D129"/>
-    <mergeCell ref="B130:B141"/>
-    <mergeCell ref="D130:D141"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="B75:B78"/>
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="D80:D82"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="D84:D85"/>
-    <mergeCell ref="B112:B116"/>
-    <mergeCell ref="D112:D116"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="D95:D97"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B86:B91"/>
-    <mergeCell ref="D86:D91"/>
-    <mergeCell ref="A112:A116"/>
-    <mergeCell ref="A86:A91"/>
-    <mergeCell ref="A84:A85"/>
-    <mergeCell ref="A102:A111"/>
-    <mergeCell ref="A117:A122"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="A170:A171"/>
-    <mergeCell ref="B170:B171"/>
-    <mergeCell ref="D170:D171"/>
-    <mergeCell ref="A160:A164"/>
-    <mergeCell ref="B160:B164"/>
-    <mergeCell ref="D160:D164"/>
-    <mergeCell ref="A157:A159"/>
-    <mergeCell ref="B157:B159"/>
-    <mergeCell ref="D157:D159"/>
-    <mergeCell ref="A152:A156"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="A150:A151"/>
-    <mergeCell ref="A123:A129"/>
-    <mergeCell ref="A130:A141"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A75:A78"/>
-    <mergeCell ref="A66:A67"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="D76:D78"/>
-    <mergeCell ref="D71:D73"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="D92:D94"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="A46:A51"/>
-    <mergeCell ref="B46:B51"/>
-    <mergeCell ref="D46:D51"/>
-    <mergeCell ref="A52:A53"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="B62:B64"/>
-    <mergeCell ref="D62:D64"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="E8:E15"/>
+    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="E26:E30"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="E33:E37"/>
+    <mergeCell ref="E38:E45"/>
+    <mergeCell ref="E46:E51"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="E62:E64"/>
+    <mergeCell ref="E66:E67"/>
+    <mergeCell ref="B8:B15"/>
+    <mergeCell ref="D8:D15"/>
+    <mergeCell ref="E68:E69"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="E75:E78"/>
+    <mergeCell ref="E80:E82"/>
+    <mergeCell ref="E84:E85"/>
+    <mergeCell ref="E86:E91"/>
+    <mergeCell ref="E92:E94"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="E157:E159"/>
+    <mergeCell ref="E160:E164"/>
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="E170:E171"/>
+    <mergeCell ref="E102:E111"/>
+    <mergeCell ref="E112:E116"/>
+    <mergeCell ref="E117:E122"/>
+    <mergeCell ref="E123:E129"/>
+    <mergeCell ref="E130:E141"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="E150:E151"/>
+    <mergeCell ref="E152:E156"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10270,90 +10273,29 @@
     </row>
   </sheetData>
   <mergeCells count="132">
-    <mergeCell ref="A145:A147"/>
-    <mergeCell ref="B145:B147"/>
-    <mergeCell ref="D145:D147"/>
-    <mergeCell ref="E145:E147"/>
-    <mergeCell ref="A149:A150"/>
-    <mergeCell ref="B149:B150"/>
-    <mergeCell ref="D149:D150"/>
-    <mergeCell ref="E149:E150"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="D131:D133"/>
-    <mergeCell ref="E131:E133"/>
-    <mergeCell ref="A135:A138"/>
-    <mergeCell ref="B135:B138"/>
-    <mergeCell ref="D135:D138"/>
-    <mergeCell ref="E135:E138"/>
-    <mergeCell ref="A139:A141"/>
-    <mergeCell ref="B139:B141"/>
-    <mergeCell ref="D139:D141"/>
-    <mergeCell ref="E139:E141"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="D114:D117"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="A118:A127"/>
-    <mergeCell ref="B118:B127"/>
-    <mergeCell ref="D118:D127"/>
-    <mergeCell ref="E118:E127"/>
-    <mergeCell ref="A81:A85"/>
-    <mergeCell ref="B81:B85"/>
-    <mergeCell ref="D81:D85"/>
-    <mergeCell ref="E81:E85"/>
-    <mergeCell ref="E87:E89"/>
-    <mergeCell ref="A90:A91"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="D90:D91"/>
-    <mergeCell ref="E90:E91"/>
-    <mergeCell ref="D1:D4"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E1:E4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="D65:D71"/>
-    <mergeCell ref="D73:D75"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="E57:E59"/>
-    <mergeCell ref="A60:A64"/>
-    <mergeCell ref="B60:B64"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="B51:B53"/>
-    <mergeCell ref="D51:D53"/>
-    <mergeCell ref="E51:E53"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="E42:E46"/>
-    <mergeCell ref="E73:E75"/>
-    <mergeCell ref="A73:A75"/>
-    <mergeCell ref="B73:B75"/>
-    <mergeCell ref="E65:E71"/>
-    <mergeCell ref="A48:A50"/>
+    <mergeCell ref="D48:D50"/>
+    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="A129:A130"/>
+    <mergeCell ref="B129:B130"/>
+    <mergeCell ref="D129:D130"/>
+    <mergeCell ref="E129:E130"/>
+    <mergeCell ref="A87:A89"/>
+    <mergeCell ref="B87:B89"/>
+    <mergeCell ref="D87:D89"/>
+    <mergeCell ref="A92:A97"/>
+    <mergeCell ref="B92:B97"/>
+    <mergeCell ref="D92:D97"/>
+    <mergeCell ref="E92:E97"/>
+    <mergeCell ref="A99:A109"/>
+    <mergeCell ref="B99:B109"/>
+    <mergeCell ref="D99:D109"/>
+    <mergeCell ref="E99:E109"/>
+    <mergeCell ref="A76:A80"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="D76:D80"/>
+    <mergeCell ref="E76:E80"/>
+    <mergeCell ref="A65:A71"/>
+    <mergeCell ref="B65:B71"/>
     <mergeCell ref="D29:D31"/>
     <mergeCell ref="E29:E31"/>
     <mergeCell ref="A20:A22"/>
@@ -10378,30 +10320,91 @@
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="B29:B31"/>
     <mergeCell ref="B1:B4"/>
+    <mergeCell ref="D65:D71"/>
+    <mergeCell ref="D73:D75"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="E57:E59"/>
+    <mergeCell ref="A60:A64"/>
+    <mergeCell ref="B60:B64"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="D51:D53"/>
+    <mergeCell ref="E51:E53"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="E42:E46"/>
+    <mergeCell ref="E73:E75"/>
+    <mergeCell ref="A73:A75"/>
+    <mergeCell ref="B73:B75"/>
+    <mergeCell ref="E65:E71"/>
+    <mergeCell ref="A48:A50"/>
     <mergeCell ref="B48:B50"/>
-    <mergeCell ref="D48:D50"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="A129:A130"/>
-    <mergeCell ref="B129:B130"/>
-    <mergeCell ref="D129:D130"/>
-    <mergeCell ref="E129:E130"/>
-    <mergeCell ref="A87:A89"/>
-    <mergeCell ref="B87:B89"/>
-    <mergeCell ref="D87:D89"/>
-    <mergeCell ref="A92:A97"/>
-    <mergeCell ref="B92:B97"/>
-    <mergeCell ref="D92:D97"/>
-    <mergeCell ref="E92:E97"/>
-    <mergeCell ref="A99:A109"/>
-    <mergeCell ref="B99:B109"/>
-    <mergeCell ref="D99:D109"/>
-    <mergeCell ref="E99:E109"/>
-    <mergeCell ref="A76:A80"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="D76:D80"/>
-    <mergeCell ref="E76:E80"/>
-    <mergeCell ref="A65:A71"/>
-    <mergeCell ref="B65:B71"/>
+    <mergeCell ref="D1:D4"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E1:E4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="A81:A85"/>
+    <mergeCell ref="B81:B85"/>
+    <mergeCell ref="D81:D85"/>
+    <mergeCell ref="E81:E85"/>
+    <mergeCell ref="E87:E89"/>
+    <mergeCell ref="A90:A91"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="D90:D91"/>
+    <mergeCell ref="E90:E91"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="D114:D117"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="A118:A127"/>
+    <mergeCell ref="B118:B127"/>
+    <mergeCell ref="D118:D127"/>
+    <mergeCell ref="E118:E127"/>
+    <mergeCell ref="A145:A147"/>
+    <mergeCell ref="B145:B147"/>
+    <mergeCell ref="D145:D147"/>
+    <mergeCell ref="E145:E147"/>
+    <mergeCell ref="A149:A150"/>
+    <mergeCell ref="B149:B150"/>
+    <mergeCell ref="D149:D150"/>
+    <mergeCell ref="E149:E150"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="D131:D133"/>
+    <mergeCell ref="E131:E133"/>
+    <mergeCell ref="A135:A138"/>
+    <mergeCell ref="B135:B138"/>
+    <mergeCell ref="D135:D138"/>
+    <mergeCell ref="E135:E138"/>
+    <mergeCell ref="A139:A141"/>
+    <mergeCell ref="B139:B141"/>
+    <mergeCell ref="D139:D141"/>
+    <mergeCell ref="E139:E141"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -12200,31 +12203,57 @@
     </row>
   </sheetData>
   <mergeCells count="92">
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="D36:D38"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="B28:B31"/>
-    <mergeCell ref="A32:A35"/>
-    <mergeCell ref="B32:B35"/>
-    <mergeCell ref="D32:D35"/>
-    <mergeCell ref="E32:E35"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D83:D89"/>
-    <mergeCell ref="E83:E89"/>
-    <mergeCell ref="A62:A67"/>
-    <mergeCell ref="B62:B67"/>
-    <mergeCell ref="D62:D67"/>
-    <mergeCell ref="E62:E67"/>
-    <mergeCell ref="A69:A72"/>
-    <mergeCell ref="B69:B72"/>
-    <mergeCell ref="D69:D72"/>
-    <mergeCell ref="E69:E72"/>
-    <mergeCell ref="A73:A82"/>
-    <mergeCell ref="B73:B82"/>
-    <mergeCell ref="D73:D82"/>
-    <mergeCell ref="E73:E82"/>
+    <mergeCell ref="A90:A95"/>
+    <mergeCell ref="A96:A100"/>
+    <mergeCell ref="A57:A61"/>
+    <mergeCell ref="A49:A54"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="A42:A47"/>
+    <mergeCell ref="A83:A89"/>
+    <mergeCell ref="A154:A156"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="D154:D156"/>
+    <mergeCell ref="E154:E156"/>
+    <mergeCell ref="A157:A158"/>
+    <mergeCell ref="B157:B158"/>
+    <mergeCell ref="D157:D158"/>
+    <mergeCell ref="E157:E158"/>
+    <mergeCell ref="D90:D95"/>
+    <mergeCell ref="E90:E95"/>
+    <mergeCell ref="B96:B100"/>
+    <mergeCell ref="D96:D100"/>
+    <mergeCell ref="E96:E100"/>
+    <mergeCell ref="B90:B95"/>
+    <mergeCell ref="D49:D54"/>
+    <mergeCell ref="E49:E54"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="D57:D61"/>
+    <mergeCell ref="E57:E61"/>
+    <mergeCell ref="B49:B54"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="B42:B47"/>
+    <mergeCell ref="D42:D47"/>
+    <mergeCell ref="E42:E47"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="A15:A24"/>
+    <mergeCell ref="B15:B24"/>
+    <mergeCell ref="D15:D24"/>
+    <mergeCell ref="E15:E24"/>
+    <mergeCell ref="D28:D31"/>
+    <mergeCell ref="E28:E31"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="E5:E8"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="B9:B13"/>
+    <mergeCell ref="D9:D13"/>
+    <mergeCell ref="E9:E13"/>
     <mergeCell ref="A129:A151"/>
     <mergeCell ref="B129:B151"/>
     <mergeCell ref="D129:D151"/>
@@ -12241,57 +12270,31 @@
     <mergeCell ref="B126:B128"/>
     <mergeCell ref="D126:D128"/>
     <mergeCell ref="E126:E128"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="D5:D8"/>
-    <mergeCell ref="E5:E8"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="B9:B13"/>
-    <mergeCell ref="D9:D13"/>
-    <mergeCell ref="E9:E13"/>
-    <mergeCell ref="A15:A24"/>
-    <mergeCell ref="B15:B24"/>
-    <mergeCell ref="D15:D24"/>
-    <mergeCell ref="E15:E24"/>
-    <mergeCell ref="D28:D31"/>
-    <mergeCell ref="E28:E31"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="D39:D41"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="B42:B47"/>
-    <mergeCell ref="D42:D47"/>
-    <mergeCell ref="E42:E47"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="D49:D54"/>
-    <mergeCell ref="E49:E54"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="D57:D61"/>
-    <mergeCell ref="E57:E61"/>
-    <mergeCell ref="B49:B54"/>
-    <mergeCell ref="D90:D95"/>
-    <mergeCell ref="E90:E95"/>
-    <mergeCell ref="B96:B100"/>
-    <mergeCell ref="D96:D100"/>
-    <mergeCell ref="E96:E100"/>
-    <mergeCell ref="B90:B95"/>
-    <mergeCell ref="A154:A156"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="D154:D156"/>
-    <mergeCell ref="E154:E156"/>
-    <mergeCell ref="A157:A158"/>
-    <mergeCell ref="B157:B158"/>
-    <mergeCell ref="D157:D158"/>
-    <mergeCell ref="E157:E158"/>
-    <mergeCell ref="A90:A95"/>
-    <mergeCell ref="A96:A100"/>
-    <mergeCell ref="A57:A61"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A42:A47"/>
-    <mergeCell ref="A83:A89"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D83:D89"/>
+    <mergeCell ref="E83:E89"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="B62:B67"/>
+    <mergeCell ref="D62:D67"/>
+    <mergeCell ref="E62:E67"/>
+    <mergeCell ref="A69:A72"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="D69:D72"/>
+    <mergeCell ref="E69:E72"/>
+    <mergeCell ref="A73:A82"/>
+    <mergeCell ref="B73:B82"/>
+    <mergeCell ref="D73:D82"/>
+    <mergeCell ref="E73:E82"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="D36:D38"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="B32:B35"/>
+    <mergeCell ref="D32:D35"/>
+    <mergeCell ref="E32:E35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14704,102 +14707,30 @@
     </row>
   </sheetData>
   <mergeCells count="144">
-    <mergeCell ref="A182:A183"/>
-    <mergeCell ref="B182:B183"/>
-    <mergeCell ref="D182:D183"/>
-    <mergeCell ref="E182:E183"/>
-    <mergeCell ref="A185:A191"/>
-    <mergeCell ref="B185:B191"/>
-    <mergeCell ref="D185:D191"/>
-    <mergeCell ref="E185:E191"/>
-    <mergeCell ref="A176:A177"/>
-    <mergeCell ref="B176:B177"/>
-    <mergeCell ref="D176:D177"/>
-    <mergeCell ref="E176:E177"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="A168:A170"/>
-    <mergeCell ref="B168:B170"/>
-    <mergeCell ref="D168:D170"/>
-    <mergeCell ref="E168:E170"/>
-    <mergeCell ref="A171:A175"/>
-    <mergeCell ref="B171:B175"/>
-    <mergeCell ref="D171:D175"/>
-    <mergeCell ref="E171:E175"/>
-    <mergeCell ref="A154:A161"/>
-    <mergeCell ref="B154:B161"/>
-    <mergeCell ref="D154:D161"/>
-    <mergeCell ref="E154:E161"/>
-    <mergeCell ref="A163:A165"/>
-    <mergeCell ref="B163:B165"/>
-    <mergeCell ref="D163:D165"/>
-    <mergeCell ref="E163:E165"/>
-    <mergeCell ref="A145:A149"/>
-    <mergeCell ref="B145:B149"/>
-    <mergeCell ref="D145:D149"/>
-    <mergeCell ref="E145:E149"/>
-    <mergeCell ref="A151:A153"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="D151:D153"/>
-    <mergeCell ref="E151:E153"/>
-    <mergeCell ref="D139:D141"/>
-    <mergeCell ref="E139:E141"/>
-    <mergeCell ref="A142:A143"/>
-    <mergeCell ref="B142:B143"/>
-    <mergeCell ref="D142:D143"/>
-    <mergeCell ref="E142:E143"/>
-    <mergeCell ref="D125:D127"/>
-    <mergeCell ref="E125:E127"/>
-    <mergeCell ref="A132:A133"/>
-    <mergeCell ref="B132:B133"/>
-    <mergeCell ref="D132:D133"/>
-    <mergeCell ref="E132:E133"/>
-    <mergeCell ref="A111:A112"/>
-    <mergeCell ref="B111:B112"/>
-    <mergeCell ref="D111:D112"/>
-    <mergeCell ref="E111:E112"/>
-    <mergeCell ref="A115:A123"/>
-    <mergeCell ref="B115:B123"/>
-    <mergeCell ref="D115:D123"/>
-    <mergeCell ref="E115:E123"/>
-    <mergeCell ref="A103:A106"/>
-    <mergeCell ref="B103:B106"/>
-    <mergeCell ref="D103:D106"/>
-    <mergeCell ref="E103:E106"/>
-    <mergeCell ref="A107:A110"/>
-    <mergeCell ref="B107:B110"/>
-    <mergeCell ref="D107:D110"/>
-    <mergeCell ref="E107:E110"/>
-    <mergeCell ref="D97:D99"/>
-    <mergeCell ref="E97:E99"/>
-    <mergeCell ref="A101:A102"/>
-    <mergeCell ref="B101:B102"/>
-    <mergeCell ref="D101:D102"/>
-    <mergeCell ref="E101:E102"/>
-    <mergeCell ref="D81:D87"/>
-    <mergeCell ref="E81:E87"/>
-    <mergeCell ref="A90:A96"/>
-    <mergeCell ref="B90:B96"/>
-    <mergeCell ref="D90:D96"/>
-    <mergeCell ref="E90:E96"/>
-    <mergeCell ref="D68:D77"/>
-    <mergeCell ref="E68:E77"/>
-    <mergeCell ref="A78:A79"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="D78:D79"/>
-    <mergeCell ref="E78:E79"/>
-    <mergeCell ref="A59:A67"/>
-    <mergeCell ref="B59:B67"/>
-    <mergeCell ref="D59:D67"/>
-    <mergeCell ref="E59:E67"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="D10:D14"/>
+    <mergeCell ref="E10:E14"/>
+    <mergeCell ref="A195:A198"/>
+    <mergeCell ref="B195:B198"/>
+    <mergeCell ref="D195:D198"/>
+    <mergeCell ref="E195:E198"/>
+    <mergeCell ref="A199:A201"/>
+    <mergeCell ref="B199:B201"/>
+    <mergeCell ref="D199:D201"/>
+    <mergeCell ref="E199:E201"/>
+    <mergeCell ref="D29:D35"/>
+    <mergeCell ref="E29:E35"/>
+    <mergeCell ref="A38:A42"/>
+    <mergeCell ref="B38:B42"/>
+    <mergeCell ref="D38:D42"/>
+    <mergeCell ref="E38:E42"/>
+    <mergeCell ref="D16:D25"/>
+    <mergeCell ref="E16:E25"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="D26:D28"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="D53:D58"/>
+    <mergeCell ref="E53:E58"/>
     <mergeCell ref="A4:A8"/>
     <mergeCell ref="B4:B8"/>
     <mergeCell ref="D4:D8"/>
@@ -14824,30 +14755,102 @@
     <mergeCell ref="B29:B35"/>
     <mergeCell ref="A16:A25"/>
     <mergeCell ref="B16:B25"/>
-    <mergeCell ref="D10:D14"/>
-    <mergeCell ref="E10:E14"/>
-    <mergeCell ref="A195:A198"/>
-    <mergeCell ref="B195:B198"/>
-    <mergeCell ref="D195:D198"/>
-    <mergeCell ref="E195:E198"/>
-    <mergeCell ref="A199:A201"/>
-    <mergeCell ref="B199:B201"/>
-    <mergeCell ref="D199:D201"/>
-    <mergeCell ref="E199:E201"/>
-    <mergeCell ref="D29:D35"/>
-    <mergeCell ref="E29:E35"/>
-    <mergeCell ref="A38:A42"/>
-    <mergeCell ref="B38:B42"/>
-    <mergeCell ref="D38:D42"/>
-    <mergeCell ref="E38:E42"/>
-    <mergeCell ref="D16:D25"/>
-    <mergeCell ref="E16:E25"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="D26:D28"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="D53:D58"/>
-    <mergeCell ref="E53:E58"/>
+    <mergeCell ref="A59:A67"/>
+    <mergeCell ref="B59:B67"/>
+    <mergeCell ref="D59:D67"/>
+    <mergeCell ref="E59:E67"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="D81:D87"/>
+    <mergeCell ref="E81:E87"/>
+    <mergeCell ref="A90:A96"/>
+    <mergeCell ref="B90:B96"/>
+    <mergeCell ref="D90:D96"/>
+    <mergeCell ref="E90:E96"/>
+    <mergeCell ref="D68:D77"/>
+    <mergeCell ref="E68:E77"/>
+    <mergeCell ref="A78:A79"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="D78:D79"/>
+    <mergeCell ref="E78:E79"/>
+    <mergeCell ref="A103:A106"/>
+    <mergeCell ref="B103:B106"/>
+    <mergeCell ref="D103:D106"/>
+    <mergeCell ref="E103:E106"/>
+    <mergeCell ref="A107:A110"/>
+    <mergeCell ref="B107:B110"/>
+    <mergeCell ref="D107:D110"/>
+    <mergeCell ref="E107:E110"/>
+    <mergeCell ref="D97:D99"/>
+    <mergeCell ref="E97:E99"/>
+    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="B101:B102"/>
+    <mergeCell ref="D101:D102"/>
+    <mergeCell ref="E101:E102"/>
+    <mergeCell ref="D125:D127"/>
+    <mergeCell ref="E125:E127"/>
+    <mergeCell ref="A132:A133"/>
+    <mergeCell ref="B132:B133"/>
+    <mergeCell ref="D132:D133"/>
+    <mergeCell ref="E132:E133"/>
+    <mergeCell ref="A111:A112"/>
+    <mergeCell ref="B111:B112"/>
+    <mergeCell ref="D111:D112"/>
+    <mergeCell ref="E111:E112"/>
+    <mergeCell ref="A115:A123"/>
+    <mergeCell ref="B115:B123"/>
+    <mergeCell ref="D115:D123"/>
+    <mergeCell ref="E115:E123"/>
+    <mergeCell ref="A145:A149"/>
+    <mergeCell ref="B145:B149"/>
+    <mergeCell ref="D145:D149"/>
+    <mergeCell ref="E145:E149"/>
+    <mergeCell ref="A151:A153"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="D151:D153"/>
+    <mergeCell ref="E151:E153"/>
+    <mergeCell ref="D139:D141"/>
+    <mergeCell ref="E139:E141"/>
+    <mergeCell ref="A142:A143"/>
+    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="D142:D143"/>
+    <mergeCell ref="E142:E143"/>
+    <mergeCell ref="A168:A170"/>
+    <mergeCell ref="B168:B170"/>
+    <mergeCell ref="D168:D170"/>
+    <mergeCell ref="E168:E170"/>
+    <mergeCell ref="A171:A175"/>
+    <mergeCell ref="B171:B175"/>
+    <mergeCell ref="D171:D175"/>
+    <mergeCell ref="E171:E175"/>
+    <mergeCell ref="A154:A161"/>
+    <mergeCell ref="B154:B161"/>
+    <mergeCell ref="D154:D161"/>
+    <mergeCell ref="E154:E161"/>
+    <mergeCell ref="A163:A165"/>
+    <mergeCell ref="B163:B165"/>
+    <mergeCell ref="D163:D165"/>
+    <mergeCell ref="E163:E165"/>
+    <mergeCell ref="A182:A183"/>
+    <mergeCell ref="B182:B183"/>
+    <mergeCell ref="D182:D183"/>
+    <mergeCell ref="E182:E183"/>
+    <mergeCell ref="A185:A191"/>
+    <mergeCell ref="B185:B191"/>
+    <mergeCell ref="D185:D191"/>
+    <mergeCell ref="E185:E191"/>
+    <mergeCell ref="A176:A177"/>
+    <mergeCell ref="B176:B177"/>
+    <mergeCell ref="D176:D177"/>
+    <mergeCell ref="E176:E177"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="E178:E181"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14855,7 +14858,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC4CFA97-D216-4292-8965-1641300B15B3}">
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E132"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.08984375" style="3" bestFit="1" customWidth="1"/>
@@ -16477,8 +16480,101 @@
         <v>468</v>
       </c>
     </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A132" s="2">
+        <v>55</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>1259</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>839</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>840</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="84">
+    <mergeCell ref="A123:A130"/>
+    <mergeCell ref="B123:B130"/>
+    <mergeCell ref="D123:D130"/>
+    <mergeCell ref="E123:E130"/>
+    <mergeCell ref="A105:A119"/>
+    <mergeCell ref="B105:B119"/>
+    <mergeCell ref="D105:D119"/>
+    <mergeCell ref="E105:E119"/>
+    <mergeCell ref="A121:A122"/>
+    <mergeCell ref="B121:B122"/>
+    <mergeCell ref="D121:D122"/>
+    <mergeCell ref="E121:E122"/>
+    <mergeCell ref="A100:A101"/>
+    <mergeCell ref="B100:B101"/>
+    <mergeCell ref="D100:D101"/>
+    <mergeCell ref="E100:E101"/>
+    <mergeCell ref="A102:A103"/>
+    <mergeCell ref="B102:B103"/>
+    <mergeCell ref="D102:D103"/>
+    <mergeCell ref="E102:E103"/>
+    <mergeCell ref="A84:A94"/>
+    <mergeCell ref="B84:B94"/>
+    <mergeCell ref="D84:D94"/>
+    <mergeCell ref="E84:E94"/>
+    <mergeCell ref="A95:A98"/>
+    <mergeCell ref="B95:B98"/>
+    <mergeCell ref="D95:D98"/>
+    <mergeCell ref="E95:E98"/>
+    <mergeCell ref="A70:A72"/>
+    <mergeCell ref="B70:B72"/>
+    <mergeCell ref="D70:D72"/>
+    <mergeCell ref="E70:E72"/>
+    <mergeCell ref="A74:A79"/>
+    <mergeCell ref="B74:B79"/>
+    <mergeCell ref="D74:D79"/>
+    <mergeCell ref="E74:E79"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="E68:E69"/>
+    <mergeCell ref="A64:A65"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="A51:A55"/>
+    <mergeCell ref="B51:B55"/>
+    <mergeCell ref="D51:D55"/>
+    <mergeCell ref="E51:E55"/>
+    <mergeCell ref="A57:A61"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="D57:D61"/>
+    <mergeCell ref="E57:E61"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="A46:A48"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="D30:D32"/>
+    <mergeCell ref="E30:E32"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="D33:D36"/>
+    <mergeCell ref="E33:E36"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="A25:A28"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="D25:D28"/>
+    <mergeCell ref="E25:E28"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
     <mergeCell ref="D5:D7"/>
     <mergeCell ref="E5:E7"/>
     <mergeCell ref="A11:A19"/>
@@ -16487,82 +16583,6 @@
     <mergeCell ref="E11:E19"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="B5:B7"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="A25:A28"/>
-    <mergeCell ref="B25:B28"/>
-    <mergeCell ref="D25:D28"/>
-    <mergeCell ref="E25:E28"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="D30:D32"/>
-    <mergeCell ref="E30:E32"/>
-    <mergeCell ref="A33:A36"/>
-    <mergeCell ref="B33:B36"/>
-    <mergeCell ref="D33:D36"/>
-    <mergeCell ref="E33:E36"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="D39:D41"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="A46:A48"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="A51:A55"/>
-    <mergeCell ref="B51:B55"/>
-    <mergeCell ref="D51:D55"/>
-    <mergeCell ref="E51:E55"/>
-    <mergeCell ref="A57:A61"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="D57:D61"/>
-    <mergeCell ref="E57:E61"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="E68:E69"/>
-    <mergeCell ref="A64:A65"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="E64:E65"/>
-    <mergeCell ref="A70:A72"/>
-    <mergeCell ref="B70:B72"/>
-    <mergeCell ref="D70:D72"/>
-    <mergeCell ref="E70:E72"/>
-    <mergeCell ref="A74:A79"/>
-    <mergeCell ref="B74:B79"/>
-    <mergeCell ref="D74:D79"/>
-    <mergeCell ref="E74:E79"/>
-    <mergeCell ref="A84:A94"/>
-    <mergeCell ref="B84:B94"/>
-    <mergeCell ref="D84:D94"/>
-    <mergeCell ref="E84:E94"/>
-    <mergeCell ref="A95:A98"/>
-    <mergeCell ref="B95:B98"/>
-    <mergeCell ref="D95:D98"/>
-    <mergeCell ref="E95:E98"/>
-    <mergeCell ref="A100:A101"/>
-    <mergeCell ref="B100:B101"/>
-    <mergeCell ref="D100:D101"/>
-    <mergeCell ref="E100:E101"/>
-    <mergeCell ref="A102:A103"/>
-    <mergeCell ref="B102:B103"/>
-    <mergeCell ref="D102:D103"/>
-    <mergeCell ref="E102:E103"/>
-    <mergeCell ref="A105:A119"/>
-    <mergeCell ref="B105:B119"/>
-    <mergeCell ref="D105:D119"/>
-    <mergeCell ref="E105:E119"/>
-    <mergeCell ref="A121:A122"/>
-    <mergeCell ref="B121:B122"/>
-    <mergeCell ref="D121:D122"/>
-    <mergeCell ref="E121:E122"/>
-    <mergeCell ref="A123:A130"/>
-    <mergeCell ref="B123:B130"/>
-    <mergeCell ref="D123:D130"/>
-    <mergeCell ref="E123:E130"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Assiut Motorsport team member
</commit_message>
<xml_diff>
--- a/Registration.xlsx
+++ b/Registration.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tsamak\Workspace\AutoDRIVE-RoboRacer-Sim-Racing-Participation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF75D124-B283-410B-8FD6-F08DB19AD05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{407E20E1-20F5-488C-AC3B-0F7A6B228563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="5" xr2:uid="{5D9342A3-8B90-4963-824C-8C358DE1DB7F}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1984" uniqueCount="1260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1985" uniqueCount="1261">
   <si>
     <t>SAGOL</t>
   </si>
@@ -3821,6 +3821,9 @@
   </si>
   <si>
     <t>FEBAuto</t>
+  </si>
+  <si>
+    <t>Abdulrahman Yasser Fouad</t>
   </si>
 </sst>
 </file>
@@ -3919,7 +3922,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -3941,6 +3944,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6200,37 +6206,85 @@
     </row>
   </sheetData>
   <mergeCells count="124">
-    <mergeCell ref="D27:D31"/>
-    <mergeCell ref="D21:D24"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="D6:D14"/>
-    <mergeCell ref="D81:D82"/>
-    <mergeCell ref="D77:D78"/>
-    <mergeCell ref="D71:D76"/>
-    <mergeCell ref="D67:D70"/>
-    <mergeCell ref="D59:D65"/>
-    <mergeCell ref="D55:D56"/>
-    <mergeCell ref="D50:D54"/>
-    <mergeCell ref="D35:D46"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="D103:D105"/>
-    <mergeCell ref="D99:D102"/>
-    <mergeCell ref="D111:D116"/>
-    <mergeCell ref="D108:D110"/>
-    <mergeCell ref="D106:D107"/>
-    <mergeCell ref="D117:D118"/>
-    <mergeCell ref="D95:D97"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="D84:D89"/>
-    <mergeCell ref="D154:D158"/>
-    <mergeCell ref="D159:D161"/>
-    <mergeCell ref="D124:D131"/>
-    <mergeCell ref="D122:D123"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="D135:D137"/>
-    <mergeCell ref="D132:D134"/>
-    <mergeCell ref="D149:D152"/>
-    <mergeCell ref="D142:D148"/>
+    <mergeCell ref="E159:E161"/>
+    <mergeCell ref="E135:E137"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="E142:E148"/>
+    <mergeCell ref="E149:E152"/>
+    <mergeCell ref="E154:E158"/>
+    <mergeCell ref="E111:E116"/>
+    <mergeCell ref="E117:E118"/>
+    <mergeCell ref="E122:E123"/>
+    <mergeCell ref="E124:E131"/>
+    <mergeCell ref="E132:E134"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="E99:E102"/>
+    <mergeCell ref="E103:E105"/>
+    <mergeCell ref="E106:E107"/>
+    <mergeCell ref="E108:E110"/>
+    <mergeCell ref="E71:E76"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="E84:E89"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="E35:E46"/>
+    <mergeCell ref="E50:E54"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E59:E65"/>
+    <mergeCell ref="E67:E70"/>
+    <mergeCell ref="E6:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E21:E24"/>
+    <mergeCell ref="E27:E31"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="A27:A31"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A35:A46"/>
+    <mergeCell ref="B35:B46"/>
+    <mergeCell ref="A6:A14"/>
+    <mergeCell ref="B6:B14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A71:A76"/>
+    <mergeCell ref="B71:B76"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="A50:A54"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="A59:A65"/>
+    <mergeCell ref="B59:B65"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="A99:A102"/>
+    <mergeCell ref="B99:B102"/>
+    <mergeCell ref="A103:A105"/>
+    <mergeCell ref="B103:B105"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="A84:A89"/>
+    <mergeCell ref="B84:B89"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A117:A118"/>
+    <mergeCell ref="B117:B118"/>
+    <mergeCell ref="A122:A123"/>
+    <mergeCell ref="B122:B123"/>
+    <mergeCell ref="A124:A131"/>
+    <mergeCell ref="B124:B131"/>
+    <mergeCell ref="A106:A107"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="A108:A110"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="A111:A116"/>
+    <mergeCell ref="B111:B116"/>
     <mergeCell ref="A142:A148"/>
     <mergeCell ref="B142:B148"/>
     <mergeCell ref="A159:A161"/>
@@ -6245,85 +6299,37 @@
     <mergeCell ref="B135:B137"/>
     <mergeCell ref="A138:A141"/>
     <mergeCell ref="B138:B141"/>
-    <mergeCell ref="A117:A118"/>
-    <mergeCell ref="B117:B118"/>
-    <mergeCell ref="A122:A123"/>
-    <mergeCell ref="B122:B123"/>
-    <mergeCell ref="A124:A131"/>
-    <mergeCell ref="B124:B131"/>
-    <mergeCell ref="A106:A107"/>
-    <mergeCell ref="B106:B107"/>
-    <mergeCell ref="A108:A110"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="A111:A116"/>
-    <mergeCell ref="B111:B116"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="A99:A102"/>
-    <mergeCell ref="B99:B102"/>
-    <mergeCell ref="A103:A105"/>
-    <mergeCell ref="B103:B105"/>
-    <mergeCell ref="A81:A82"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="A84:A89"/>
-    <mergeCell ref="B84:B89"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A71:A76"/>
-    <mergeCell ref="B71:B76"/>
-    <mergeCell ref="A77:A78"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="A50:A54"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="A59:A65"/>
-    <mergeCell ref="B59:B65"/>
-    <mergeCell ref="A27:A31"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A35:A46"/>
-    <mergeCell ref="B35:B46"/>
-    <mergeCell ref="A6:A14"/>
-    <mergeCell ref="B6:B14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="B21:B24"/>
-    <mergeCell ref="E35:E46"/>
-    <mergeCell ref="E50:E54"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E59:E65"/>
-    <mergeCell ref="E67:E70"/>
-    <mergeCell ref="E6:E14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E21:E24"/>
-    <mergeCell ref="E27:E31"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="E99:E102"/>
-    <mergeCell ref="E103:E105"/>
-    <mergeCell ref="E106:E107"/>
-    <mergeCell ref="E108:E110"/>
-    <mergeCell ref="E71:E76"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="E84:E89"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="E159:E161"/>
-    <mergeCell ref="E135:E137"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="E142:E148"/>
-    <mergeCell ref="E149:E152"/>
-    <mergeCell ref="E154:E158"/>
-    <mergeCell ref="E111:E116"/>
-    <mergeCell ref="E117:E118"/>
-    <mergeCell ref="E122:E123"/>
-    <mergeCell ref="E124:E131"/>
-    <mergeCell ref="E132:E134"/>
+    <mergeCell ref="D154:D158"/>
+    <mergeCell ref="D159:D161"/>
+    <mergeCell ref="D124:D131"/>
+    <mergeCell ref="D122:D123"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="D135:D137"/>
+    <mergeCell ref="D132:D134"/>
+    <mergeCell ref="D149:D152"/>
+    <mergeCell ref="D142:D148"/>
+    <mergeCell ref="D103:D105"/>
+    <mergeCell ref="D99:D102"/>
+    <mergeCell ref="D111:D116"/>
+    <mergeCell ref="D108:D110"/>
+    <mergeCell ref="D106:D107"/>
+    <mergeCell ref="D117:D118"/>
+    <mergeCell ref="D95:D97"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="D84:D89"/>
+    <mergeCell ref="D27:D31"/>
+    <mergeCell ref="D21:D24"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="D6:D14"/>
+    <mergeCell ref="D81:D82"/>
+    <mergeCell ref="D77:D78"/>
+    <mergeCell ref="D71:D76"/>
+    <mergeCell ref="D67:D70"/>
+    <mergeCell ref="D59:D65"/>
+    <mergeCell ref="D55:D56"/>
+    <mergeCell ref="D50:D54"/>
+    <mergeCell ref="D35:D46"/>
+    <mergeCell ref="D33:D34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -8295,6 +8301,126 @@
     </row>
   </sheetData>
   <mergeCells count="144">
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="E170:E171"/>
+    <mergeCell ref="E102:E111"/>
+    <mergeCell ref="E112:E116"/>
+    <mergeCell ref="E117:E122"/>
+    <mergeCell ref="E123:E129"/>
+    <mergeCell ref="E130:E141"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="E150:E151"/>
+    <mergeCell ref="E152:E156"/>
+    <mergeCell ref="E75:E78"/>
+    <mergeCell ref="E80:E82"/>
+    <mergeCell ref="E84:E85"/>
+    <mergeCell ref="E86:E91"/>
+    <mergeCell ref="E92:E94"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="E157:E159"/>
+    <mergeCell ref="E160:E164"/>
+    <mergeCell ref="E38:E45"/>
+    <mergeCell ref="E46:E51"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="E62:E64"/>
+    <mergeCell ref="E66:E67"/>
+    <mergeCell ref="B8:B15"/>
+    <mergeCell ref="D8:D15"/>
+    <mergeCell ref="E68:E69"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="E8:E15"/>
+    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="E26:E30"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="E33:E37"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="D4:D7"/>
+    <mergeCell ref="A8:A15"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="B33:B37"/>
+    <mergeCell ref="D33:D37"/>
+    <mergeCell ref="A38:A45"/>
+    <mergeCell ref="B38:B45"/>
+    <mergeCell ref="D38:D45"/>
+    <mergeCell ref="A26:A30"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="D26:D30"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="D16:D19"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="D150:D151"/>
+    <mergeCell ref="B152:B156"/>
+    <mergeCell ref="D152:D156"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="B117:B122"/>
+    <mergeCell ref="D117:D122"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="B102:B111"/>
+    <mergeCell ref="D102:D111"/>
+    <mergeCell ref="B123:B129"/>
+    <mergeCell ref="D123:D129"/>
+    <mergeCell ref="B130:B141"/>
+    <mergeCell ref="D130:D141"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="B75:B78"/>
+    <mergeCell ref="B80:B82"/>
+    <mergeCell ref="D80:D82"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="D84:D85"/>
+    <mergeCell ref="B112:B116"/>
+    <mergeCell ref="D112:D116"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="D95:D97"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B86:B91"/>
+    <mergeCell ref="D86:D91"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="A170:A171"/>
+    <mergeCell ref="B170:B171"/>
+    <mergeCell ref="D170:D171"/>
+    <mergeCell ref="A160:A164"/>
+    <mergeCell ref="B160:B164"/>
+    <mergeCell ref="D160:D164"/>
+    <mergeCell ref="A157:A159"/>
+    <mergeCell ref="B157:B159"/>
+    <mergeCell ref="D157:D159"/>
+    <mergeCell ref="A152:A156"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="A150:A151"/>
+    <mergeCell ref="A123:A129"/>
+    <mergeCell ref="A130:A141"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="A75:A78"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="A112:A116"/>
+    <mergeCell ref="A86:A91"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="A102:A111"/>
+    <mergeCell ref="A117:A122"/>
+    <mergeCell ref="A98:A101"/>
     <mergeCell ref="A62:A64"/>
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="A16:A19"/>
@@ -8319,126 +8445,6 @@
     <mergeCell ref="D62:D64"/>
     <mergeCell ref="B66:B67"/>
     <mergeCell ref="D66:D67"/>
-    <mergeCell ref="A152:A156"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="A150:A151"/>
-    <mergeCell ref="A123:A129"/>
-    <mergeCell ref="A130:A141"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A75:A78"/>
-    <mergeCell ref="A66:A67"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="A170:A171"/>
-    <mergeCell ref="B170:B171"/>
-    <mergeCell ref="D170:D171"/>
-    <mergeCell ref="A160:A164"/>
-    <mergeCell ref="B160:B164"/>
-    <mergeCell ref="D160:D164"/>
-    <mergeCell ref="A157:A159"/>
-    <mergeCell ref="B157:B159"/>
-    <mergeCell ref="D157:D159"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="B75:B78"/>
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="D80:D82"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="D84:D85"/>
-    <mergeCell ref="B112:B116"/>
-    <mergeCell ref="D112:D116"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="D95:D97"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B86:B91"/>
-    <mergeCell ref="D86:D91"/>
-    <mergeCell ref="A112:A116"/>
-    <mergeCell ref="A86:A91"/>
-    <mergeCell ref="A84:A85"/>
-    <mergeCell ref="A102:A111"/>
-    <mergeCell ref="A117:A122"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="D150:D151"/>
-    <mergeCell ref="B152:B156"/>
-    <mergeCell ref="D152:D156"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="B117:B122"/>
-    <mergeCell ref="D117:D122"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="B102:B111"/>
-    <mergeCell ref="D102:D111"/>
-    <mergeCell ref="B123:B129"/>
-    <mergeCell ref="D123:D129"/>
-    <mergeCell ref="B130:B141"/>
-    <mergeCell ref="D130:D141"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="D4:D7"/>
-    <mergeCell ref="A8:A15"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="A33:A37"/>
-    <mergeCell ref="B33:B37"/>
-    <mergeCell ref="D33:D37"/>
-    <mergeCell ref="A38:A45"/>
-    <mergeCell ref="B38:B45"/>
-    <mergeCell ref="D38:D45"/>
-    <mergeCell ref="A26:A30"/>
-    <mergeCell ref="B26:B30"/>
-    <mergeCell ref="D26:D30"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="D16:D19"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E4:E7"/>
-    <mergeCell ref="E8:E15"/>
-    <mergeCell ref="E16:E19"/>
-    <mergeCell ref="E21:E23"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="E26:E30"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="E33:E37"/>
-    <mergeCell ref="E38:E45"/>
-    <mergeCell ref="E46:E51"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="E62:E64"/>
-    <mergeCell ref="E66:E67"/>
-    <mergeCell ref="B8:B15"/>
-    <mergeCell ref="D8:D15"/>
-    <mergeCell ref="E68:E69"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="E75:E78"/>
-    <mergeCell ref="E80:E82"/>
-    <mergeCell ref="E84:E85"/>
-    <mergeCell ref="E86:E91"/>
-    <mergeCell ref="E92:E94"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="E157:E159"/>
-    <mergeCell ref="E160:E164"/>
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="E170:E171"/>
-    <mergeCell ref="E102:E111"/>
-    <mergeCell ref="E112:E116"/>
-    <mergeCell ref="E117:E122"/>
-    <mergeCell ref="E123:E129"/>
-    <mergeCell ref="E130:E141"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="E150:E151"/>
-    <mergeCell ref="E152:E156"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10273,29 +10279,90 @@
     </row>
   </sheetData>
   <mergeCells count="132">
-    <mergeCell ref="D48:D50"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="A129:A130"/>
-    <mergeCell ref="B129:B130"/>
-    <mergeCell ref="D129:D130"/>
-    <mergeCell ref="E129:E130"/>
-    <mergeCell ref="A87:A89"/>
-    <mergeCell ref="B87:B89"/>
-    <mergeCell ref="D87:D89"/>
-    <mergeCell ref="A92:A97"/>
-    <mergeCell ref="B92:B97"/>
-    <mergeCell ref="D92:D97"/>
-    <mergeCell ref="E92:E97"/>
-    <mergeCell ref="A99:A109"/>
-    <mergeCell ref="B99:B109"/>
-    <mergeCell ref="D99:D109"/>
-    <mergeCell ref="E99:E109"/>
-    <mergeCell ref="A76:A80"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="D76:D80"/>
-    <mergeCell ref="E76:E80"/>
-    <mergeCell ref="A65:A71"/>
-    <mergeCell ref="B65:B71"/>
+    <mergeCell ref="A145:A147"/>
+    <mergeCell ref="B145:B147"/>
+    <mergeCell ref="D145:D147"/>
+    <mergeCell ref="E145:E147"/>
+    <mergeCell ref="A149:A150"/>
+    <mergeCell ref="B149:B150"/>
+    <mergeCell ref="D149:D150"/>
+    <mergeCell ref="E149:E150"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="D131:D133"/>
+    <mergeCell ref="E131:E133"/>
+    <mergeCell ref="A135:A138"/>
+    <mergeCell ref="B135:B138"/>
+    <mergeCell ref="D135:D138"/>
+    <mergeCell ref="E135:E138"/>
+    <mergeCell ref="A139:A141"/>
+    <mergeCell ref="B139:B141"/>
+    <mergeCell ref="D139:D141"/>
+    <mergeCell ref="E139:E141"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="D114:D117"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="A118:A127"/>
+    <mergeCell ref="B118:B127"/>
+    <mergeCell ref="D118:D127"/>
+    <mergeCell ref="E118:E127"/>
+    <mergeCell ref="A81:A85"/>
+    <mergeCell ref="B81:B85"/>
+    <mergeCell ref="D81:D85"/>
+    <mergeCell ref="E81:E85"/>
+    <mergeCell ref="E87:E89"/>
+    <mergeCell ref="A90:A91"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="D90:D91"/>
+    <mergeCell ref="E90:E91"/>
+    <mergeCell ref="D1:D4"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E1:E4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="D73:D75"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="E57:E59"/>
+    <mergeCell ref="A60:A64"/>
+    <mergeCell ref="B60:B64"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="D51:D53"/>
+    <mergeCell ref="E51:E53"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="E42:E46"/>
+    <mergeCell ref="E73:E75"/>
+    <mergeCell ref="A73:A75"/>
+    <mergeCell ref="B73:B75"/>
+    <mergeCell ref="E65:E71"/>
+    <mergeCell ref="A48:A50"/>
+    <mergeCell ref="B48:B50"/>
     <mergeCell ref="D29:D31"/>
     <mergeCell ref="E29:E31"/>
     <mergeCell ref="A20:A22"/>
@@ -10320,91 +10387,30 @@
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="B29:B31"/>
     <mergeCell ref="B1:B4"/>
+    <mergeCell ref="D48:D50"/>
+    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="A129:A130"/>
+    <mergeCell ref="B129:B130"/>
+    <mergeCell ref="D129:D130"/>
+    <mergeCell ref="E129:E130"/>
+    <mergeCell ref="A87:A89"/>
+    <mergeCell ref="B87:B89"/>
+    <mergeCell ref="D87:D89"/>
+    <mergeCell ref="A92:A97"/>
+    <mergeCell ref="B92:B97"/>
+    <mergeCell ref="D92:D97"/>
+    <mergeCell ref="E92:E97"/>
+    <mergeCell ref="A99:A109"/>
+    <mergeCell ref="B99:B109"/>
+    <mergeCell ref="D99:D109"/>
+    <mergeCell ref="E99:E109"/>
+    <mergeCell ref="A76:A80"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="D76:D80"/>
+    <mergeCell ref="E76:E80"/>
+    <mergeCell ref="A65:A71"/>
+    <mergeCell ref="B65:B71"/>
     <mergeCell ref="D65:D71"/>
-    <mergeCell ref="D73:D75"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="E57:E59"/>
-    <mergeCell ref="A60:A64"/>
-    <mergeCell ref="B60:B64"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="B51:B53"/>
-    <mergeCell ref="D51:D53"/>
-    <mergeCell ref="E51:E53"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="E42:E46"/>
-    <mergeCell ref="E73:E75"/>
-    <mergeCell ref="A73:A75"/>
-    <mergeCell ref="B73:B75"/>
-    <mergeCell ref="E65:E71"/>
-    <mergeCell ref="A48:A50"/>
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="D1:D4"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E1:E4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="A81:A85"/>
-    <mergeCell ref="B81:B85"/>
-    <mergeCell ref="D81:D85"/>
-    <mergeCell ref="E81:E85"/>
-    <mergeCell ref="E87:E89"/>
-    <mergeCell ref="A90:A91"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="D90:D91"/>
-    <mergeCell ref="E90:E91"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="D114:D117"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="A118:A127"/>
-    <mergeCell ref="B118:B127"/>
-    <mergeCell ref="D118:D127"/>
-    <mergeCell ref="E118:E127"/>
-    <mergeCell ref="A145:A147"/>
-    <mergeCell ref="B145:B147"/>
-    <mergeCell ref="D145:D147"/>
-    <mergeCell ref="E145:E147"/>
-    <mergeCell ref="A149:A150"/>
-    <mergeCell ref="B149:B150"/>
-    <mergeCell ref="D149:D150"/>
-    <mergeCell ref="E149:E150"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="D131:D133"/>
-    <mergeCell ref="E131:E133"/>
-    <mergeCell ref="A135:A138"/>
-    <mergeCell ref="B135:B138"/>
-    <mergeCell ref="D135:D138"/>
-    <mergeCell ref="E135:E138"/>
-    <mergeCell ref="A139:A141"/>
-    <mergeCell ref="B139:B141"/>
-    <mergeCell ref="D139:D141"/>
-    <mergeCell ref="E139:E141"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -12203,57 +12209,31 @@
     </row>
   </sheetData>
   <mergeCells count="92">
-    <mergeCell ref="A90:A95"/>
-    <mergeCell ref="A96:A100"/>
-    <mergeCell ref="A57:A61"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A42:A47"/>
-    <mergeCell ref="A83:A89"/>
-    <mergeCell ref="A154:A156"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="D154:D156"/>
-    <mergeCell ref="E154:E156"/>
-    <mergeCell ref="A157:A158"/>
-    <mergeCell ref="B157:B158"/>
-    <mergeCell ref="D157:D158"/>
-    <mergeCell ref="E157:E158"/>
-    <mergeCell ref="D90:D95"/>
-    <mergeCell ref="E90:E95"/>
-    <mergeCell ref="B96:B100"/>
-    <mergeCell ref="D96:D100"/>
-    <mergeCell ref="E96:E100"/>
-    <mergeCell ref="B90:B95"/>
-    <mergeCell ref="D49:D54"/>
-    <mergeCell ref="E49:E54"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="D57:D61"/>
-    <mergeCell ref="E57:E61"/>
-    <mergeCell ref="B49:B54"/>
-    <mergeCell ref="D39:D41"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="B42:B47"/>
-    <mergeCell ref="D42:D47"/>
-    <mergeCell ref="E42:E47"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="A15:A24"/>
-    <mergeCell ref="B15:B24"/>
-    <mergeCell ref="D15:D24"/>
-    <mergeCell ref="E15:E24"/>
-    <mergeCell ref="D28:D31"/>
-    <mergeCell ref="E28:E31"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="D5:D8"/>
-    <mergeCell ref="E5:E8"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="B9:B13"/>
-    <mergeCell ref="D9:D13"/>
-    <mergeCell ref="E9:E13"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="D36:D38"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="B32:B35"/>
+    <mergeCell ref="D32:D35"/>
+    <mergeCell ref="E32:E35"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D83:D89"/>
+    <mergeCell ref="E83:E89"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="B62:B67"/>
+    <mergeCell ref="D62:D67"/>
+    <mergeCell ref="E62:E67"/>
+    <mergeCell ref="A69:A72"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="D69:D72"/>
+    <mergeCell ref="E69:E72"/>
+    <mergeCell ref="A73:A82"/>
+    <mergeCell ref="B73:B82"/>
+    <mergeCell ref="D73:D82"/>
+    <mergeCell ref="E73:E82"/>
     <mergeCell ref="A129:A151"/>
     <mergeCell ref="B129:B151"/>
     <mergeCell ref="D129:D151"/>
@@ -12270,31 +12250,57 @@
     <mergeCell ref="B126:B128"/>
     <mergeCell ref="D126:D128"/>
     <mergeCell ref="E126:E128"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D83:D89"/>
-    <mergeCell ref="E83:E89"/>
-    <mergeCell ref="A62:A67"/>
-    <mergeCell ref="B62:B67"/>
-    <mergeCell ref="D62:D67"/>
-    <mergeCell ref="E62:E67"/>
-    <mergeCell ref="A69:A72"/>
-    <mergeCell ref="B69:B72"/>
-    <mergeCell ref="D69:D72"/>
-    <mergeCell ref="E69:E72"/>
-    <mergeCell ref="A73:A82"/>
-    <mergeCell ref="B73:B82"/>
-    <mergeCell ref="D73:D82"/>
-    <mergeCell ref="E73:E82"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="D36:D38"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="B28:B31"/>
-    <mergeCell ref="A32:A35"/>
-    <mergeCell ref="B32:B35"/>
-    <mergeCell ref="D32:D35"/>
-    <mergeCell ref="E32:E35"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="E5:E8"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="B9:B13"/>
+    <mergeCell ref="D9:D13"/>
+    <mergeCell ref="E9:E13"/>
+    <mergeCell ref="A15:A24"/>
+    <mergeCell ref="B15:B24"/>
+    <mergeCell ref="D15:D24"/>
+    <mergeCell ref="E15:E24"/>
+    <mergeCell ref="D28:D31"/>
+    <mergeCell ref="E28:E31"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="B42:B47"/>
+    <mergeCell ref="D42:D47"/>
+    <mergeCell ref="E42:E47"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="D49:D54"/>
+    <mergeCell ref="E49:E54"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="D57:D61"/>
+    <mergeCell ref="E57:E61"/>
+    <mergeCell ref="B49:B54"/>
+    <mergeCell ref="D90:D95"/>
+    <mergeCell ref="E90:E95"/>
+    <mergeCell ref="B96:B100"/>
+    <mergeCell ref="D96:D100"/>
+    <mergeCell ref="E96:E100"/>
+    <mergeCell ref="B90:B95"/>
+    <mergeCell ref="A154:A156"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="D154:D156"/>
+    <mergeCell ref="E154:E156"/>
+    <mergeCell ref="A157:A158"/>
+    <mergeCell ref="B157:B158"/>
+    <mergeCell ref="D157:D158"/>
+    <mergeCell ref="E157:E158"/>
+    <mergeCell ref="A90:A95"/>
+    <mergeCell ref="A96:A100"/>
+    <mergeCell ref="A57:A61"/>
+    <mergeCell ref="A49:A54"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="A42:A47"/>
+    <mergeCell ref="A83:A89"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14707,6 +14713,126 @@
     </row>
   </sheetData>
   <mergeCells count="144">
+    <mergeCell ref="A182:A183"/>
+    <mergeCell ref="B182:B183"/>
+    <mergeCell ref="D182:D183"/>
+    <mergeCell ref="E182:E183"/>
+    <mergeCell ref="A185:A191"/>
+    <mergeCell ref="B185:B191"/>
+    <mergeCell ref="D185:D191"/>
+    <mergeCell ref="E185:E191"/>
+    <mergeCell ref="A176:A177"/>
+    <mergeCell ref="B176:B177"/>
+    <mergeCell ref="D176:D177"/>
+    <mergeCell ref="E176:E177"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="A168:A170"/>
+    <mergeCell ref="B168:B170"/>
+    <mergeCell ref="D168:D170"/>
+    <mergeCell ref="E168:E170"/>
+    <mergeCell ref="A171:A175"/>
+    <mergeCell ref="B171:B175"/>
+    <mergeCell ref="D171:D175"/>
+    <mergeCell ref="E171:E175"/>
+    <mergeCell ref="A154:A161"/>
+    <mergeCell ref="B154:B161"/>
+    <mergeCell ref="D154:D161"/>
+    <mergeCell ref="E154:E161"/>
+    <mergeCell ref="A163:A165"/>
+    <mergeCell ref="B163:B165"/>
+    <mergeCell ref="D163:D165"/>
+    <mergeCell ref="E163:E165"/>
+    <mergeCell ref="A145:A149"/>
+    <mergeCell ref="B145:B149"/>
+    <mergeCell ref="D145:D149"/>
+    <mergeCell ref="E145:E149"/>
+    <mergeCell ref="A151:A153"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="D151:D153"/>
+    <mergeCell ref="E151:E153"/>
+    <mergeCell ref="D139:D141"/>
+    <mergeCell ref="E139:E141"/>
+    <mergeCell ref="A142:A143"/>
+    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="D142:D143"/>
+    <mergeCell ref="E142:E143"/>
+    <mergeCell ref="D125:D127"/>
+    <mergeCell ref="E125:E127"/>
+    <mergeCell ref="A132:A133"/>
+    <mergeCell ref="B132:B133"/>
+    <mergeCell ref="D132:D133"/>
+    <mergeCell ref="E132:E133"/>
+    <mergeCell ref="A111:A112"/>
+    <mergeCell ref="B111:B112"/>
+    <mergeCell ref="D111:D112"/>
+    <mergeCell ref="E111:E112"/>
+    <mergeCell ref="A115:A123"/>
+    <mergeCell ref="B115:B123"/>
+    <mergeCell ref="D115:D123"/>
+    <mergeCell ref="E115:E123"/>
+    <mergeCell ref="A103:A106"/>
+    <mergeCell ref="B103:B106"/>
+    <mergeCell ref="D103:D106"/>
+    <mergeCell ref="E103:E106"/>
+    <mergeCell ref="A107:A110"/>
+    <mergeCell ref="B107:B110"/>
+    <mergeCell ref="D107:D110"/>
+    <mergeCell ref="E107:E110"/>
+    <mergeCell ref="D97:D99"/>
+    <mergeCell ref="E97:E99"/>
+    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="B101:B102"/>
+    <mergeCell ref="D101:D102"/>
+    <mergeCell ref="E101:E102"/>
+    <mergeCell ref="D81:D87"/>
+    <mergeCell ref="E81:E87"/>
+    <mergeCell ref="A90:A96"/>
+    <mergeCell ref="B90:B96"/>
+    <mergeCell ref="D90:D96"/>
+    <mergeCell ref="E90:E96"/>
+    <mergeCell ref="D68:D77"/>
+    <mergeCell ref="E68:E77"/>
+    <mergeCell ref="A78:A79"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="D78:D79"/>
+    <mergeCell ref="E78:E79"/>
+    <mergeCell ref="A59:A67"/>
+    <mergeCell ref="B59:B67"/>
+    <mergeCell ref="D59:D67"/>
+    <mergeCell ref="E59:E67"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="D4:D8"/>
+    <mergeCell ref="E4:E8"/>
+    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="A139:A141"/>
+    <mergeCell ref="B139:B141"/>
+    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="B125:B127"/>
+    <mergeCell ref="A97:A99"/>
+    <mergeCell ref="B97:B99"/>
+    <mergeCell ref="A81:A87"/>
+    <mergeCell ref="B81:B87"/>
+    <mergeCell ref="A68:A77"/>
+    <mergeCell ref="B68:B77"/>
+    <mergeCell ref="A53:A58"/>
+    <mergeCell ref="B53:B58"/>
+    <mergeCell ref="A46:A48"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="A29:A35"/>
+    <mergeCell ref="B29:B35"/>
+    <mergeCell ref="A16:A25"/>
+    <mergeCell ref="B16:B25"/>
     <mergeCell ref="D10:D14"/>
     <mergeCell ref="E10:E14"/>
     <mergeCell ref="A195:A198"/>
@@ -14731,126 +14857,6 @@
     <mergeCell ref="E26:E28"/>
     <mergeCell ref="D53:D58"/>
     <mergeCell ref="E53:E58"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="B4:B8"/>
-    <mergeCell ref="D4:D8"/>
-    <mergeCell ref="E4:E8"/>
-    <mergeCell ref="A10:A14"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="A139:A141"/>
-    <mergeCell ref="B139:B141"/>
-    <mergeCell ref="A125:A127"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="A97:A99"/>
-    <mergeCell ref="B97:B99"/>
-    <mergeCell ref="A81:A87"/>
-    <mergeCell ref="B81:B87"/>
-    <mergeCell ref="A68:A77"/>
-    <mergeCell ref="B68:B77"/>
-    <mergeCell ref="A53:A58"/>
-    <mergeCell ref="B53:B58"/>
-    <mergeCell ref="A46:A48"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="A29:A35"/>
-    <mergeCell ref="B29:B35"/>
-    <mergeCell ref="A16:A25"/>
-    <mergeCell ref="B16:B25"/>
-    <mergeCell ref="A59:A67"/>
-    <mergeCell ref="B59:B67"/>
-    <mergeCell ref="D59:D67"/>
-    <mergeCell ref="E59:E67"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="D81:D87"/>
-    <mergeCell ref="E81:E87"/>
-    <mergeCell ref="A90:A96"/>
-    <mergeCell ref="B90:B96"/>
-    <mergeCell ref="D90:D96"/>
-    <mergeCell ref="E90:E96"/>
-    <mergeCell ref="D68:D77"/>
-    <mergeCell ref="E68:E77"/>
-    <mergeCell ref="A78:A79"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="D78:D79"/>
-    <mergeCell ref="E78:E79"/>
-    <mergeCell ref="A103:A106"/>
-    <mergeCell ref="B103:B106"/>
-    <mergeCell ref="D103:D106"/>
-    <mergeCell ref="E103:E106"/>
-    <mergeCell ref="A107:A110"/>
-    <mergeCell ref="B107:B110"/>
-    <mergeCell ref="D107:D110"/>
-    <mergeCell ref="E107:E110"/>
-    <mergeCell ref="D97:D99"/>
-    <mergeCell ref="E97:E99"/>
-    <mergeCell ref="A101:A102"/>
-    <mergeCell ref="B101:B102"/>
-    <mergeCell ref="D101:D102"/>
-    <mergeCell ref="E101:E102"/>
-    <mergeCell ref="D125:D127"/>
-    <mergeCell ref="E125:E127"/>
-    <mergeCell ref="A132:A133"/>
-    <mergeCell ref="B132:B133"/>
-    <mergeCell ref="D132:D133"/>
-    <mergeCell ref="E132:E133"/>
-    <mergeCell ref="A111:A112"/>
-    <mergeCell ref="B111:B112"/>
-    <mergeCell ref="D111:D112"/>
-    <mergeCell ref="E111:E112"/>
-    <mergeCell ref="A115:A123"/>
-    <mergeCell ref="B115:B123"/>
-    <mergeCell ref="D115:D123"/>
-    <mergeCell ref="E115:E123"/>
-    <mergeCell ref="A145:A149"/>
-    <mergeCell ref="B145:B149"/>
-    <mergeCell ref="D145:D149"/>
-    <mergeCell ref="E145:E149"/>
-    <mergeCell ref="A151:A153"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="D151:D153"/>
-    <mergeCell ref="E151:E153"/>
-    <mergeCell ref="D139:D141"/>
-    <mergeCell ref="E139:E141"/>
-    <mergeCell ref="A142:A143"/>
-    <mergeCell ref="B142:B143"/>
-    <mergeCell ref="D142:D143"/>
-    <mergeCell ref="E142:E143"/>
-    <mergeCell ref="A168:A170"/>
-    <mergeCell ref="B168:B170"/>
-    <mergeCell ref="D168:D170"/>
-    <mergeCell ref="E168:E170"/>
-    <mergeCell ref="A171:A175"/>
-    <mergeCell ref="B171:B175"/>
-    <mergeCell ref="D171:D175"/>
-    <mergeCell ref="E171:E175"/>
-    <mergeCell ref="A154:A161"/>
-    <mergeCell ref="B154:B161"/>
-    <mergeCell ref="D154:D161"/>
-    <mergeCell ref="E154:E161"/>
-    <mergeCell ref="A163:A165"/>
-    <mergeCell ref="B163:B165"/>
-    <mergeCell ref="D163:D165"/>
-    <mergeCell ref="E163:E165"/>
-    <mergeCell ref="A182:A183"/>
-    <mergeCell ref="B182:B183"/>
-    <mergeCell ref="D182:D183"/>
-    <mergeCell ref="E182:E183"/>
-    <mergeCell ref="A185:A191"/>
-    <mergeCell ref="B185:B191"/>
-    <mergeCell ref="D185:D191"/>
-    <mergeCell ref="E185:E191"/>
-    <mergeCell ref="A176:A177"/>
-    <mergeCell ref="B176:B177"/>
-    <mergeCell ref="D176:D177"/>
-    <mergeCell ref="E176:E177"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="E178:E181"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14858,7 +14864,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC4CFA97-D216-4292-8965-1641300B15B3}">
-  <dimension ref="A1:E132"/>
+  <dimension ref="A1:E133"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.08984375" style="3" bestFit="1" customWidth="1"/>
@@ -16068,36 +16074,36 @@
       <c r="E94" s="4"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A95" s="4">
+      <c r="A95" s="4"/>
+      <c r="B95" s="4"/>
+      <c r="C95" s="8" t="s">
+        <v>1260</v>
+      </c>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A96" s="4">
         <v>45</v>
       </c>
-      <c r="B95" s="4" t="s">
+      <c r="B96" s="4" t="s">
         <v>1227</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="C96" s="2" t="s">
         <v>1228</v>
       </c>
-      <c r="D95" s="4" t="s">
+      <c r="D96" s="4" t="s">
         <v>1232</v>
       </c>
-      <c r="E95" s="4" t="s">
+      <c r="E96" s="4" t="s">
         <v>491</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A96" s="4"/>
-      <c r="B96" s="4"/>
-      <c r="C96" s="2" t="s">
-        <v>1229</v>
-      </c>
-      <c r="D96" s="4"/>
-      <c r="E96" s="4"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="4"/>
       <c r="B97" s="4"/>
       <c r="C97" s="2" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="D97" s="4"/>
       <c r="E97" s="4"/>
@@ -16106,128 +16112,128 @@
       <c r="A98" s="4"/>
       <c r="B98" s="4"/>
       <c r="C98" s="2" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="D98" s="4"/>
       <c r="E98" s="4"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A99" s="2">
+      <c r="A99" s="4"/>
+      <c r="B99" s="4"/>
+      <c r="C99" s="2" t="s">
+        <v>1231</v>
+      </c>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A100" s="2">
         <v>46</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="B100" s="2" t="s">
         <v>1233</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="C100" s="2" t="s">
         <v>1234</v>
       </c>
-      <c r="D99" s="2" t="s">
+      <c r="D100" s="2" t="s">
         <v>1235</v>
       </c>
-      <c r="E99" s="2" t="s">
+      <c r="E100" s="2" t="s">
         <v>486</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A100" s="4">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A101" s="4">
         <v>47</v>
       </c>
-      <c r="B100" s="4" t="s">
+      <c r="B101" s="4" t="s">
         <v>1095</v>
       </c>
-      <c r="C100" s="2" t="s">
+      <c r="C101" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D100" s="4" t="s">
+      <c r="D101" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E100" s="4" t="s">
+      <c r="E101" s="4" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A101" s="4"/>
-      <c r="B101" s="4"/>
-      <c r="C101" s="2" t="s">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A102" s="4"/>
+      <c r="B102" s="4"/>
+      <c r="C102" s="2" t="s">
         <v>1096</v>
       </c>
-      <c r="D101" s="4"/>
-      <c r="E101" s="4"/>
-    </row>
-    <row r="102" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A102" s="4">
+      <c r="D102" s="4"/>
+      <c r="E102" s="4"/>
+    </row>
+    <row r="103" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A103" s="4">
         <v>48</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B103" s="4" t="s">
         <v>1236</v>
       </c>
-      <c r="C102" s="2" t="s">
+      <c r="C103" s="2" t="s">
         <v>1237</v>
       </c>
-      <c r="D102" s="4" t="s">
+      <c r="D103" s="4" t="s">
         <v>1239</v>
       </c>
-      <c r="E102" s="4" t="s">
+      <c r="E103" s="4" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A103" s="4"/>
-      <c r="B103" s="4"/>
-      <c r="C103" s="2" t="s">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A104" s="4"/>
+      <c r="B104" s="4"/>
+      <c r="C104" s="2" t="s">
         <v>1238</v>
       </c>
-      <c r="D103" s="4"/>
-      <c r="E103" s="4"/>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A104" s="2">
+      <c r="D104" s="4"/>
+      <c r="E104" s="4"/>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A105" s="2">
         <v>49</v>
       </c>
-      <c r="B104" s="2" t="s">
+      <c r="B105" s="2" t="s">
         <v>1240</v>
       </c>
-      <c r="C104" s="2" t="s">
+      <c r="C105" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="D104" s="2" t="s">
+      <c r="D105" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E104" s="2" t="s">
+      <c r="E105" s="2" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A105" s="4">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A106" s="4">
         <v>50</v>
       </c>
-      <c r="B105" s="4" t="s">
+      <c r="B106" s="4" t="s">
         <v>420</v>
       </c>
-      <c r="C105" s="2" t="s">
+      <c r="C106" s="2" t="s">
         <v>777</v>
       </c>
-      <c r="D105" s="4" t="s">
+      <c r="D106" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="E105" s="4" t="s">
+      <c r="E106" s="4" t="s">
         <v>468</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A106" s="4"/>
-      <c r="B106" s="4"/>
-      <c r="C106" s="2" t="s">
-        <v>1241</v>
-      </c>
-      <c r="D106" s="4"/>
-      <c r="E106" s="4"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="4"/>
       <c r="B107" s="4"/>
       <c r="C107" s="2" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="D107" s="4"/>
       <c r="E107" s="4"/>
@@ -16236,7 +16242,7 @@
       <c r="A108" s="4"/>
       <c r="B108" s="4"/>
       <c r="C108" s="2" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="D108" s="4"/>
       <c r="E108" s="4"/>
@@ -16245,7 +16251,7 @@
       <c r="A109" s="4"/>
       <c r="B109" s="4"/>
       <c r="C109" s="2" t="s">
-        <v>786</v>
+        <v>1243</v>
       </c>
       <c r="D109" s="4"/>
       <c r="E109" s="4"/>
@@ -16254,7 +16260,7 @@
       <c r="A110" s="4"/>
       <c r="B110" s="4"/>
       <c r="C110" s="2" t="s">
-        <v>1244</v>
+        <v>786</v>
       </c>
       <c r="D110" s="4"/>
       <c r="E110" s="4"/>
@@ -16263,7 +16269,7 @@
       <c r="A111" s="4"/>
       <c r="B111" s="4"/>
       <c r="C111" s="2" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="D111" s="4"/>
       <c r="E111" s="4"/>
@@ -16272,7 +16278,7 @@
       <c r="A112" s="4"/>
       <c r="B112" s="4"/>
       <c r="C112" s="2" t="s">
-        <v>427</v>
+        <v>1245</v>
       </c>
       <c r="D112" s="4"/>
       <c r="E112" s="4"/>
@@ -16281,7 +16287,7 @@
       <c r="A113" s="4"/>
       <c r="B113" s="4"/>
       <c r="C113" s="2" t="s">
-        <v>781</v>
+        <v>427</v>
       </c>
       <c r="D113" s="4"/>
       <c r="E113" s="4"/>
@@ -16290,7 +16296,7 @@
       <c r="A114" s="4"/>
       <c r="B114" s="4"/>
       <c r="C114" s="2" t="s">
-        <v>1246</v>
+        <v>781</v>
       </c>
       <c r="D114" s="4"/>
       <c r="E114" s="4"/>
@@ -16299,7 +16305,7 @@
       <c r="A115" s="4"/>
       <c r="B115" s="4"/>
       <c r="C115" s="2" t="s">
-        <v>778</v>
+        <v>1246</v>
       </c>
       <c r="D115" s="4"/>
       <c r="E115" s="4"/>
@@ -16308,7 +16314,7 @@
       <c r="A116" s="4"/>
       <c r="B116" s="4"/>
       <c r="C116" s="2" t="s">
-        <v>1247</v>
+        <v>778</v>
       </c>
       <c r="D116" s="4"/>
       <c r="E116" s="4"/>
@@ -16317,7 +16323,7 @@
       <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="2" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="D117" s="4"/>
       <c r="E117" s="4"/>
@@ -16326,7 +16332,7 @@
       <c r="A118" s="4"/>
       <c r="B118" s="4"/>
       <c r="C118" s="2" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="D118" s="4"/>
       <c r="E118" s="4"/>
@@ -16335,85 +16341,85 @@
       <c r="A119" s="4"/>
       <c r="B119" s="4"/>
       <c r="C119" s="2" t="s">
-        <v>779</v>
+        <v>1249</v>
       </c>
       <c r="D119" s="4"/>
       <c r="E119" s="4"/>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A120" s="2">
+      <c r="A120" s="4"/>
+      <c r="B120" s="4"/>
+      <c r="C120" s="2" t="s">
+        <v>779</v>
+      </c>
+      <c r="D120" s="4"/>
+      <c r="E120" s="4"/>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A121" s="2">
         <v>51</v>
       </c>
-      <c r="B120" s="2" t="s">
+      <c r="B121" s="2" t="s">
         <v>1250</v>
       </c>
-      <c r="C120" s="2" t="s">
+      <c r="C121" s="2" t="s">
         <v>1005</v>
       </c>
-      <c r="D120" s="2" t="s">
+      <c r="D121" s="2" t="s">
         <v>1251</v>
       </c>
-      <c r="E120" s="2" t="s">
+      <c r="E121" s="2" t="s">
         <v>1010</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A121" s="4">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A122" s="4">
         <v>52</v>
       </c>
-      <c r="B121" s="4" t="s">
+      <c r="B122" s="4" t="s">
         <v>1102</v>
       </c>
-      <c r="C121" s="2" t="s">
+      <c r="C122" s="2" t="s">
         <v>1103</v>
       </c>
-      <c r="D121" s="4" t="s">
+      <c r="D122" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E121" s="4" t="s">
+      <c r="E122" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A122" s="4"/>
-      <c r="B122" s="4"/>
-      <c r="C122" s="2" t="s">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A123" s="4"/>
+      <c r="B123" s="4"/>
+      <c r="C123" s="2" t="s">
         <v>1252</v>
       </c>
-      <c r="D122" s="4"/>
-      <c r="E122" s="4"/>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A123" s="4">
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A124" s="4">
         <v>53</v>
       </c>
-      <c r="B123" s="4" t="s">
+      <c r="B124" s="4" t="s">
         <v>1167</v>
       </c>
-      <c r="C123" s="2" t="s">
+      <c r="C124" s="2" t="s">
         <v>1168</v>
       </c>
-      <c r="D123" s="4" t="s">
+      <c r="D124" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="E123" s="4" t="s">
+      <c r="E124" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="124" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A124" s="4"/>
-      <c r="B124" s="4"/>
-      <c r="C124" s="2" t="s">
-        <v>1169</v>
-      </c>
-      <c r="D124" s="4"/>
-      <c r="E124" s="4"/>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A125" s="4"/>
       <c r="B125" s="4"/>
       <c r="C125" s="2" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="D125" s="4"/>
       <c r="E125" s="4"/>
@@ -16422,7 +16428,7 @@
       <c r="A126" s="4"/>
       <c r="B126" s="4"/>
       <c r="C126" s="2" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="D126" s="4"/>
       <c r="E126" s="4"/>
@@ -16431,7 +16437,7 @@
       <c r="A127" s="4"/>
       <c r="B127" s="4"/>
       <c r="C127" s="2" t="s">
-        <v>1253</v>
+        <v>1171</v>
       </c>
       <c r="D127" s="4"/>
       <c r="E127" s="4"/>
@@ -16440,7 +16446,7 @@
       <c r="A128" s="4"/>
       <c r="B128" s="4"/>
       <c r="C128" s="2" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="D128" s="4"/>
       <c r="E128" s="4"/>
@@ -16449,7 +16455,7 @@
       <c r="A129" s="4"/>
       <c r="B129" s="4"/>
       <c r="C129" s="2" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="D129" s="4"/>
       <c r="E129" s="4"/>
@@ -16458,75 +16464,104 @@
       <c r="A130" s="4"/>
       <c r="B130" s="4"/>
       <c r="C130" s="2" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="D130" s="4"/>
       <c r="E130" s="4"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A131" s="2">
-        <v>54</v>
-      </c>
-      <c r="B131" s="2" t="s">
-        <v>1257</v>
-      </c>
+      <c r="A131" s="4"/>
+      <c r="B131" s="4"/>
       <c r="C131" s="2" t="s">
-        <v>1258</v>
-      </c>
-      <c r="D131" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E131" s="2" t="s">
-        <v>468</v>
-      </c>
+        <v>1256</v>
+      </c>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
+        <v>54</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>1257</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>1258</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A133" s="2">
         <v>55</v>
       </c>
-      <c r="B132" s="2" t="s">
+      <c r="B133" s="2" t="s">
         <v>1259</v>
       </c>
-      <c r="C132" s="2" t="s">
+      <c r="C133" s="2" t="s">
         <v>839</v>
       </c>
-      <c r="D132" s="2" t="s">
+      <c r="D133" s="2" t="s">
         <v>840</v>
       </c>
-      <c r="E132" s="2" t="s">
+      <c r="E133" s="2" t="s">
         <v>486</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="A123:A130"/>
-    <mergeCell ref="B123:B130"/>
-    <mergeCell ref="D123:D130"/>
-    <mergeCell ref="E123:E130"/>
-    <mergeCell ref="A105:A119"/>
-    <mergeCell ref="B105:B119"/>
-    <mergeCell ref="D105:D119"/>
-    <mergeCell ref="E105:E119"/>
-    <mergeCell ref="A121:A122"/>
-    <mergeCell ref="B121:B122"/>
-    <mergeCell ref="D121:D122"/>
-    <mergeCell ref="E121:E122"/>
-    <mergeCell ref="A100:A101"/>
-    <mergeCell ref="B100:B101"/>
-    <mergeCell ref="D100:D101"/>
-    <mergeCell ref="E100:E101"/>
-    <mergeCell ref="A102:A103"/>
-    <mergeCell ref="B102:B103"/>
-    <mergeCell ref="D102:D103"/>
-    <mergeCell ref="E102:E103"/>
-    <mergeCell ref="A84:A94"/>
-    <mergeCell ref="B84:B94"/>
-    <mergeCell ref="D84:D94"/>
-    <mergeCell ref="E84:E94"/>
-    <mergeCell ref="A95:A98"/>
-    <mergeCell ref="B95:B98"/>
-    <mergeCell ref="D95:D98"/>
-    <mergeCell ref="E95:E98"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="A11:A19"/>
+    <mergeCell ref="B11:B19"/>
+    <mergeCell ref="D11:D19"/>
+    <mergeCell ref="E11:E19"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="A25:A28"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="D25:D28"/>
+    <mergeCell ref="E25:E28"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="D30:D32"/>
+    <mergeCell ref="E30:E32"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="D33:D36"/>
+    <mergeCell ref="E33:E36"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="A46:A48"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="A51:A55"/>
+    <mergeCell ref="B51:B55"/>
+    <mergeCell ref="D51:D55"/>
+    <mergeCell ref="E51:E55"/>
+    <mergeCell ref="A57:A61"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="D57:D61"/>
+    <mergeCell ref="E57:E61"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="E68:E69"/>
+    <mergeCell ref="A64:A65"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="E64:E65"/>
     <mergeCell ref="A70:A72"/>
     <mergeCell ref="B70:B72"/>
     <mergeCell ref="D70:D72"/>
@@ -16535,54 +16570,34 @@
     <mergeCell ref="B74:B79"/>
     <mergeCell ref="D74:D79"/>
     <mergeCell ref="E74:E79"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="E68:E69"/>
-    <mergeCell ref="A64:A65"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="E64:E65"/>
-    <mergeCell ref="A51:A55"/>
-    <mergeCell ref="B51:B55"/>
-    <mergeCell ref="D51:D55"/>
-    <mergeCell ref="E51:E55"/>
-    <mergeCell ref="A57:A61"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="D57:D61"/>
-    <mergeCell ref="E57:E61"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="D39:D41"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="A46:A48"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="D30:D32"/>
-    <mergeCell ref="E30:E32"/>
-    <mergeCell ref="A33:A36"/>
-    <mergeCell ref="B33:B36"/>
-    <mergeCell ref="D33:D36"/>
-    <mergeCell ref="E33:E36"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="A25:A28"/>
-    <mergeCell ref="B25:B28"/>
-    <mergeCell ref="D25:D28"/>
-    <mergeCell ref="E25:E28"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="A11:A19"/>
-    <mergeCell ref="B11:B19"/>
-    <mergeCell ref="D11:D19"/>
-    <mergeCell ref="E11:E19"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="A84:A95"/>
+    <mergeCell ref="B84:B95"/>
+    <mergeCell ref="D84:D95"/>
+    <mergeCell ref="E84:E95"/>
+    <mergeCell ref="A96:A99"/>
+    <mergeCell ref="B96:B99"/>
+    <mergeCell ref="D96:D99"/>
+    <mergeCell ref="E96:E99"/>
+    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="B101:B102"/>
+    <mergeCell ref="D101:D102"/>
+    <mergeCell ref="E101:E102"/>
+    <mergeCell ref="A103:A104"/>
+    <mergeCell ref="B103:B104"/>
+    <mergeCell ref="D103:D104"/>
+    <mergeCell ref="E103:E104"/>
+    <mergeCell ref="A124:A131"/>
+    <mergeCell ref="B124:B131"/>
+    <mergeCell ref="D124:D131"/>
+    <mergeCell ref="E124:E131"/>
+    <mergeCell ref="A106:A120"/>
+    <mergeCell ref="B106:B120"/>
+    <mergeCell ref="D106:D120"/>
+    <mergeCell ref="E106:E120"/>
+    <mergeCell ref="A122:A123"/>
+    <mergeCell ref="B122:B123"/>
+    <mergeCell ref="D122:D123"/>
+    <mergeCell ref="E122:E123"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>